<commit_message>
Update soccer trades 2026-07-26 11:20:50 UTC
</commit_message>
<xml_diff>
--- a/data/sxbet/ligas/Besta Deild Karla/trades.xlsx
+++ b/data/sxbet/ligas/Besta Deild Karla/trades.xlsx
@@ -544,11 +544,15 @@
           <t>1</t>
         </is>
       </c>
-      <c r="D2" t="n">
-        <v>35</v>
-      </c>
-      <c r="E2" t="n">
-        <v>1.5987</v>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>35.0</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>1.5987</t>
+        </is>
       </c>
       <c r="F2" t="inlineStr"/>
       <c r="G2" t="inlineStr"/>
@@ -582,25 +586,35 @@
           <t>L19520873</t>
         </is>
       </c>
-      <c r="N2" t="n">
-        <v>1</v>
-      </c>
-      <c r="O2" t="n">
-        <v>0</v>
+      <c r="N2" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="O2" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
       </c>
       <c r="P2" t="inlineStr">
         <is>
           <t>SUCCESS</t>
         </is>
       </c>
-      <c r="Q2" t="n">
-        <v>1</v>
-      </c>
-      <c r="R2" t="n">
-        <v>1784987195</v>
-      </c>
-      <c r="S2" t="n">
-        <v>1784988000</v>
+      <c r="Q2" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="R2" t="inlineStr">
+        <is>
+          <t>1784987195</t>
+        </is>
+      </c>
+      <c r="S2" t="inlineStr">
+        <is>
+          <t>1784988000</t>
+        </is>
       </c>
       <c r="T2" t="inlineStr">
         <is>
@@ -630,11 +644,15 @@
           <t>2</t>
         </is>
       </c>
-      <c r="D3" t="n">
-        <v>12</v>
-      </c>
-      <c r="E3" t="n">
-        <v>1.7862</v>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>12.0</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>1.7862</t>
+        </is>
       </c>
       <c r="F3" t="inlineStr"/>
       <c r="G3" t="inlineStr"/>
@@ -668,25 +686,35 @@
           <t>L19520873</t>
         </is>
       </c>
-      <c r="N3" t="n">
-        <v>1</v>
-      </c>
-      <c r="O3" t="n">
-        <v>0</v>
+      <c r="N3" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="O3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
       </c>
       <c r="P3" t="inlineStr">
         <is>
           <t>SUCCESS</t>
         </is>
       </c>
-      <c r="Q3" t="n">
-        <v>1</v>
-      </c>
-      <c r="R3" t="n">
-        <v>1784986980</v>
-      </c>
-      <c r="S3" t="n">
-        <v>1784988000</v>
+      <c r="Q3" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="R3" t="inlineStr">
+        <is>
+          <t>1784986980</t>
+        </is>
+      </c>
+      <c r="S3" t="inlineStr">
+        <is>
+          <t>1784988000</t>
+        </is>
       </c>
       <c r="T3" t="inlineStr">
         <is>
@@ -716,11 +744,15 @@
           <t>2</t>
         </is>
       </c>
-      <c r="D4" t="n">
-        <v>37</v>
-      </c>
-      <c r="E4" t="n">
-        <v>1.7875</v>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>37.0</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>1.7875</t>
+        </is>
       </c>
       <c r="F4" t="inlineStr"/>
       <c r="G4" t="inlineStr"/>
@@ -754,25 +786,35 @@
           <t>L19520873</t>
         </is>
       </c>
-      <c r="N4" t="n">
-        <v>1</v>
-      </c>
-      <c r="O4" t="n">
-        <v>0</v>
+      <c r="N4" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="O4" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
       </c>
       <c r="P4" t="inlineStr">
         <is>
           <t>SUCCESS</t>
         </is>
       </c>
-      <c r="Q4" t="n">
-        <v>1</v>
-      </c>
-      <c r="R4" t="n">
-        <v>1784986980</v>
-      </c>
-      <c r="S4" t="n">
-        <v>1784988000</v>
+      <c r="Q4" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="R4" t="inlineStr">
+        <is>
+          <t>1784986980</t>
+        </is>
+      </c>
+      <c r="S4" t="inlineStr">
+        <is>
+          <t>1784988000</t>
+        </is>
       </c>
       <c r="T4" t="inlineStr">
         <is>
@@ -802,11 +844,15 @@
           <t>1</t>
         </is>
       </c>
-      <c r="D5" t="n">
-        <v>69</v>
-      </c>
-      <c r="E5" t="n">
-        <v>1.6012</v>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>69.0</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>1.6012</t>
+        </is>
       </c>
       <c r="F5" t="inlineStr"/>
       <c r="G5" t="inlineStr"/>
@@ -840,25 +886,35 @@
           <t>L19520873</t>
         </is>
       </c>
-      <c r="N5" t="n">
-        <v>1</v>
-      </c>
-      <c r="O5" t="n">
-        <v>0</v>
+      <c r="N5" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="O5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
       </c>
       <c r="P5" t="inlineStr">
         <is>
           <t>SUCCESS</t>
         </is>
       </c>
-      <c r="Q5" t="n">
-        <v>1</v>
-      </c>
-      <c r="R5" t="n">
-        <v>1784986978</v>
-      </c>
-      <c r="S5" t="n">
-        <v>1784988000</v>
+      <c r="Q5" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="R5" t="inlineStr">
+        <is>
+          <t>1784986978</t>
+        </is>
+      </c>
+      <c r="S5" t="inlineStr">
+        <is>
+          <t>1784988000</t>
+        </is>
       </c>
       <c r="T5" t="inlineStr">
         <is>
@@ -888,11 +944,15 @@
           <t>1</t>
         </is>
       </c>
-      <c r="D6" t="n">
-        <v>15</v>
-      </c>
-      <c r="E6" t="n">
-        <v>1.2712</v>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>15.0</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>1.2712</t>
+        </is>
       </c>
       <c r="F6" t="inlineStr"/>
       <c r="G6" t="inlineStr"/>
@@ -926,25 +986,35 @@
           <t>L19520873</t>
         </is>
       </c>
-      <c r="N6" t="n">
-        <v>1</v>
-      </c>
-      <c r="O6" t="n">
-        <v>0</v>
+      <c r="N6" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="O6" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
       </c>
       <c r="P6" t="inlineStr">
         <is>
           <t>SUCCESS</t>
         </is>
       </c>
-      <c r="Q6" t="n">
-        <v>1</v>
-      </c>
-      <c r="R6" t="n">
-        <v>1784984833</v>
-      </c>
-      <c r="S6" t="n">
-        <v>1784988000</v>
+      <c r="Q6" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="R6" t="inlineStr">
+        <is>
+          <t>1784984833</t>
+        </is>
+      </c>
+      <c r="S6" t="inlineStr">
+        <is>
+          <t>1784988000</t>
+        </is>
       </c>
       <c r="T6" t="inlineStr">
         <is>
@@ -961,7 +1031,7 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>0x78e73a1fbc4bce58e1469ba84a7a75afedee1c817a9927ff72cae6f55f5b4a58</t>
+          <t>0x832d570bfcb61240d74893710e1758118ea62888a2bf55921f3190b9a71f4561</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
@@ -974,11 +1044,15 @@
           <t>2</t>
         </is>
       </c>
-      <c r="D7" t="n">
-        <v>8</v>
-      </c>
-      <c r="E7" t="n">
-        <v>1.7887</v>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>3.0</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>1.7887</t>
+        </is>
       </c>
       <c r="F7" t="inlineStr"/>
       <c r="G7" t="inlineStr"/>
@@ -1012,29 +1086,39 @@
           <t>L19520873</t>
         </is>
       </c>
-      <c r="N7" t="n">
-        <v>1</v>
-      </c>
-      <c r="O7" t="n">
-        <v>0</v>
+      <c r="N7" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="O7" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
       </c>
       <c r="P7" t="inlineStr">
         <is>
           <t>SUCCESS</t>
         </is>
       </c>
-      <c r="Q7" t="n">
-        <v>1</v>
-      </c>
-      <c r="R7" t="n">
-        <v>1784984812</v>
-      </c>
-      <c r="S7" t="n">
-        <v>1784988000</v>
+      <c r="Q7" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="R7" t="inlineStr">
+        <is>
+          <t>1784984812</t>
+        </is>
+      </c>
+      <c r="S7" t="inlineStr">
+        <is>
+          <t>1784988000</t>
+        </is>
       </c>
       <c r="T7" t="inlineStr">
         <is>
-          <t>10.745559</t>
+          <t>4.733718</t>
         </is>
       </c>
       <c r="U7" t="inlineStr">
@@ -1047,7 +1131,7 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>0x02053d570c2ec6485bf734b3e9d25cb6962b678b5212cc142c9b62d371752a01</t>
+          <t>0x78e73a1fbc4bce58e1469ba84a7a75afedee1c817a9927ff72cae6f55f5b4a58</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
@@ -1057,14 +1141,18 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="D8" t="n">
-        <v>13</v>
-      </c>
-      <c r="E8" t="n">
-        <v>1.5737</v>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>8.0</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>1.7887</t>
+        </is>
       </c>
       <c r="F8" t="inlineStr"/>
       <c r="G8" t="inlineStr"/>
@@ -1090,7 +1178,7 @@
       </c>
       <c r="L8" t="inlineStr">
         <is>
-          <t>0x04fd78e33c10fb928e409323c26948f49fe4c81fcd47748d9153c9c611b38d0b</t>
+          <t>0x91a9ea8ebfd8b049218a8e072590d2f657e26fdb1f2a49b1016ae42171c68ef2</t>
         </is>
       </c>
       <c r="M8" t="inlineStr">
@@ -1098,29 +1186,39 @@
           <t>L19520873</t>
         </is>
       </c>
-      <c r="N8" t="n">
-        <v>1</v>
-      </c>
-      <c r="O8" t="n">
-        <v>0</v>
+      <c r="N8" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="O8" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
       </c>
       <c r="P8" t="inlineStr">
         <is>
           <t>SUCCESS</t>
         </is>
       </c>
-      <c r="Q8" t="n">
-        <v>1</v>
-      </c>
-      <c r="R8" t="n">
-        <v>1784984812</v>
-      </c>
-      <c r="S8" t="n">
-        <v>1784988000</v>
+      <c r="Q8" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="R8" t="inlineStr">
+        <is>
+          <t>1784984812</t>
+        </is>
+      </c>
+      <c r="S8" t="inlineStr">
+        <is>
+          <t>1784988000</t>
+        </is>
       </c>
       <c r="T8" t="inlineStr">
         <is>
-          <t>23.46041</t>
+          <t>10.745559</t>
         </is>
       </c>
       <c r="U8" t="inlineStr">
@@ -1133,7 +1231,7 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>0x832d570bfcb61240d74893710e1758118ea62888a2bf55921f3190b9a71f4561</t>
+          <t>0x02053d570c2ec6485bf734b3e9d25cb6962b678b5212cc142c9b62d371752a01</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
@@ -1143,14 +1241,18 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>2</t>
-        </is>
-      </c>
-      <c r="D9" t="n">
-        <v>3</v>
-      </c>
-      <c r="E9" t="n">
-        <v>1.7887</v>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>13.0</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>1.5737</t>
+        </is>
       </c>
       <c r="F9" t="inlineStr"/>
       <c r="G9" t="inlineStr"/>
@@ -1176,7 +1278,7 @@
       </c>
       <c r="L9" t="inlineStr">
         <is>
-          <t>0x91a9ea8ebfd8b049218a8e072590d2f657e26fdb1f2a49b1016ae42171c68ef2</t>
+          <t>0x04fd78e33c10fb928e409323c26948f49fe4c81fcd47748d9153c9c611b38d0b</t>
         </is>
       </c>
       <c r="M9" t="inlineStr">
@@ -1184,29 +1286,39 @@
           <t>L19520873</t>
         </is>
       </c>
-      <c r="N9" t="n">
-        <v>1</v>
-      </c>
-      <c r="O9" t="n">
-        <v>0</v>
+      <c r="N9" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="O9" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
       </c>
       <c r="P9" t="inlineStr">
         <is>
           <t>SUCCESS</t>
         </is>
       </c>
-      <c r="Q9" t="n">
-        <v>1</v>
-      </c>
-      <c r="R9" t="n">
-        <v>1784984812</v>
-      </c>
-      <c r="S9" t="n">
-        <v>1784988000</v>
+      <c r="Q9" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="R9" t="inlineStr">
+        <is>
+          <t>1784984812</t>
+        </is>
+      </c>
+      <c r="S9" t="inlineStr">
+        <is>
+          <t>1784988000</t>
+        </is>
       </c>
       <c r="T9" t="inlineStr">
         <is>
-          <t>4.733718</t>
+          <t>23.46041</t>
         </is>
       </c>
       <c r="U9" t="inlineStr">
@@ -1232,11 +1344,15 @@
           <t>1</t>
         </is>
       </c>
-      <c r="D10" t="n">
-        <v>15</v>
-      </c>
-      <c r="E10" t="n">
-        <v>1.2712</v>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>15.0</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>1.2712</t>
+        </is>
       </c>
       <c r="F10" t="inlineStr"/>
       <c r="G10" t="inlineStr"/>
@@ -1270,25 +1386,35 @@
           <t>L19520873</t>
         </is>
       </c>
-      <c r="N10" t="n">
-        <v>1</v>
-      </c>
-      <c r="O10" t="n">
-        <v>0</v>
+      <c r="N10" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="O10" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
       </c>
       <c r="P10" t="inlineStr">
         <is>
           <t>SUCCESS</t>
         </is>
       </c>
-      <c r="Q10" t="n">
-        <v>1</v>
-      </c>
-      <c r="R10" t="n">
-        <v>1784984810</v>
-      </c>
-      <c r="S10" t="n">
-        <v>1784988000</v>
+      <c r="Q10" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="R10" t="inlineStr">
+        <is>
+          <t>1784984810</t>
+        </is>
+      </c>
+      <c r="S10" t="inlineStr">
+        <is>
+          <t>1784988000</t>
+        </is>
       </c>
       <c r="T10" t="inlineStr">
         <is>
@@ -1318,11 +1444,15 @@
           <t>1</t>
         </is>
       </c>
-      <c r="D11" t="n">
-        <v>16</v>
-      </c>
-      <c r="E11" t="n">
-        <v>1.2712</v>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>16.0</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>1.2712</t>
+        </is>
       </c>
       <c r="F11" t="inlineStr"/>
       <c r="G11" t="inlineStr"/>
@@ -1356,25 +1486,35 @@
           <t>L19520873</t>
         </is>
       </c>
-      <c r="N11" t="n">
-        <v>1</v>
-      </c>
-      <c r="O11" t="n">
-        <v>0</v>
+      <c r="N11" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="O11" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
       </c>
       <c r="P11" t="inlineStr">
         <is>
           <t>SUCCESS</t>
         </is>
       </c>
-      <c r="Q11" t="n">
-        <v>1</v>
-      </c>
-      <c r="R11" t="n">
-        <v>1784984670</v>
-      </c>
-      <c r="S11" t="n">
-        <v>1784988000</v>
+      <c r="Q11" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="R11" t="inlineStr">
+        <is>
+          <t>1784984670</t>
+        </is>
+      </c>
+      <c r="S11" t="inlineStr">
+        <is>
+          <t>1784988000</t>
+        </is>
       </c>
       <c r="T11" t="inlineStr">
         <is>
@@ -1404,11 +1544,15 @@
           <t>1</t>
         </is>
       </c>
-      <c r="D12" t="n">
-        <v>16</v>
-      </c>
-      <c r="E12" t="n">
-        <v>1.2712</v>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>16.0</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>1.2712</t>
+        </is>
       </c>
       <c r="F12" t="inlineStr"/>
       <c r="G12" t="inlineStr"/>
@@ -1442,25 +1586,35 @@
           <t>L19520873</t>
         </is>
       </c>
-      <c r="N12" t="n">
-        <v>1</v>
-      </c>
-      <c r="O12" t="n">
-        <v>0</v>
+      <c r="N12" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="O12" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
       </c>
       <c r="P12" t="inlineStr">
         <is>
           <t>SUCCESS</t>
         </is>
       </c>
-      <c r="Q12" t="n">
-        <v>1</v>
-      </c>
-      <c r="R12" t="n">
-        <v>1784984617</v>
-      </c>
-      <c r="S12" t="n">
-        <v>1784988000</v>
+      <c r="Q12" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="R12" t="inlineStr">
+        <is>
+          <t>1784984617</t>
+        </is>
+      </c>
+      <c r="S12" t="inlineStr">
+        <is>
+          <t>1784988000</t>
+        </is>
       </c>
       <c r="T12" t="inlineStr">
         <is>
@@ -1490,11 +1644,15 @@
           <t>1</t>
         </is>
       </c>
-      <c r="D13" t="n">
-        <v>16</v>
-      </c>
-      <c r="E13" t="n">
-        <v>1.2712</v>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>16.0</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>1.2712</t>
+        </is>
       </c>
       <c r="F13" t="inlineStr"/>
       <c r="G13" t="inlineStr"/>
@@ -1528,25 +1686,35 @@
           <t>L19520873</t>
         </is>
       </c>
-      <c r="N13" t="n">
-        <v>1</v>
-      </c>
-      <c r="O13" t="n">
-        <v>0</v>
+      <c r="N13" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="O13" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
       </c>
       <c r="P13" t="inlineStr">
         <is>
           <t>SUCCESS</t>
         </is>
       </c>
-      <c r="Q13" t="n">
-        <v>1</v>
-      </c>
-      <c r="R13" t="n">
-        <v>1784984581</v>
-      </c>
-      <c r="S13" t="n">
-        <v>1784988000</v>
+      <c r="Q13" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="R13" t="inlineStr">
+        <is>
+          <t>1784984581</t>
+        </is>
+      </c>
+      <c r="S13" t="inlineStr">
+        <is>
+          <t>1784988000</t>
+        </is>
       </c>
       <c r="T13" t="inlineStr">
         <is>
@@ -1576,11 +1744,15 @@
           <t>1</t>
         </is>
       </c>
-      <c r="D14" t="n">
-        <v>16</v>
-      </c>
-      <c r="E14" t="n">
-        <v>1.2712</v>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>16.0</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>1.2712</t>
+        </is>
       </c>
       <c r="F14" t="inlineStr"/>
       <c r="G14" t="inlineStr"/>
@@ -1614,25 +1786,35 @@
           <t>L19520873</t>
         </is>
       </c>
-      <c r="N14" t="n">
-        <v>1</v>
-      </c>
-      <c r="O14" t="n">
-        <v>0</v>
+      <c r="N14" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="O14" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
       </c>
       <c r="P14" t="inlineStr">
         <is>
           <t>SUCCESS</t>
         </is>
       </c>
-      <c r="Q14" t="n">
-        <v>1</v>
-      </c>
-      <c r="R14" t="n">
-        <v>1784984563</v>
-      </c>
-      <c r="S14" t="n">
-        <v>1784988000</v>
+      <c r="Q14" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="R14" t="inlineStr">
+        <is>
+          <t>1784984563</t>
+        </is>
+      </c>
+      <c r="S14" t="inlineStr">
+        <is>
+          <t>1784988000</t>
+        </is>
       </c>
       <c r="T14" t="inlineStr">
         <is>
@@ -1662,11 +1844,15 @@
           <t>1</t>
         </is>
       </c>
-      <c r="D15" t="n">
-        <v>9</v>
-      </c>
-      <c r="E15" t="n">
-        <v>1.3013</v>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>9.0</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>1.3013</t>
+        </is>
       </c>
       <c r="F15" t="inlineStr"/>
       <c r="G15" t="inlineStr"/>
@@ -1700,25 +1886,35 @@
           <t>L19520873</t>
         </is>
       </c>
-      <c r="N15" t="n">
-        <v>1</v>
-      </c>
-      <c r="O15" t="n">
-        <v>0</v>
+      <c r="N15" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="O15" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
       </c>
       <c r="P15" t="inlineStr">
         <is>
           <t>SUCCESS</t>
         </is>
       </c>
-      <c r="Q15" t="n">
-        <v>1</v>
-      </c>
-      <c r="R15" t="n">
-        <v>1784984538</v>
-      </c>
-      <c r="S15" t="n">
-        <v>1784988000</v>
+      <c r="Q15" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="R15" t="inlineStr">
+        <is>
+          <t>1784984538</t>
+        </is>
+      </c>
+      <c r="S15" t="inlineStr">
+        <is>
+          <t>1784988000</t>
+        </is>
       </c>
       <c r="T15" t="inlineStr">
         <is>
@@ -1748,11 +1944,15 @@
           <t>1</t>
         </is>
       </c>
-      <c r="D16" t="n">
-        <v>21</v>
-      </c>
-      <c r="E16" t="n">
-        <v>1.4363</v>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>21.0</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>1.4363</t>
+        </is>
       </c>
       <c r="F16" t="inlineStr"/>
       <c r="G16" t="inlineStr"/>
@@ -1786,25 +1986,35 @@
           <t>L19520873</t>
         </is>
       </c>
-      <c r="N16" t="n">
-        <v>1</v>
-      </c>
-      <c r="O16" t="n">
-        <v>0</v>
+      <c r="N16" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="O16" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
       </c>
       <c r="P16" t="inlineStr">
         <is>
           <t>SUCCESS</t>
         </is>
       </c>
-      <c r="Q16" t="n">
-        <v>1</v>
-      </c>
-      <c r="R16" t="n">
-        <v>1784984537</v>
-      </c>
-      <c r="S16" t="n">
-        <v>1784988000</v>
+      <c r="Q16" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="R16" t="inlineStr">
+        <is>
+          <t>1784984537</t>
+        </is>
+      </c>
+      <c r="S16" t="inlineStr">
+        <is>
+          <t>1784988000</t>
+        </is>
       </c>
       <c r="T16" t="inlineStr">
         <is>
@@ -1834,11 +2044,15 @@
           <t>1</t>
         </is>
       </c>
-      <c r="D17" t="n">
-        <v>38</v>
-      </c>
-      <c r="E17" t="n">
-        <v>1.5537</v>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>38.0</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>1.5537</t>
+        </is>
       </c>
       <c r="F17" t="inlineStr"/>
       <c r="G17" t="inlineStr"/>
@@ -1872,25 +2086,35 @@
           <t>L19520873</t>
         </is>
       </c>
-      <c r="N17" t="n">
-        <v>1</v>
-      </c>
-      <c r="O17" t="n">
-        <v>0</v>
+      <c r="N17" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="O17" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
       </c>
       <c r="P17" t="inlineStr">
         <is>
           <t>SUCCESS</t>
         </is>
       </c>
-      <c r="Q17" t="n">
-        <v>1</v>
-      </c>
-      <c r="R17" t="n">
-        <v>1784984536</v>
-      </c>
-      <c r="S17" t="n">
-        <v>1784988000</v>
+      <c r="Q17" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="R17" t="inlineStr">
+        <is>
+          <t>1784984536</t>
+        </is>
+      </c>
+      <c r="S17" t="inlineStr">
+        <is>
+          <t>1784988000</t>
+        </is>
       </c>
       <c r="T17" t="inlineStr">
         <is>
@@ -1920,11 +2144,15 @@
           <t>1</t>
         </is>
       </c>
-      <c r="D18" t="n">
-        <v>29</v>
-      </c>
-      <c r="E18" t="n">
-        <v>1.5537</v>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>29.0</t>
+        </is>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>1.5537</t>
+        </is>
       </c>
       <c r="F18" t="inlineStr"/>
       <c r="G18" t="inlineStr"/>
@@ -1958,25 +2186,35 @@
           <t>L19520873</t>
         </is>
       </c>
-      <c r="N18" t="n">
-        <v>1</v>
-      </c>
-      <c r="O18" t="n">
-        <v>0</v>
+      <c r="N18" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="O18" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
       </c>
       <c r="P18" t="inlineStr">
         <is>
           <t>SUCCESS</t>
         </is>
       </c>
-      <c r="Q18" t="n">
-        <v>1</v>
-      </c>
-      <c r="R18" t="n">
-        <v>1784984502</v>
-      </c>
-      <c r="S18" t="n">
-        <v>1784988000</v>
+      <c r="Q18" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="R18" t="inlineStr">
+        <is>
+          <t>1784984502</t>
+        </is>
+      </c>
+      <c r="S18" t="inlineStr">
+        <is>
+          <t>1784988000</t>
+        </is>
       </c>
       <c r="T18" t="inlineStr">
         <is>
@@ -2006,11 +2244,15 @@
           <t>1</t>
         </is>
       </c>
-      <c r="D19" t="n">
-        <v>25</v>
-      </c>
-      <c r="E19" t="n">
-        <v>1.5537</v>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>25.0</t>
+        </is>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>1.5537</t>
+        </is>
       </c>
       <c r="F19" t="inlineStr"/>
       <c r="G19" t="inlineStr"/>
@@ -2044,25 +2286,35 @@
           <t>L19520873</t>
         </is>
       </c>
-      <c r="N19" t="n">
-        <v>1</v>
-      </c>
-      <c r="O19" t="n">
-        <v>0</v>
+      <c r="N19" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="O19" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
       </c>
       <c r="P19" t="inlineStr">
         <is>
           <t>SUCCESS</t>
         </is>
       </c>
-      <c r="Q19" t="n">
-        <v>1</v>
-      </c>
-      <c r="R19" t="n">
-        <v>1784984501</v>
-      </c>
-      <c r="S19" t="n">
-        <v>1784988000</v>
+      <c r="Q19" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="R19" t="inlineStr">
+        <is>
+          <t>1784984501</t>
+        </is>
+      </c>
+      <c r="S19" t="inlineStr">
+        <is>
+          <t>1784988000</t>
+        </is>
       </c>
       <c r="T19" t="inlineStr">
         <is>
@@ -2092,11 +2344,15 @@
           <t>1</t>
         </is>
       </c>
-      <c r="D20" t="n">
-        <v>6</v>
-      </c>
-      <c r="E20" t="n">
-        <v>1.3013</v>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>6.0</t>
+        </is>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>1.3013</t>
+        </is>
       </c>
       <c r="F20" t="inlineStr"/>
       <c r="G20" t="inlineStr"/>
@@ -2130,25 +2386,35 @@
           <t>L19520873</t>
         </is>
       </c>
-      <c r="N20" t="n">
-        <v>1</v>
-      </c>
-      <c r="O20" t="n">
-        <v>0</v>
+      <c r="N20" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="O20" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
       </c>
       <c r="P20" t="inlineStr">
         <is>
           <t>SUCCESS</t>
         </is>
       </c>
-      <c r="Q20" t="n">
-        <v>1</v>
-      </c>
-      <c r="R20" t="n">
-        <v>1784984431</v>
-      </c>
-      <c r="S20" t="n">
-        <v>1784988000</v>
+      <c r="Q20" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="R20" t="inlineStr">
+        <is>
+          <t>1784984431</t>
+        </is>
+      </c>
+      <c r="S20" t="inlineStr">
+        <is>
+          <t>1784988000</t>
+        </is>
       </c>
       <c r="T20" t="inlineStr">
         <is>
@@ -2178,11 +2444,15 @@
           <t>1</t>
         </is>
       </c>
-      <c r="D21" t="n">
-        <v>27</v>
-      </c>
-      <c r="E21" t="n">
-        <v>1.4537</v>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>27.0</t>
+        </is>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>1.4537</t>
+        </is>
       </c>
       <c r="F21" t="inlineStr"/>
       <c r="G21" t="inlineStr"/>
@@ -2216,25 +2486,35 @@
           <t>L19520873</t>
         </is>
       </c>
-      <c r="N21" t="n">
-        <v>1</v>
-      </c>
-      <c r="O21" t="n">
-        <v>0</v>
+      <c r="N21" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="O21" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
       </c>
       <c r="P21" t="inlineStr">
         <is>
           <t>SUCCESS</t>
         </is>
       </c>
-      <c r="Q21" t="n">
-        <v>1</v>
-      </c>
-      <c r="R21" t="n">
-        <v>1784984405</v>
-      </c>
-      <c r="S21" t="n">
-        <v>1784988000</v>
+      <c r="Q21" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="R21" t="inlineStr">
+        <is>
+          <t>1784984405</t>
+        </is>
+      </c>
+      <c r="S21" t="inlineStr">
+        <is>
+          <t>1784988000</t>
+        </is>
       </c>
       <c r="T21" t="inlineStr">
         <is>
@@ -2264,11 +2544,15 @@
           <t>1</t>
         </is>
       </c>
-      <c r="D22" t="n">
-        <v>35</v>
-      </c>
-      <c r="E22" t="n">
-        <v>1.595</v>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>35.0</t>
+        </is>
+      </c>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>1.595</t>
+        </is>
       </c>
       <c r="F22" t="inlineStr"/>
       <c r="G22" t="inlineStr"/>
@@ -2302,25 +2586,35 @@
           <t>L19520873</t>
         </is>
       </c>
-      <c r="N22" t="n">
-        <v>1</v>
-      </c>
-      <c r="O22" t="n">
-        <v>0</v>
+      <c r="N22" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="O22" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
       </c>
       <c r="P22" t="inlineStr">
         <is>
           <t>SUCCESS</t>
         </is>
       </c>
-      <c r="Q22" t="n">
-        <v>1</v>
-      </c>
-      <c r="R22" t="n">
-        <v>1784984404</v>
-      </c>
-      <c r="S22" t="n">
-        <v>1784988000</v>
+      <c r="Q22" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="R22" t="inlineStr">
+        <is>
+          <t>1784984404</t>
+        </is>
+      </c>
+      <c r="S22" t="inlineStr">
+        <is>
+          <t>1784988000</t>
+        </is>
       </c>
       <c r="T22" t="inlineStr">
         <is>
@@ -2350,11 +2644,15 @@
           <t>2</t>
         </is>
       </c>
-      <c r="D23" t="n">
-        <v>22</v>
-      </c>
-      <c r="E23" t="n">
-        <v>1.7712</v>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>22.0</t>
+        </is>
+      </c>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>1.7712</t>
+        </is>
       </c>
       <c r="F23" t="inlineStr"/>
       <c r="G23" t="inlineStr"/>
@@ -2388,25 +2686,35 @@
           <t>L19520873</t>
         </is>
       </c>
-      <c r="N23" t="n">
-        <v>1</v>
-      </c>
-      <c r="O23" t="n">
-        <v>0</v>
+      <c r="N23" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="O23" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
       </c>
       <c r="P23" t="inlineStr">
         <is>
           <t>SUCCESS</t>
         </is>
       </c>
-      <c r="Q23" t="n">
-        <v>1</v>
-      </c>
-      <c r="R23" t="n">
-        <v>1784984403</v>
-      </c>
-      <c r="S23" t="n">
-        <v>1784988000</v>
+      <c r="Q23" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="R23" t="inlineStr">
+        <is>
+          <t>1784984403</t>
+        </is>
+      </c>
+      <c r="S23" t="inlineStr">
+        <is>
+          <t>1784988000</t>
+        </is>
       </c>
       <c r="T23" t="inlineStr">
         <is>
@@ -2436,11 +2744,15 @@
           <t>2</t>
         </is>
       </c>
-      <c r="D24" t="n">
-        <v>3</v>
-      </c>
-      <c r="E24" t="n">
-        <v>1.775</v>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>3.0</t>
+        </is>
+      </c>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>1.775</t>
+        </is>
       </c>
       <c r="F24" t="inlineStr"/>
       <c r="G24" t="inlineStr"/>
@@ -2474,25 +2786,35 @@
           <t>L19520873</t>
         </is>
       </c>
-      <c r="N24" t="n">
-        <v>1</v>
-      </c>
-      <c r="O24" t="n">
-        <v>0</v>
+      <c r="N24" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="O24" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
       </c>
       <c r="P24" t="inlineStr">
         <is>
           <t>SUCCESS</t>
         </is>
       </c>
-      <c r="Q24" t="n">
-        <v>1</v>
-      </c>
-      <c r="R24" t="n">
-        <v>1784984403</v>
-      </c>
-      <c r="S24" t="n">
-        <v>1784988000</v>
+      <c r="Q24" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="R24" t="inlineStr">
+        <is>
+          <t>1784984403</t>
+        </is>
+      </c>
+      <c r="S24" t="inlineStr">
+        <is>
+          <t>1784988000</t>
+        </is>
       </c>
       <c r="T24" t="inlineStr">
         <is>
@@ -2522,11 +2844,15 @@
           <t>1</t>
         </is>
       </c>
-      <c r="D25" t="n">
-        <v>17</v>
-      </c>
-      <c r="E25" t="n">
-        <v>1.2988</v>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>17.0</t>
+        </is>
+      </c>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>1.2988</t>
+        </is>
       </c>
       <c r="F25" t="inlineStr"/>
       <c r="G25" t="inlineStr"/>
@@ -2560,25 +2886,35 @@
           <t>L19520873</t>
         </is>
       </c>
-      <c r="N25" t="n">
-        <v>1</v>
-      </c>
-      <c r="O25" t="n">
-        <v>0</v>
+      <c r="N25" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="O25" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
       </c>
       <c r="P25" t="inlineStr">
         <is>
           <t>SUCCESS</t>
         </is>
       </c>
-      <c r="Q25" t="n">
-        <v>1</v>
-      </c>
-      <c r="R25" t="n">
-        <v>1784984402</v>
-      </c>
-      <c r="S25" t="n">
-        <v>1784988000</v>
+      <c r="Q25" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="R25" t="inlineStr">
+        <is>
+          <t>1784984402</t>
+        </is>
+      </c>
+      <c r="S25" t="inlineStr">
+        <is>
+          <t>1784988000</t>
+        </is>
       </c>
       <c r="T25" t="inlineStr">
         <is>
@@ -2608,11 +2944,15 @@
           <t>1</t>
         </is>
       </c>
-      <c r="D26" t="n">
-        <v>41</v>
-      </c>
-      <c r="E26" t="n">
-        <v>1.685</v>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>41.0</t>
+        </is>
+      </c>
+      <c r="E26" t="inlineStr">
+        <is>
+          <t>1.685</t>
+        </is>
       </c>
       <c r="F26" t="inlineStr"/>
       <c r="G26" t="inlineStr"/>
@@ -2646,25 +2986,35 @@
           <t>L19520873</t>
         </is>
       </c>
-      <c r="N26" t="n">
-        <v>1</v>
-      </c>
-      <c r="O26" t="n">
-        <v>0</v>
+      <c r="N26" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="O26" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
       </c>
       <c r="P26" t="inlineStr">
         <is>
           <t>SUCCESS</t>
         </is>
       </c>
-      <c r="Q26" t="n">
-        <v>1</v>
-      </c>
-      <c r="R26" t="n">
-        <v>1784984401</v>
-      </c>
-      <c r="S26" t="n">
-        <v>1784988000</v>
+      <c r="Q26" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="R26" t="inlineStr">
+        <is>
+          <t>1784984401</t>
+        </is>
+      </c>
+      <c r="S26" t="inlineStr">
+        <is>
+          <t>1784988000</t>
+        </is>
       </c>
       <c r="T26" t="inlineStr">
         <is>
@@ -2694,11 +3044,15 @@
           <t>1</t>
         </is>
       </c>
-      <c r="D27" t="n">
-        <v>6</v>
-      </c>
-      <c r="E27" t="n">
-        <v>1.5537</v>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>6.0</t>
+        </is>
+      </c>
+      <c r="E27" t="inlineStr">
+        <is>
+          <t>1.5537</t>
+        </is>
       </c>
       <c r="F27" t="inlineStr"/>
       <c r="G27" t="inlineStr"/>
@@ -2732,25 +3086,35 @@
           <t>L19520873</t>
         </is>
       </c>
-      <c r="N27" t="n">
-        <v>1</v>
-      </c>
-      <c r="O27" t="n">
-        <v>0</v>
+      <c r="N27" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="O27" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
       </c>
       <c r="P27" t="inlineStr">
         <is>
           <t>SUCCESS</t>
         </is>
       </c>
-      <c r="Q27" t="n">
-        <v>1</v>
-      </c>
-      <c r="R27" t="n">
-        <v>1784983849</v>
-      </c>
-      <c r="S27" t="n">
-        <v>1784988000</v>
+      <c r="Q27" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="R27" t="inlineStr">
+        <is>
+          <t>1784983849</t>
+        </is>
+      </c>
+      <c r="S27" t="inlineStr">
+        <is>
+          <t>1784988000</t>
+        </is>
       </c>
       <c r="T27" t="inlineStr">
         <is>
@@ -2780,11 +3144,15 @@
           <t>1</t>
         </is>
       </c>
-      <c r="D28" t="n">
-        <v>25</v>
-      </c>
-      <c r="E28" t="n">
-        <v>1.5513</v>
+      <c r="D28" t="inlineStr">
+        <is>
+          <t>25.0</t>
+        </is>
+      </c>
+      <c r="E28" t="inlineStr">
+        <is>
+          <t>1.5513</t>
+        </is>
       </c>
       <c r="F28" t="inlineStr"/>
       <c r="G28" t="inlineStr"/>
@@ -2818,25 +3186,35 @@
           <t>L19520873</t>
         </is>
       </c>
-      <c r="N28" t="n">
-        <v>1</v>
-      </c>
-      <c r="O28" t="n">
-        <v>0</v>
+      <c r="N28" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="O28" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
       </c>
       <c r="P28" t="inlineStr">
         <is>
           <t>SUCCESS</t>
         </is>
       </c>
-      <c r="Q28" t="n">
-        <v>1</v>
-      </c>
-      <c r="R28" t="n">
-        <v>1784983797</v>
-      </c>
-      <c r="S28" t="n">
-        <v>1784988000</v>
+      <c r="Q28" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="R28" t="inlineStr">
+        <is>
+          <t>1784983797</t>
+        </is>
+      </c>
+      <c r="S28" t="inlineStr">
+        <is>
+          <t>1784988000</t>
+        </is>
       </c>
       <c r="T28" t="inlineStr">
         <is>
@@ -2853,7 +3231,7 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>0x78c593e23cd10a2517f77039f922e2d360ba0b6d4c89dc91bac22f6854ce01ea</t>
+          <t>0xc913b7104d801ceb0283dc9eefcce577969c93f7b16c1cc5515036561b5b8d8e</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
@@ -2863,14 +3241,18 @@
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="D29" t="n">
-        <v>2</v>
-      </c>
-      <c r="E29" t="n">
-        <v>1.5513</v>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="D29" t="inlineStr">
+        <is>
+          <t>4.0</t>
+        </is>
+      </c>
+      <c r="E29" t="inlineStr">
+        <is>
+          <t>1.7712</t>
+        </is>
       </c>
       <c r="F29" t="inlineStr"/>
       <c r="G29" t="inlineStr"/>
@@ -2896,7 +3278,7 @@
       </c>
       <c r="L29" t="inlineStr">
         <is>
-          <t>0x04fd78e33c10fb928e409323c26948f49fe4c81fcd47748d9153c9c611b38d0b</t>
+          <t>0x91a9ea8ebfd8b049218a8e072590d2f657e26fdb1f2a49b1016ae42171c68ef2</t>
         </is>
       </c>
       <c r="M29" t="inlineStr">
@@ -2904,29 +3286,39 @@
           <t>L19520873</t>
         </is>
       </c>
-      <c r="N29" t="n">
-        <v>1</v>
-      </c>
-      <c r="O29" t="n">
-        <v>0</v>
+      <c r="N29" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="O29" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
       </c>
       <c r="P29" t="inlineStr">
         <is>
           <t>SUCCESS</t>
         </is>
       </c>
-      <c r="Q29" t="n">
-        <v>1</v>
-      </c>
-      <c r="R29" t="n">
-        <v>1784983703</v>
-      </c>
-      <c r="S29" t="n">
-        <v>1784988000</v>
+      <c r="Q29" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="R29" t="inlineStr">
+        <is>
+          <t>1784983703</t>
+        </is>
+      </c>
+      <c r="S29" t="inlineStr">
+        <is>
+          <t>1784988000</t>
+        </is>
       </c>
       <c r="T29" t="inlineStr">
         <is>
-          <t>4.389968</t>
+          <t>5.770489</t>
         </is>
       </c>
       <c r="U29" t="inlineStr">
@@ -2939,7 +3331,7 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>0xc913b7104d801ceb0283dc9eefcce577969c93f7b16c1cc5515036561b5b8d8e</t>
+          <t>0x78c593e23cd10a2517f77039f922e2d360ba0b6d4c89dc91bac22f6854ce01ea</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
@@ -2949,14 +3341,18 @@
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>2</t>
-        </is>
-      </c>
-      <c r="D30" t="n">
-        <v>4</v>
-      </c>
-      <c r="E30" t="n">
-        <v>1.7712</v>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="D30" t="inlineStr">
+        <is>
+          <t>2.0</t>
+        </is>
+      </c>
+      <c r="E30" t="inlineStr">
+        <is>
+          <t>1.5513</t>
+        </is>
       </c>
       <c r="F30" t="inlineStr"/>
       <c r="G30" t="inlineStr"/>
@@ -2982,7 +3378,7 @@
       </c>
       <c r="L30" t="inlineStr">
         <is>
-          <t>0x91a9ea8ebfd8b049218a8e072590d2f657e26fdb1f2a49b1016ae42171c68ef2</t>
+          <t>0x04fd78e33c10fb928e409323c26948f49fe4c81fcd47748d9153c9c611b38d0b</t>
         </is>
       </c>
       <c r="M30" t="inlineStr">
@@ -2990,29 +3386,39 @@
           <t>L19520873</t>
         </is>
       </c>
-      <c r="N30" t="n">
-        <v>1</v>
-      </c>
-      <c r="O30" t="n">
-        <v>0</v>
+      <c r="N30" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="O30" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
       </c>
       <c r="P30" t="inlineStr">
         <is>
           <t>SUCCESS</t>
         </is>
       </c>
-      <c r="Q30" t="n">
-        <v>1</v>
-      </c>
-      <c r="R30" t="n">
-        <v>1784983703</v>
-      </c>
-      <c r="S30" t="n">
-        <v>1784988000</v>
+      <c r="Q30" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="R30" t="inlineStr">
+        <is>
+          <t>1784983703</t>
+        </is>
+      </c>
+      <c r="S30" t="inlineStr">
+        <is>
+          <t>1784988000</t>
+        </is>
       </c>
       <c r="T30" t="inlineStr">
         <is>
-          <t>5.770489</t>
+          <t>4.389968</t>
         </is>
       </c>
       <c r="U30" t="inlineStr">
@@ -3038,11 +3444,15 @@
           <t>1</t>
         </is>
       </c>
-      <c r="D31" t="n">
-        <v>12</v>
-      </c>
-      <c r="E31" t="n">
-        <v>1.5513</v>
+      <c r="D31" t="inlineStr">
+        <is>
+          <t>12.0</t>
+        </is>
+      </c>
+      <c r="E31" t="inlineStr">
+        <is>
+          <t>1.5513</t>
+        </is>
       </c>
       <c r="F31" t="inlineStr"/>
       <c r="G31" t="inlineStr"/>
@@ -3076,25 +3486,35 @@
           <t>L19520873</t>
         </is>
       </c>
-      <c r="N31" t="n">
-        <v>1</v>
-      </c>
-      <c r="O31" t="n">
-        <v>0</v>
+      <c r="N31" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="O31" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
       </c>
       <c r="P31" t="inlineStr">
         <is>
           <t>SUCCESS</t>
         </is>
       </c>
-      <c r="Q31" t="n">
-        <v>1</v>
-      </c>
-      <c r="R31" t="n">
-        <v>1784983480</v>
-      </c>
-      <c r="S31" t="n">
-        <v>1784988000</v>
+      <c r="Q31" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="R31" t="inlineStr">
+        <is>
+          <t>1784983480</t>
+        </is>
+      </c>
+      <c r="S31" t="inlineStr">
+        <is>
+          <t>1784988000</t>
+        </is>
       </c>
       <c r="T31" t="inlineStr">
         <is>
@@ -3124,11 +3544,15 @@
           <t>1</t>
         </is>
       </c>
-      <c r="D32" t="n">
-        <v>1</v>
-      </c>
-      <c r="E32" t="n">
-        <v>1.5513</v>
+      <c r="D32" t="inlineStr">
+        <is>
+          <t>1.0</t>
+        </is>
+      </c>
+      <c r="E32" t="inlineStr">
+        <is>
+          <t>1.5513</t>
+        </is>
       </c>
       <c r="F32" t="inlineStr"/>
       <c r="G32" t="inlineStr"/>
@@ -3162,25 +3586,35 @@
           <t>L19520873</t>
         </is>
       </c>
-      <c r="N32" t="n">
-        <v>1</v>
-      </c>
-      <c r="O32" t="n">
-        <v>0</v>
+      <c r="N32" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="O32" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
       </c>
       <c r="P32" t="inlineStr">
         <is>
           <t>SUCCESS</t>
         </is>
       </c>
-      <c r="Q32" t="n">
-        <v>1</v>
-      </c>
-      <c r="R32" t="n">
-        <v>1784983361</v>
-      </c>
-      <c r="S32" t="n">
-        <v>1784988000</v>
+      <c r="Q32" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="R32" t="inlineStr">
+        <is>
+          <t>1784983361</t>
+        </is>
+      </c>
+      <c r="S32" t="inlineStr">
+        <is>
+          <t>1784988000</t>
+        </is>
       </c>
       <c r="T32" t="inlineStr">
         <is>
@@ -3210,11 +3644,15 @@
           <t>1</t>
         </is>
       </c>
-      <c r="D33" t="n">
-        <v>0</v>
-      </c>
-      <c r="E33" t="n">
-        <v>1.215</v>
+      <c r="D33" t="inlineStr">
+        <is>
+          <t>0.0</t>
+        </is>
+      </c>
+      <c r="E33" t="inlineStr">
+        <is>
+          <t>1.215</t>
+        </is>
       </c>
       <c r="F33" t="inlineStr"/>
       <c r="G33" t="inlineStr"/>
@@ -3248,25 +3686,35 @@
           <t>L19520873</t>
         </is>
       </c>
-      <c r="N33" t="n">
-        <v>1</v>
-      </c>
-      <c r="O33" t="n">
-        <v>0</v>
+      <c r="N33" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="O33" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
       </c>
       <c r="P33" t="inlineStr">
         <is>
           <t>SUCCESS</t>
         </is>
       </c>
-      <c r="Q33" t="n">
-        <v>1</v>
-      </c>
-      <c r="R33" t="n">
-        <v>1784981088</v>
-      </c>
-      <c r="S33" t="n">
-        <v>1784988000</v>
+      <c r="Q33" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="R33" t="inlineStr">
+        <is>
+          <t>1784981088</t>
+        </is>
+      </c>
+      <c r="S33" t="inlineStr">
+        <is>
+          <t>1784988000</t>
+        </is>
       </c>
       <c r="T33" t="inlineStr">
         <is>
@@ -3296,11 +3744,15 @@
           <t>2</t>
         </is>
       </c>
-      <c r="D34" t="n">
-        <v>16</v>
-      </c>
-      <c r="E34" t="n">
-        <v>1.7712</v>
+      <c r="D34" t="inlineStr">
+        <is>
+          <t>16.0</t>
+        </is>
+      </c>
+      <c r="E34" t="inlineStr">
+        <is>
+          <t>1.7712</t>
+        </is>
       </c>
       <c r="F34" t="inlineStr"/>
       <c r="G34" t="inlineStr"/>
@@ -3334,25 +3786,35 @@
           <t>L19520873</t>
         </is>
       </c>
-      <c r="N34" t="n">
-        <v>1</v>
-      </c>
-      <c r="O34" t="n">
-        <v>0</v>
+      <c r="N34" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="O34" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
       </c>
       <c r="P34" t="inlineStr">
         <is>
           <t>SUCCESS</t>
         </is>
       </c>
-      <c r="Q34" t="n">
-        <v>1</v>
-      </c>
-      <c r="R34" t="n">
-        <v>1784981082</v>
-      </c>
-      <c r="S34" t="n">
-        <v>1784988000</v>
+      <c r="Q34" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="R34" t="inlineStr">
+        <is>
+          <t>1784981082</t>
+        </is>
+      </c>
+      <c r="S34" t="inlineStr">
+        <is>
+          <t>1784988000</t>
+        </is>
       </c>
       <c r="T34" t="inlineStr">
         <is>
@@ -3382,11 +3844,15 @@
           <t>1</t>
         </is>
       </c>
-      <c r="D35" t="n">
-        <v>19</v>
-      </c>
-      <c r="E35" t="n">
-        <v>1.5513</v>
+      <c r="D35" t="inlineStr">
+        <is>
+          <t>19.0</t>
+        </is>
+      </c>
+      <c r="E35" t="inlineStr">
+        <is>
+          <t>1.5513</t>
+        </is>
       </c>
       <c r="F35" t="inlineStr"/>
       <c r="G35" t="inlineStr"/>
@@ -3420,25 +3886,35 @@
           <t>L19520873</t>
         </is>
       </c>
-      <c r="N35" t="n">
-        <v>1</v>
-      </c>
-      <c r="O35" t="n">
-        <v>0</v>
+      <c r="N35" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="O35" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
       </c>
       <c r="P35" t="inlineStr">
         <is>
           <t>SUCCESS</t>
         </is>
       </c>
-      <c r="Q35" t="n">
-        <v>1</v>
-      </c>
-      <c r="R35" t="n">
-        <v>1784980847</v>
-      </c>
-      <c r="S35" t="n">
-        <v>1784988000</v>
+      <c r="Q35" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="R35" t="inlineStr">
+        <is>
+          <t>1784980847</t>
+        </is>
+      </c>
+      <c r="S35" t="inlineStr">
+        <is>
+          <t>1784988000</t>
+        </is>
       </c>
       <c r="T35" t="inlineStr">
         <is>
@@ -3468,11 +3944,15 @@
           <t>1</t>
         </is>
       </c>
-      <c r="D36" t="n">
-        <v>22</v>
-      </c>
-      <c r="E36" t="n">
-        <v>1.555</v>
+      <c r="D36" t="inlineStr">
+        <is>
+          <t>22.0</t>
+        </is>
+      </c>
+      <c r="E36" t="inlineStr">
+        <is>
+          <t>1.555</t>
+        </is>
       </c>
       <c r="F36" t="inlineStr"/>
       <c r="G36" t="inlineStr"/>
@@ -3506,25 +3986,35 @@
           <t>L19520873</t>
         </is>
       </c>
-      <c r="N36" t="n">
-        <v>1</v>
-      </c>
-      <c r="O36" t="n">
-        <v>0</v>
+      <c r="N36" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="O36" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
       </c>
       <c r="P36" t="inlineStr">
         <is>
           <t>SUCCESS</t>
         </is>
       </c>
-      <c r="Q36" t="n">
-        <v>1</v>
-      </c>
-      <c r="R36" t="n">
-        <v>1784977858</v>
-      </c>
-      <c r="S36" t="n">
-        <v>1784988000</v>
+      <c r="Q36" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="R36" t="inlineStr">
+        <is>
+          <t>1784977858</t>
+        </is>
+      </c>
+      <c r="S36" t="inlineStr">
+        <is>
+          <t>1784988000</t>
+        </is>
       </c>
       <c r="T36" t="inlineStr">
         <is>
@@ -3554,11 +4044,15 @@
           <t>1</t>
         </is>
       </c>
-      <c r="D37" t="n">
-        <v>27</v>
-      </c>
-      <c r="E37" t="n">
-        <v>1.555</v>
+      <c r="D37" t="inlineStr">
+        <is>
+          <t>27.0</t>
+        </is>
+      </c>
+      <c r="E37" t="inlineStr">
+        <is>
+          <t>1.555</t>
+        </is>
       </c>
       <c r="F37" t="inlineStr"/>
       <c r="G37" t="inlineStr"/>
@@ -3592,25 +4086,35 @@
           <t>L19520873</t>
         </is>
       </c>
-      <c r="N37" t="n">
-        <v>1</v>
-      </c>
-      <c r="O37" t="n">
-        <v>0</v>
+      <c r="N37" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="O37" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
       </c>
       <c r="P37" t="inlineStr">
         <is>
           <t>SUCCESS</t>
         </is>
       </c>
-      <c r="Q37" t="n">
-        <v>1</v>
-      </c>
-      <c r="R37" t="n">
-        <v>1784977853</v>
-      </c>
-      <c r="S37" t="n">
-        <v>1784988000</v>
+      <c r="Q37" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="R37" t="inlineStr">
+        <is>
+          <t>1784977853</t>
+        </is>
+      </c>
+      <c r="S37" t="inlineStr">
+        <is>
+          <t>1784988000</t>
+        </is>
       </c>
       <c r="T37" t="inlineStr">
         <is>
@@ -3640,11 +4144,15 @@
           <t>2</t>
         </is>
       </c>
-      <c r="D38" t="n">
-        <v>20</v>
-      </c>
-      <c r="E38" t="n">
-        <v>1.435</v>
+      <c r="D38" t="inlineStr">
+        <is>
+          <t>20.0</t>
+        </is>
+      </c>
+      <c r="E38" t="inlineStr">
+        <is>
+          <t>1.435</t>
+        </is>
       </c>
       <c r="F38" t="inlineStr"/>
       <c r="G38" t="inlineStr"/>
@@ -3678,25 +4186,35 @@
           <t>L19520873</t>
         </is>
       </c>
-      <c r="N38" t="n">
-        <v>1</v>
-      </c>
-      <c r="O38" t="n">
-        <v>0</v>
+      <c r="N38" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="O38" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
       </c>
       <c r="P38" t="inlineStr">
         <is>
           <t>SUCCESS</t>
         </is>
       </c>
-      <c r="Q38" t="n">
-        <v>1</v>
-      </c>
-      <c r="R38" t="n">
-        <v>1784968614</v>
-      </c>
-      <c r="S38" t="n">
-        <v>1784988000</v>
+      <c r="Q38" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="R38" t="inlineStr">
+        <is>
+          <t>1784968614</t>
+        </is>
+      </c>
+      <c r="S38" t="inlineStr">
+        <is>
+          <t>1784988000</t>
+        </is>
       </c>
       <c r="T38" t="inlineStr">
         <is>
@@ -3726,11 +4244,15 @@
           <t>1</t>
         </is>
       </c>
-      <c r="D39" t="n">
-        <v>10</v>
-      </c>
-      <c r="E39" t="n">
-        <v>1.56</v>
+      <c r="D39" t="inlineStr">
+        <is>
+          <t>10.0</t>
+        </is>
+      </c>
+      <c r="E39" t="inlineStr">
+        <is>
+          <t>1.56</t>
+        </is>
       </c>
       <c r="F39" t="inlineStr"/>
       <c r="G39" t="inlineStr"/>
@@ -3764,25 +4286,35 @@
           <t>L19520873</t>
         </is>
       </c>
-      <c r="N39" t="n">
-        <v>1</v>
-      </c>
-      <c r="O39" t="n">
-        <v>0</v>
+      <c r="N39" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="O39" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
       </c>
       <c r="P39" t="inlineStr">
         <is>
           <t>SUCCESS</t>
         </is>
       </c>
-      <c r="Q39" t="n">
-        <v>1</v>
-      </c>
-      <c r="R39" t="n">
-        <v>1784907257</v>
-      </c>
-      <c r="S39" t="n">
-        <v>1784988000</v>
+      <c r="Q39" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="R39" t="inlineStr">
+        <is>
+          <t>1784907257</t>
+        </is>
+      </c>
+      <c r="S39" t="inlineStr">
+        <is>
+          <t>1784988000</t>
+        </is>
       </c>
       <c r="T39" t="inlineStr">
         <is>
@@ -3812,11 +4344,15 @@
           <t>1</t>
         </is>
       </c>
-      <c r="D40" t="n">
-        <v>26</v>
-      </c>
-      <c r="E40" t="n">
-        <v>1.5737</v>
+      <c r="D40" t="inlineStr">
+        <is>
+          <t>26.0</t>
+        </is>
+      </c>
+      <c r="E40" t="inlineStr">
+        <is>
+          <t>1.5737</t>
+        </is>
       </c>
       <c r="F40" t="inlineStr"/>
       <c r="G40" t="inlineStr"/>
@@ -3850,25 +4386,35 @@
           <t>L19520873</t>
         </is>
       </c>
-      <c r="N40" t="n">
-        <v>1</v>
-      </c>
-      <c r="O40" t="n">
-        <v>0</v>
+      <c r="N40" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="O40" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
       </c>
       <c r="P40" t="inlineStr">
         <is>
           <t>SUCCESS</t>
         </is>
       </c>
-      <c r="Q40" t="n">
-        <v>1</v>
-      </c>
-      <c r="R40" t="n">
-        <v>1784907053</v>
-      </c>
-      <c r="S40" t="n">
-        <v>1784988000</v>
+      <c r="Q40" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="R40" t="inlineStr">
+        <is>
+          <t>1784907053</t>
+        </is>
+      </c>
+      <c r="S40" t="inlineStr">
+        <is>
+          <t>1784988000</t>
+        </is>
       </c>
       <c r="T40" t="inlineStr">
         <is>
@@ -3898,11 +4444,15 @@
           <t>1</t>
         </is>
       </c>
-      <c r="D41" t="n">
-        <v>14</v>
-      </c>
-      <c r="E41" t="n">
-        <v>1.315</v>
+      <c r="D41" t="inlineStr">
+        <is>
+          <t>14.0</t>
+        </is>
+      </c>
+      <c r="E41" t="inlineStr">
+        <is>
+          <t>1.315</t>
+        </is>
       </c>
       <c r="F41" t="inlineStr"/>
       <c r="G41" t="inlineStr"/>
@@ -3936,25 +4486,35 @@
           <t>L19520873</t>
         </is>
       </c>
-      <c r="N41" t="n">
-        <v>1</v>
-      </c>
-      <c r="O41" t="n">
-        <v>0</v>
+      <c r="N41" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="O41" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
       </c>
       <c r="P41" t="inlineStr">
         <is>
           <t>SUCCESS</t>
         </is>
       </c>
-      <c r="Q41" t="n">
-        <v>1</v>
-      </c>
-      <c r="R41" t="n">
-        <v>1784907041</v>
-      </c>
-      <c r="S41" t="n">
-        <v>1784988000</v>
+      <c r="Q41" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="R41" t="inlineStr">
+        <is>
+          <t>1784907041</t>
+        </is>
+      </c>
+      <c r="S41" t="inlineStr">
+        <is>
+          <t>1784988000</t>
+        </is>
       </c>
       <c r="T41" t="inlineStr">
         <is>
@@ -3984,11 +4544,15 @@
           <t>1</t>
         </is>
       </c>
-      <c r="D42" t="n">
-        <v>14</v>
-      </c>
-      <c r="E42" t="n">
-        <v>1.315</v>
+      <c r="D42" t="inlineStr">
+        <is>
+          <t>14.0</t>
+        </is>
+      </c>
+      <c r="E42" t="inlineStr">
+        <is>
+          <t>1.315</t>
+        </is>
       </c>
       <c r="F42" t="inlineStr"/>
       <c r="G42" t="inlineStr"/>
@@ -4022,25 +4586,35 @@
           <t>L19520873</t>
         </is>
       </c>
-      <c r="N42" t="n">
-        <v>1</v>
-      </c>
-      <c r="O42" t="n">
-        <v>0</v>
+      <c r="N42" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="O42" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
       </c>
       <c r="P42" t="inlineStr">
         <is>
           <t>SUCCESS</t>
         </is>
       </c>
-      <c r="Q42" t="n">
-        <v>1</v>
-      </c>
-      <c r="R42" t="n">
-        <v>1784907041</v>
-      </c>
-      <c r="S42" t="n">
-        <v>1784988000</v>
+      <c r="Q42" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="R42" t="inlineStr">
+        <is>
+          <t>1784907041</t>
+        </is>
+      </c>
+      <c r="S42" t="inlineStr">
+        <is>
+          <t>1784988000</t>
+        </is>
       </c>
       <c r="T42" t="inlineStr">
         <is>
@@ -4057,7 +4631,7 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>0x3f981c0415a637d3cb9137ae5b4b0b4b0c50f1a3af5d4e42f65e682f80daadba</t>
+          <t>0xdaf8fe8a287cecb340987a0eebd287e9d8e007af24d015fcadd720fceba485cd</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
@@ -4070,11 +4644,15 @@
           <t>1</t>
         </is>
       </c>
-      <c r="D43" t="n">
-        <v>22</v>
-      </c>
-      <c r="E43" t="n">
-        <v>1.4625</v>
+      <c r="D43" t="inlineStr">
+        <is>
+          <t>26.0</t>
+        </is>
+      </c>
+      <c r="E43" t="inlineStr">
+        <is>
+          <t>1.57</t>
+        </is>
       </c>
       <c r="F43" t="inlineStr"/>
       <c r="G43" t="inlineStr"/>
@@ -4100,7 +4678,7 @@
       </c>
       <c r="L43" t="inlineStr">
         <is>
-          <t>0xd5ae8f2322bcc6adaca1c1bb1baf6a74afa50cc30131840c87632f67865c23d0</t>
+          <t>0xe1204c11efd43d8d3a0377591c468bba3ac169f58ab541c6d60665f2e0bbb051</t>
         </is>
       </c>
       <c r="M43" t="inlineStr">
@@ -4108,29 +4686,39 @@
           <t>L19520873</t>
         </is>
       </c>
-      <c r="N43" t="n">
-        <v>1</v>
-      </c>
-      <c r="O43" t="n">
-        <v>0</v>
+      <c r="N43" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="O43" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
       </c>
       <c r="P43" t="inlineStr">
         <is>
           <t>SUCCESS</t>
         </is>
       </c>
-      <c r="Q43" t="n">
-        <v>1</v>
-      </c>
-      <c r="R43" t="n">
-        <v>1784907040</v>
-      </c>
-      <c r="S43" t="n">
-        <v>1784988000</v>
+      <c r="Q43" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="R43" t="inlineStr">
+        <is>
+          <t>1784907040</t>
+        </is>
+      </c>
+      <c r="S43" t="inlineStr">
+        <is>
+          <t>1784988000</t>
+        </is>
       </c>
       <c r="T43" t="inlineStr">
         <is>
-          <t>47.589189</t>
+          <t>47.046509</t>
         </is>
       </c>
       <c r="U43" t="inlineStr">
@@ -4143,7 +4731,7 @@
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>0xdaf8fe8a287cecb340987a0eebd287e9d8e007af24d015fcadd720fceba485cd</t>
+          <t>0x3f981c0415a637d3cb9137ae5b4b0b4b0c50f1a3af5d4e42f65e682f80daadba</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
@@ -4156,11 +4744,15 @@
           <t>1</t>
         </is>
       </c>
-      <c r="D44" t="n">
-        <v>26</v>
-      </c>
-      <c r="E44" t="n">
-        <v>1.57</v>
+      <c r="D44" t="inlineStr">
+        <is>
+          <t>22.0</t>
+        </is>
+      </c>
+      <c r="E44" t="inlineStr">
+        <is>
+          <t>1.4625</t>
+        </is>
       </c>
       <c r="F44" t="inlineStr"/>
       <c r="G44" t="inlineStr"/>
@@ -4186,7 +4778,7 @@
       </c>
       <c r="L44" t="inlineStr">
         <is>
-          <t>0xe1204c11efd43d8d3a0377591c468bba3ac169f58ab541c6d60665f2e0bbb051</t>
+          <t>0xd5ae8f2322bcc6adaca1c1bb1baf6a74afa50cc30131840c87632f67865c23d0</t>
         </is>
       </c>
       <c r="M44" t="inlineStr">
@@ -4194,29 +4786,39 @@
           <t>L19520873</t>
         </is>
       </c>
-      <c r="N44" t="n">
-        <v>1</v>
-      </c>
-      <c r="O44" t="n">
-        <v>0</v>
+      <c r="N44" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="O44" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
       </c>
       <c r="P44" t="inlineStr">
         <is>
           <t>SUCCESS</t>
         </is>
       </c>
-      <c r="Q44" t="n">
-        <v>1</v>
-      </c>
-      <c r="R44" t="n">
-        <v>1784907040</v>
-      </c>
-      <c r="S44" t="n">
-        <v>1784988000</v>
+      <c r="Q44" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="R44" t="inlineStr">
+        <is>
+          <t>1784907040</t>
+        </is>
+      </c>
+      <c r="S44" t="inlineStr">
+        <is>
+          <t>1784988000</t>
+        </is>
       </c>
       <c r="T44" t="inlineStr">
         <is>
-          <t>47.046509</t>
+          <t>47.589189</t>
         </is>
       </c>
       <c r="U44" t="inlineStr">

</xml_diff>

<commit_message>
Update soccer trades 2026-07-26 13:06:15 UTC
</commit_message>
<xml_diff>
--- a/data/sxbet/ligas/Besta Deild Karla/trades.xlsx
+++ b/data/sxbet/ligas/Besta Deild Karla/trades.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Sheet" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>

</xml_diff>

<commit_message>
Update soccer trades 2026-07-28 12:01:26 UTC
</commit_message>
<xml_diff>
--- a/data/sxbet/ligas/Besta Deild Karla/trades.xlsx
+++ b/data/sxbet/ligas/Besta Deild Karla/trades.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:V44"/>
+  <dimension ref="A1:V48"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -531,30 +531,30 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>0x65bc0b70a6148d6f136b1552723c33dcf058e2ee7e6097ad6d18a39367f4821b</t>
+          <t>0x79c1f616b380c93f42fe785c942a2cc39edc55c4cdd4d5b6a09024c926a74f60</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>0x4a09916b1325Eed50eE8973B13742a205B0B7c7E</t>
-        </is>
-      </c>
-      <c r="C2" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
+          <t>0x97EC1C9682F70091efB04e97b0B34698cF815EE1</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr"/>
       <c r="D2" t="inlineStr">
         <is>
-          <t>35.0</t>
+          <t>11.22999</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>1.5987</t>
-        </is>
-      </c>
-      <c r="F2" t="inlineStr"/>
+          <t>1.5413</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>Under/Over (4)</t>
+        </is>
+      </c>
       <c r="G2" t="inlineStr"/>
       <c r="H2" t="inlineStr">
         <is>
@@ -563,32 +563,32 @@
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>IR Reykjavik vs Fylkir</t>
+          <t>Aegir vs Njardvik</t>
         </is>
       </c>
       <c r="J2" t="inlineStr">
         <is>
-          <t>IR Reykjavik</t>
+          <t>Aegir</t>
         </is>
       </c>
       <c r="K2" t="inlineStr">
         <is>
-          <t>Fylkir</t>
+          <t>Njardvik</t>
         </is>
       </c>
       <c r="L2" t="inlineStr">
         <is>
-          <t>0xef2cff3047642c7d3f79713526decc2ed1438c01d374590eb62929362f824801</t>
+          <t>0xde9c2677ae0e84c01c06a23050c75f29399db6bd766b2ef90484b73f8e0bbaed</t>
         </is>
       </c>
       <c r="M2" t="inlineStr">
         <is>
-          <t>L19520873</t>
+          <t>L19548408</t>
         </is>
       </c>
       <c r="N2" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>0</t>
         </is>
       </c>
       <c r="O2" t="inlineStr">
@@ -608,17 +608,17 @@
       </c>
       <c r="R2" t="inlineStr">
         <is>
-          <t>1784987195</t>
+          <t>1785237449</t>
         </is>
       </c>
       <c r="S2" t="inlineStr">
         <is>
-          <t>1784988000</t>
+          <t>1785266100</t>
         </is>
       </c>
       <c r="T2" t="inlineStr">
         <is>
-          <t>59.090338</t>
+          <t>20.748249</t>
         </is>
       </c>
       <c r="U2" t="inlineStr">
@@ -626,35 +626,39 @@
           <t>SXR</t>
         </is>
       </c>
-      <c r="V2" t="inlineStr"/>
+      <c r="V2" t="inlineStr">
+        <is>
+          <t>0x6629Ce1Cf35Cc1329ebB4F63202F3f197b3F050B</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>0xd5e3b95bd82e0d7627a9203f0fe8fdd3b068e15fd373a543e05b207e66faf2a0</t>
+          <t>0xce612ac2221331f875649902eb6a0cde4b9db2f0f597bbc86e7caced63d25b99</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>0x68E1818FF20BBe84F9be9E0A4A395FB11079Bd35</t>
-        </is>
-      </c>
-      <c r="C3" t="inlineStr">
-        <is>
-          <t>2</t>
-        </is>
-      </c>
+          <t>0x97EC1C9682F70091efB04e97b0B34698cF815EE1</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr"/>
       <c r="D3" t="inlineStr">
         <is>
-          <t>12.0</t>
+          <t>11.73</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>1.7862</t>
-        </is>
-      </c>
-      <c r="F3" t="inlineStr"/>
+          <t>1.4412</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>Under/Over (3.5)</t>
+        </is>
+      </c>
       <c r="G3" t="inlineStr"/>
       <c r="H3" t="inlineStr">
         <is>
@@ -663,32 +667,32 @@
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>IR Reykjavik vs Fylkir</t>
+          <t>Aegir vs Njardvik</t>
         </is>
       </c>
       <c r="J3" t="inlineStr">
         <is>
-          <t>IR Reykjavik</t>
+          <t>Aegir</t>
         </is>
       </c>
       <c r="K3" t="inlineStr">
         <is>
-          <t>Fylkir</t>
+          <t>Njardvik</t>
         </is>
       </c>
       <c r="L3" t="inlineStr">
         <is>
-          <t>0x2b00f05607bf61216841f59440e877cc0eeb424e834132492c721bd4faedc556</t>
+          <t>0x0825c99784fd72c055ffaeeb62e8e792f152ccd5a39c675722acf968b754f571</t>
         </is>
       </c>
       <c r="M3" t="inlineStr">
         <is>
-          <t>L19520873</t>
+          <t>L19548408</t>
         </is>
       </c>
       <c r="N3" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>0</t>
         </is>
       </c>
       <c r="O3" t="inlineStr">
@@ -708,17 +712,17 @@
       </c>
       <c r="R3" t="inlineStr">
         <is>
-          <t>1784986980</t>
+          <t>1785236520</t>
         </is>
       </c>
       <c r="S3" t="inlineStr">
         <is>
-          <t>1784988000</t>
+          <t>1785266100</t>
         </is>
       </c>
       <c r="T3" t="inlineStr">
         <is>
-          <t>16.327479</t>
+          <t>26.583569</t>
         </is>
       </c>
       <c r="U3" t="inlineStr">
@@ -726,35 +730,39 @@
           <t>SXR</t>
         </is>
       </c>
-      <c r="V3" t="inlineStr"/>
+      <c r="V3" t="inlineStr">
+        <is>
+          <t>0x6629Ce1Cf35Cc1329ebB4F63202F3f197b3F050B</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>0xbfc0a906e601c3195b374e6d33b07e4c0b0dcbf09e05e45b8bd53226678d5d88</t>
+          <t>0x7ae96391e38cfe39539922631da2025b36f57f1831d5f35ec6338463f27cb2a2</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>0x68E1818FF20BBe84F9be9E0A4A395FB11079Bd35</t>
-        </is>
-      </c>
-      <c r="C4" t="inlineStr">
-        <is>
-          <t>2</t>
-        </is>
-      </c>
+          <t>0x5D69C3af95Ff47088b415B25F41b1fFDc8571063</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr"/>
       <c r="D4" t="inlineStr">
         <is>
-          <t>37.0</t>
+          <t>1.03</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>1.7875</t>
-        </is>
-      </c>
-      <c r="F4" t="inlineStr"/>
+          <t>1.5525</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>Under/Over (4)</t>
+        </is>
+      </c>
       <c r="G4" t="inlineStr"/>
       <c r="H4" t="inlineStr">
         <is>
@@ -763,32 +771,32 @@
       </c>
       <c r="I4" t="inlineStr">
         <is>
-          <t>IR Reykjavik vs Fylkir</t>
+          <t>Aegir vs Njardvik</t>
         </is>
       </c>
       <c r="J4" t="inlineStr">
         <is>
-          <t>IR Reykjavik</t>
+          <t>Aegir</t>
         </is>
       </c>
       <c r="K4" t="inlineStr">
         <is>
-          <t>Fylkir</t>
+          <t>Njardvik</t>
         </is>
       </c>
       <c r="L4" t="inlineStr">
         <is>
-          <t>0x2b00f05607bf61216841f59440e877cc0eeb424e834132492c721bd4faedc556</t>
+          <t>0xde9c2677ae0e84c01c06a23050c75f29399db6bd766b2ef90484b73f8e0bbaed</t>
         </is>
       </c>
       <c r="M4" t="inlineStr">
         <is>
-          <t>L19520873</t>
+          <t>L19548408</t>
         </is>
       </c>
       <c r="N4" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>0</t>
         </is>
       </c>
       <c r="O4" t="inlineStr">
@@ -808,17 +816,17 @@
       </c>
       <c r="R4" t="inlineStr">
         <is>
-          <t>1784986980</t>
+          <t>1785236069</t>
         </is>
       </c>
       <c r="S4" t="inlineStr">
         <is>
-          <t>1784988000</t>
+          <t>1785266100</t>
         </is>
       </c>
       <c r="T4" t="inlineStr">
         <is>
-          <t>47.105879</t>
+          <t>1.864253</t>
         </is>
       </c>
       <c r="U4" t="inlineStr">
@@ -826,35 +834,39 @@
           <t>SXR</t>
         </is>
       </c>
-      <c r="V4" t="inlineStr"/>
+      <c r="V4" t="inlineStr">
+        <is>
+          <t>0x6629Ce1Cf35Cc1329ebB4F63202F3f197b3F050B</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>0x5724a3badfc2012619fbf8e1a14ab0e7f4c66de896315371280c186505e86b85</t>
+          <t>0xc979cd389b2d4ca831b9a44b7738a2ae46abf46b1bd95d0fbe5b654a09413b1e</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>0xe2C68b7ef85645e47F9b94382c3Db59b046945a2</t>
-        </is>
-      </c>
-      <c r="C5" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
+          <t>0x97EC1C9682F70091efB04e97b0B34698cF815EE1</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr"/>
       <c r="D5" t="inlineStr">
         <is>
-          <t>69.0</t>
+          <t>5.59</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>1.6012</t>
-        </is>
-      </c>
-      <c r="F5" t="inlineStr"/>
+          <t>1.4525</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>Under/Over (3.5)</t>
+        </is>
+      </c>
       <c r="G5" t="inlineStr"/>
       <c r="H5" t="inlineStr">
         <is>
@@ -863,32 +875,32 @@
       </c>
       <c r="I5" t="inlineStr">
         <is>
-          <t>IR Reykjavik vs Fylkir</t>
+          <t>Aegir vs Njardvik</t>
         </is>
       </c>
       <c r="J5" t="inlineStr">
         <is>
-          <t>IR Reykjavik</t>
+          <t>Aegir</t>
         </is>
       </c>
       <c r="K5" t="inlineStr">
         <is>
-          <t>Fylkir</t>
+          <t>Njardvik</t>
         </is>
       </c>
       <c r="L5" t="inlineStr">
         <is>
-          <t>0x04fd78e33c10fb928e409323c26948f49fe4c81fcd47748d9153c9c611b38d0b</t>
+          <t>0x0825c99784fd72c055ffaeeb62e8e792f152ccd5a39c675722acf968b754f571</t>
         </is>
       </c>
       <c r="M5" t="inlineStr">
         <is>
-          <t>L19520873</t>
+          <t>L19548408</t>
         </is>
       </c>
       <c r="N5" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>0</t>
         </is>
       </c>
       <c r="O5" t="inlineStr">
@@ -908,17 +920,17 @@
       </c>
       <c r="R5" t="inlineStr">
         <is>
-          <t>1784986978</t>
+          <t>1785235526</t>
         </is>
       </c>
       <c r="S5" t="inlineStr">
         <is>
-          <t>1784988000</t>
+          <t>1785266100</t>
         </is>
       </c>
       <c r="T5" t="inlineStr">
         <is>
-          <t>114.884008</t>
+          <t>12.353591</t>
         </is>
       </c>
       <c r="U5" t="inlineStr">
@@ -926,12 +938,16 @@
           <t>SXR</t>
         </is>
       </c>
-      <c r="V5" t="inlineStr"/>
+      <c r="V5" t="inlineStr">
+        <is>
+          <t>0x6629Ce1Cf35Cc1329ebB4F63202F3f197b3F050B</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>0xf825a9ec3149d5a232253fd07078e2ed75a62b287df75e59fbb6c1546f6912a3</t>
+          <t>0x65bc0b70a6148d6f136b1552723c33dcf058e2ee7e6097ad6d18a39367f4821b</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
@@ -946,12 +962,12 @@
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>15.0</t>
+          <t>35.0</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>1.2712</t>
+          <t>1.5987</t>
         </is>
       </c>
       <c r="F6" t="inlineStr"/>
@@ -978,7 +994,7 @@
       </c>
       <c r="L6" t="inlineStr">
         <is>
-          <t>0x06a233f1b733d63cee459a37ac1beffad92b8f9ec21c414e0c26e2876b05eebd</t>
+          <t>0xef2cff3047642c7d3f79713526decc2ed1438c01d374590eb62929362f824801</t>
         </is>
       </c>
       <c r="M6" t="inlineStr">
@@ -1008,7 +1024,7 @@
       </c>
       <c r="R6" t="inlineStr">
         <is>
-          <t>1784984833</t>
+          <t>1784987195</t>
         </is>
       </c>
       <c r="S6" t="inlineStr">
@@ -1018,7 +1034,7 @@
       </c>
       <c r="T6" t="inlineStr">
         <is>
-          <t>58.211982</t>
+          <t>59.090338</t>
         </is>
       </c>
       <c r="U6" t="inlineStr">
@@ -1031,7 +1047,7 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>0x832d570bfcb61240d74893710e1758118ea62888a2bf55921f3190b9a71f4561</t>
+          <t>0xd5e3b95bd82e0d7627a9203f0fe8fdd3b068e15fd373a543e05b207e66faf2a0</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
@@ -1046,12 +1062,12 @@
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>3.0</t>
+          <t>12.0</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>1.7887</t>
+          <t>1.7862</t>
         </is>
       </c>
       <c r="F7" t="inlineStr"/>
@@ -1078,7 +1094,7 @@
       </c>
       <c r="L7" t="inlineStr">
         <is>
-          <t>0x91a9ea8ebfd8b049218a8e072590d2f657e26fdb1f2a49b1016ae42171c68ef2</t>
+          <t>0x2b00f05607bf61216841f59440e877cc0eeb424e834132492c721bd4faedc556</t>
         </is>
       </c>
       <c r="M7" t="inlineStr">
@@ -1108,7 +1124,7 @@
       </c>
       <c r="R7" t="inlineStr">
         <is>
-          <t>1784984812</t>
+          <t>1784986980</t>
         </is>
       </c>
       <c r="S7" t="inlineStr">
@@ -1118,7 +1134,7 @@
       </c>
       <c r="T7" t="inlineStr">
         <is>
-          <t>4.733718</t>
+          <t>16.327479</t>
         </is>
       </c>
       <c r="U7" t="inlineStr">
@@ -1131,7 +1147,7 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>0x78e73a1fbc4bce58e1469ba84a7a75afedee1c817a9927ff72cae6f55f5b4a58</t>
+          <t>0xbfc0a906e601c3195b374e6d33b07e4c0b0dcbf09e05e45b8bd53226678d5d88</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
@@ -1146,12 +1162,12 @@
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>8.0</t>
+          <t>37.0</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>1.7887</t>
+          <t>1.7875</t>
         </is>
       </c>
       <c r="F8" t="inlineStr"/>
@@ -1178,7 +1194,7 @@
       </c>
       <c r="L8" t="inlineStr">
         <is>
-          <t>0x91a9ea8ebfd8b049218a8e072590d2f657e26fdb1f2a49b1016ae42171c68ef2</t>
+          <t>0x2b00f05607bf61216841f59440e877cc0eeb424e834132492c721bd4faedc556</t>
         </is>
       </c>
       <c r="M8" t="inlineStr">
@@ -1208,7 +1224,7 @@
       </c>
       <c r="R8" t="inlineStr">
         <is>
-          <t>1784984812</t>
+          <t>1784986980</t>
         </is>
       </c>
       <c r="S8" t="inlineStr">
@@ -1218,7 +1234,7 @@
       </c>
       <c r="T8" t="inlineStr">
         <is>
-          <t>10.745559</t>
+          <t>47.105879</t>
         </is>
       </c>
       <c r="U8" t="inlineStr">
@@ -1231,12 +1247,12 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>0x02053d570c2ec6485bf734b3e9d25cb6962b678b5212cc142c9b62d371752a01</t>
+          <t>0x5724a3badfc2012619fbf8e1a14ab0e7f4c66de896315371280c186505e86b85</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>0x68E1818FF20BBe84F9be9E0A4A395FB11079Bd35</t>
+          <t>0xe2C68b7ef85645e47F9b94382c3Db59b046945a2</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
@@ -1246,12 +1262,12 @@
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>13.0</t>
+          <t>69.0</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>1.5737</t>
+          <t>1.6012</t>
         </is>
       </c>
       <c r="F9" t="inlineStr"/>
@@ -1308,7 +1324,7 @@
       </c>
       <c r="R9" t="inlineStr">
         <is>
-          <t>1784984812</t>
+          <t>1784986978</t>
         </is>
       </c>
       <c r="S9" t="inlineStr">
@@ -1318,7 +1334,7 @@
       </c>
       <c r="T9" t="inlineStr">
         <is>
-          <t>23.46041</t>
+          <t>114.884008</t>
         </is>
       </c>
       <c r="U9" t="inlineStr">
@@ -1331,7 +1347,7 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>0x6c8964e487e133d59a699205a9a6514d54217a61ad5ca3887aa005a89c8cbdfa</t>
+          <t>0xf825a9ec3149d5a232253fd07078e2ed75a62b287df75e59fbb6c1546f6912a3</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
@@ -1408,7 +1424,7 @@
       </c>
       <c r="R10" t="inlineStr">
         <is>
-          <t>1784984810</t>
+          <t>1784984833</t>
         </is>
       </c>
       <c r="S10" t="inlineStr">
@@ -1418,7 +1434,7 @@
       </c>
       <c r="T10" t="inlineStr">
         <is>
-          <t>58.209253</t>
+          <t>58.211982</t>
         </is>
       </c>
       <c r="U10" t="inlineStr">
@@ -1431,27 +1447,27 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>0xb8b680dda4305fed43c95dc6dbc059c9678abe5f31da65b83ac57ecd5c8d3903</t>
+          <t>0x832d570bfcb61240d74893710e1758118ea62888a2bf55921f3190b9a71f4561</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>0x4a09916b1325Eed50eE8973B13742a205B0B7c7E</t>
+          <t>0x68E1818FF20BBe84F9be9E0A4A395FB11079Bd35</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>16.0</t>
+          <t>3.0</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>1.2712</t>
+          <t>1.7887</t>
         </is>
       </c>
       <c r="F11" t="inlineStr"/>
@@ -1478,7 +1494,7 @@
       </c>
       <c r="L11" t="inlineStr">
         <is>
-          <t>0x06a233f1b733d63cee459a37ac1beffad92b8f9ec21c414e0c26e2876b05eebd</t>
+          <t>0x91a9ea8ebfd8b049218a8e072590d2f657e26fdb1f2a49b1016ae42171c68ef2</t>
         </is>
       </c>
       <c r="M11" t="inlineStr">
@@ -1508,7 +1524,7 @@
       </c>
       <c r="R11" t="inlineStr">
         <is>
-          <t>1784984670</t>
+          <t>1784984812</t>
         </is>
       </c>
       <c r="S11" t="inlineStr">
@@ -1518,7 +1534,7 @@
       </c>
       <c r="T11" t="inlineStr">
         <is>
-          <t>60.198968</t>
+          <t>4.733718</t>
         </is>
       </c>
       <c r="U11" t="inlineStr">
@@ -1531,27 +1547,27 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>0x374cde0708e064be0b99fea4bb71434540b7ca7bbd1a444cb12a8b14c6aa3c48</t>
+          <t>0x78e73a1fbc4bce58e1469ba84a7a75afedee1c817a9927ff72cae6f55f5b4a58</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>0x4a09916b1325Eed50eE8973B13742a205B0B7c7E</t>
+          <t>0x68E1818FF20BBe84F9be9E0A4A395FB11079Bd35</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>16.0</t>
+          <t>8.0</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>1.2712</t>
+          <t>1.7887</t>
         </is>
       </c>
       <c r="F12" t="inlineStr"/>
@@ -1578,7 +1594,7 @@
       </c>
       <c r="L12" t="inlineStr">
         <is>
-          <t>0x06a233f1b733d63cee459a37ac1beffad92b8f9ec21c414e0c26e2876b05eebd</t>
+          <t>0x91a9ea8ebfd8b049218a8e072590d2f657e26fdb1f2a49b1016ae42171c68ef2</t>
         </is>
       </c>
       <c r="M12" t="inlineStr">
@@ -1608,7 +1624,7 @@
       </c>
       <c r="R12" t="inlineStr">
         <is>
-          <t>1784984617</t>
+          <t>1784984812</t>
         </is>
       </c>
       <c r="S12" t="inlineStr">
@@ -1618,7 +1634,7 @@
       </c>
       <c r="T12" t="inlineStr">
         <is>
-          <t>60.198968</t>
+          <t>10.745559</t>
         </is>
       </c>
       <c r="U12" t="inlineStr">
@@ -1631,12 +1647,12 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>0x4c094ddc4f89a7cbd768baf6a26f7e686ead028a4b15ee75fd8f4927e1ad7989</t>
+          <t>0x02053d570c2ec6485bf734b3e9d25cb6962b678b5212cc142c9b62d371752a01</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>0x4a09916b1325Eed50eE8973B13742a205B0B7c7E</t>
+          <t>0x68E1818FF20BBe84F9be9E0A4A395FB11079Bd35</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
@@ -1646,12 +1662,12 @@
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>16.0</t>
+          <t>13.0</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>1.2712</t>
+          <t>1.5737</t>
         </is>
       </c>
       <c r="F13" t="inlineStr"/>
@@ -1678,7 +1694,7 @@
       </c>
       <c r="L13" t="inlineStr">
         <is>
-          <t>0x06a233f1b733d63cee459a37ac1beffad92b8f9ec21c414e0c26e2876b05eebd</t>
+          <t>0x04fd78e33c10fb928e409323c26948f49fe4c81fcd47748d9153c9c611b38d0b</t>
         </is>
       </c>
       <c r="M13" t="inlineStr">
@@ -1708,7 +1724,7 @@
       </c>
       <c r="R13" t="inlineStr">
         <is>
-          <t>1784984581</t>
+          <t>1784984812</t>
         </is>
       </c>
       <c r="S13" t="inlineStr">
@@ -1718,7 +1734,7 @@
       </c>
       <c r="T13" t="inlineStr">
         <is>
-          <t>60.198968</t>
+          <t>23.46041</t>
         </is>
       </c>
       <c r="U13" t="inlineStr">
@@ -1731,7 +1747,7 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>0x7dd8d48e4f9e00707e79d58d5900292571189d9de19bd23c6c6a9a433ea96f72</t>
+          <t>0x6c8964e487e133d59a699205a9a6514d54217a61ad5ca3887aa005a89c8cbdfa</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
@@ -1746,7 +1762,7 @@
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>16.0</t>
+          <t>15.0</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
@@ -1808,7 +1824,7 @@
       </c>
       <c r="R14" t="inlineStr">
         <is>
-          <t>1784984563</t>
+          <t>1784984810</t>
         </is>
       </c>
       <c r="S14" t="inlineStr">
@@ -1818,7 +1834,7 @@
       </c>
       <c r="T14" t="inlineStr">
         <is>
-          <t>60.198968</t>
+          <t>58.209253</t>
         </is>
       </c>
       <c r="U14" t="inlineStr">
@@ -1831,7 +1847,7 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>0x7354c940dd56ae7caca9fa9b1a548dcf53e1a3516f531216c677cf582affb4fe</t>
+          <t>0xb8b680dda4305fed43c95dc6dbc059c9678abe5f31da65b83ac57ecd5c8d3903</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
@@ -1846,12 +1862,12 @@
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>9.0</t>
+          <t>16.0</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>1.3013</t>
+          <t>1.2712</t>
         </is>
       </c>
       <c r="F15" t="inlineStr"/>
@@ -1908,7 +1924,7 @@
       </c>
       <c r="R15" t="inlineStr">
         <is>
-          <t>1784984538</t>
+          <t>1784984670</t>
         </is>
       </c>
       <c r="S15" t="inlineStr">
@@ -1918,7 +1934,7 @@
       </c>
       <c r="T15" t="inlineStr">
         <is>
-          <t>31.184232</t>
+          <t>60.198968</t>
         </is>
       </c>
       <c r="U15" t="inlineStr">
@@ -1931,12 +1947,12 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>0xdc3c1508859b265a9cc7ea3dadc58bb672f939bf46cde2c06081ec2891a03946</t>
+          <t>0x374cde0708e064be0b99fea4bb71434540b7ca7bbd1a444cb12a8b14c6aa3c48</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>0xC88F614A48f8A705d7465b03aAF62ddaca0c3754</t>
+          <t>0x4a09916b1325Eed50eE8973B13742a205B0B7c7E</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
@@ -1946,12 +1962,12 @@
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>21.0</t>
+          <t>16.0</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>1.4363</t>
+          <t>1.2712</t>
         </is>
       </c>
       <c r="F16" t="inlineStr"/>
@@ -1978,7 +1994,7 @@
       </c>
       <c r="L16" t="inlineStr">
         <is>
-          <t>0xd5ae8f2322bcc6adaca1c1bb1baf6a74afa50cc30131840c87632f67865c23d0</t>
+          <t>0x06a233f1b733d63cee459a37ac1beffad92b8f9ec21c414e0c26e2876b05eebd</t>
         </is>
       </c>
       <c r="M16" t="inlineStr">
@@ -2008,7 +2024,7 @@
       </c>
       <c r="R16" t="inlineStr">
         <is>
-          <t>1784984537</t>
+          <t>1784984617</t>
         </is>
       </c>
       <c r="S16" t="inlineStr">
@@ -2018,7 +2034,7 @@
       </c>
       <c r="T16" t="inlineStr">
         <is>
-          <t>48.297994</t>
+          <t>60.198968</t>
         </is>
       </c>
       <c r="U16" t="inlineStr">
@@ -2031,12 +2047,12 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>0x0bf6c8f6ea5d7452bf543eb72d99a66c1b6ff74a5e56b4ad9449b6870f225d2d</t>
+          <t>0x4c094ddc4f89a7cbd768baf6a26f7e686ead028a4b15ee75fd8f4927e1ad7989</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>0x47D0CE9b8d653c8884DB7E2a7F88d4849E0CD980</t>
+          <t>0x4a09916b1325Eed50eE8973B13742a205B0B7c7E</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
@@ -2046,12 +2062,12 @@
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>38.0</t>
+          <t>16.0</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>1.5537</t>
+          <t>1.2712</t>
         </is>
       </c>
       <c r="F17" t="inlineStr"/>
@@ -2078,7 +2094,7 @@
       </c>
       <c r="L17" t="inlineStr">
         <is>
-          <t>0x04fd78e33c10fb928e409323c26948f49fe4c81fcd47748d9153c9c611b38d0b</t>
+          <t>0x06a233f1b733d63cee459a37ac1beffad92b8f9ec21c414e0c26e2876b05eebd</t>
         </is>
       </c>
       <c r="M17" t="inlineStr">
@@ -2108,7 +2124,7 @@
       </c>
       <c r="R17" t="inlineStr">
         <is>
-          <t>1784984536</t>
+          <t>1784984581</t>
         </is>
       </c>
       <c r="S17" t="inlineStr">
@@ -2118,7 +2134,7 @@
       </c>
       <c r="T17" t="inlineStr">
         <is>
-          <t>68.833427</t>
+          <t>60.198968</t>
         </is>
       </c>
       <c r="U17" t="inlineStr">
@@ -2131,12 +2147,12 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>0xa4b5b4c3c3766e7d708b5373412745aa0b0d5f4c097f5451a2210d6d019269c6</t>
+          <t>0x7dd8d48e4f9e00707e79d58d5900292571189d9de19bd23c6c6a9a433ea96f72</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>0x47D0CE9b8d653c8884DB7E2a7F88d4849E0CD980</t>
+          <t>0x4a09916b1325Eed50eE8973B13742a205B0B7c7E</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
@@ -2146,12 +2162,12 @@
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>29.0</t>
+          <t>16.0</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>1.5537</t>
+          <t>1.2712</t>
         </is>
       </c>
       <c r="F18" t="inlineStr"/>
@@ -2178,7 +2194,7 @@
       </c>
       <c r="L18" t="inlineStr">
         <is>
-          <t>0x04fd78e33c10fb928e409323c26948f49fe4c81fcd47748d9153c9c611b38d0b</t>
+          <t>0x06a233f1b733d63cee459a37ac1beffad92b8f9ec21c414e0c26e2876b05eebd</t>
         </is>
       </c>
       <c r="M18" t="inlineStr">
@@ -2208,7 +2224,7 @@
       </c>
       <c r="R18" t="inlineStr">
         <is>
-          <t>1784984502</t>
+          <t>1784984563</t>
         </is>
       </c>
       <c r="S18" t="inlineStr">
@@ -2218,7 +2234,7 @@
       </c>
       <c r="T18" t="inlineStr">
         <is>
-          <t>53.355738</t>
+          <t>60.198968</t>
         </is>
       </c>
       <c r="U18" t="inlineStr">
@@ -2231,12 +2247,12 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>0xfac3960037b540d1b0b49f14ff5313d7db5bd6320c356e510ef3e6bdaca6d1ff</t>
+          <t>0x7354c940dd56ae7caca9fa9b1a548dcf53e1a3516f531216c677cf582affb4fe</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>0x47D0CE9b8d653c8884DB7E2a7F88d4849E0CD980</t>
+          <t>0x4a09916b1325Eed50eE8973B13742a205B0B7c7E</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
@@ -2246,12 +2262,12 @@
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>25.0</t>
+          <t>9.0</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>1.5537</t>
+          <t>1.3013</t>
         </is>
       </c>
       <c r="F19" t="inlineStr"/>
@@ -2278,7 +2294,7 @@
       </c>
       <c r="L19" t="inlineStr">
         <is>
-          <t>0x04fd78e33c10fb928e409323c26948f49fe4c81fcd47748d9153c9c611b38d0b</t>
+          <t>0x06a233f1b733d63cee459a37ac1beffad92b8f9ec21c414e0c26e2876b05eebd</t>
         </is>
       </c>
       <c r="M19" t="inlineStr">
@@ -2308,7 +2324,7 @@
       </c>
       <c r="R19" t="inlineStr">
         <is>
-          <t>1784984501</t>
+          <t>1784984538</t>
         </is>
       </c>
       <c r="S19" t="inlineStr">
@@ -2318,7 +2334,7 @@
       </c>
       <c r="T19" t="inlineStr">
         <is>
-          <t>46.408957</t>
+          <t>31.184232</t>
         </is>
       </c>
       <c r="U19" t="inlineStr">
@@ -2331,12 +2347,12 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>0xf3b65016998beda20548812c7503abc20be0fa3abedc59c3ac7e08e6b82c70f1</t>
+          <t>0xdc3c1508859b265a9cc7ea3dadc58bb672f939bf46cde2c06081ec2891a03946</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>0x4a09916b1325Eed50eE8973B13742a205B0B7c7E</t>
+          <t>0xC88F614A48f8A705d7465b03aAF62ddaca0c3754</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
@@ -2346,12 +2362,12 @@
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>6.0</t>
+          <t>21.0</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>1.3013</t>
+          <t>1.4363</t>
         </is>
       </c>
       <c r="F20" t="inlineStr"/>
@@ -2378,7 +2394,7 @@
       </c>
       <c r="L20" t="inlineStr">
         <is>
-          <t>0x06a233f1b733d63cee459a37ac1beffad92b8f9ec21c414e0c26e2876b05eebd</t>
+          <t>0xd5ae8f2322bcc6adaca1c1bb1baf6a74afa50cc30131840c87632f67865c23d0</t>
         </is>
       </c>
       <c r="M20" t="inlineStr">
@@ -2408,7 +2424,7 @@
       </c>
       <c r="R20" t="inlineStr">
         <is>
-          <t>1784984431</t>
+          <t>1784984537</t>
         </is>
       </c>
       <c r="S20" t="inlineStr">
@@ -2418,7 +2434,7 @@
       </c>
       <c r="T20" t="inlineStr">
         <is>
-          <t>22.912332</t>
+          <t>48.297994</t>
         </is>
       </c>
       <c r="U20" t="inlineStr">
@@ -2431,12 +2447,12 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>0xa04fcfb1b689fd17d1c3c66ac2ed73a6e0b99d30bdfd296529ca6549b4642440</t>
+          <t>0x0bf6c8f6ea5d7452bf543eb72d99a66c1b6ff74a5e56b4ad9449b6870f225d2d</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>0x4a09916b1325Eed50eE8973B13742a205B0B7c7E</t>
+          <t>0x47D0CE9b8d653c8884DB7E2a7F88d4849E0CD980</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
@@ -2446,12 +2462,12 @@
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>27.0</t>
+          <t>38.0</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>1.4537</t>
+          <t>1.5537</t>
         </is>
       </c>
       <c r="F21" t="inlineStr"/>
@@ -2478,7 +2494,7 @@
       </c>
       <c r="L21" t="inlineStr">
         <is>
-          <t>0xd5ae8f2322bcc6adaca1c1bb1baf6a74afa50cc30131840c87632f67865c23d0</t>
+          <t>0x04fd78e33c10fb928e409323c26948f49fe4c81fcd47748d9153c9c611b38d0b</t>
         </is>
       </c>
       <c r="M21" t="inlineStr">
@@ -2508,7 +2524,7 @@
       </c>
       <c r="R21" t="inlineStr">
         <is>
-          <t>1784984405</t>
+          <t>1784984536</t>
         </is>
       </c>
       <c r="S21" t="inlineStr">
@@ -2518,7 +2534,7 @@
       </c>
       <c r="T21" t="inlineStr">
         <is>
-          <t>60.187328</t>
+          <t>68.833427</t>
         </is>
       </c>
       <c r="U21" t="inlineStr">
@@ -2531,12 +2547,12 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>0xb07983b62c387b953f021bde51a561f510162701d56466ec78a20a598c01d8c4</t>
+          <t>0xa4b5b4c3c3766e7d708b5373412745aa0b0d5f4c097f5451a2210d6d019269c6</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>0x4a09916b1325Eed50eE8973B13742a205B0B7c7E</t>
+          <t>0x47D0CE9b8d653c8884DB7E2a7F88d4849E0CD980</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
@@ -2546,12 +2562,12 @@
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>35.0</t>
+          <t>29.0</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>1.595</t>
+          <t>1.5537</t>
         </is>
       </c>
       <c r="F22" t="inlineStr"/>
@@ -2578,7 +2594,7 @@
       </c>
       <c r="L22" t="inlineStr">
         <is>
-          <t>0xe1204c11efd43d8d3a0377591c468bba3ac169f58ab541c6d60665f2e0bbb051</t>
+          <t>0x04fd78e33c10fb928e409323c26948f49fe4c81fcd47748d9153c9c611b38d0b</t>
         </is>
       </c>
       <c r="M22" t="inlineStr">
@@ -2608,7 +2624,7 @@
       </c>
       <c r="R22" t="inlineStr">
         <is>
-          <t>1784984404</t>
+          <t>1784984502</t>
         </is>
       </c>
       <c r="S22" t="inlineStr">
@@ -2618,7 +2634,7 @@
       </c>
       <c r="T22" t="inlineStr">
         <is>
-          <t>60.197529</t>
+          <t>53.355738</t>
         </is>
       </c>
       <c r="U22" t="inlineStr">
@@ -2631,27 +2647,27 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>0xc41db21ce0b5921299bba16424467dff9a9a6eb4d744a5aadf04422f8138f34f</t>
+          <t>0xfac3960037b540d1b0b49f14ff5313d7db5bd6320c356e510ef3e6bdaca6d1ff</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>0x68E1818FF20BBe84F9be9E0A4A395FB11079Bd35</t>
+          <t>0x47D0CE9b8d653c8884DB7E2a7F88d4849E0CD980</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>1</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>22.0</t>
+          <t>25.0</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>1.7712</t>
+          <t>1.5537</t>
         </is>
       </c>
       <c r="F23" t="inlineStr"/>
@@ -2678,7 +2694,7 @@
       </c>
       <c r="L23" t="inlineStr">
         <is>
-          <t>0x91a9ea8ebfd8b049218a8e072590d2f657e26fdb1f2a49b1016ae42171c68ef2</t>
+          <t>0x04fd78e33c10fb928e409323c26948f49fe4c81fcd47748d9153c9c611b38d0b</t>
         </is>
       </c>
       <c r="M23" t="inlineStr">
@@ -2708,7 +2724,7 @@
       </c>
       <c r="R23" t="inlineStr">
         <is>
-          <t>1784984403</t>
+          <t>1784984501</t>
         </is>
       </c>
       <c r="S23" t="inlineStr">
@@ -2718,7 +2734,7 @@
       </c>
       <c r="T23" t="inlineStr">
         <is>
-          <t>29.185737</t>
+          <t>46.408957</t>
         </is>
       </c>
       <c r="U23" t="inlineStr">
@@ -2731,27 +2747,27 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>0x97d57842a441d56ad4d0172a6e2460bdd3644bd55476d419863d144ec4fb3f02</t>
+          <t>0xf3b65016998beda20548812c7503abc20be0fa3abedc59c3ac7e08e6b82c70f1</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>0x68E1818FF20BBe84F9be9E0A4A395FB11079Bd35</t>
+          <t>0x4a09916b1325Eed50eE8973B13742a205B0B7c7E</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>1</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>3.0</t>
+          <t>6.0</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>1.775</t>
+          <t>1.3013</t>
         </is>
       </c>
       <c r="F24" t="inlineStr"/>
@@ -2778,7 +2794,7 @@
       </c>
       <c r="L24" t="inlineStr">
         <is>
-          <t>0x2b00f05607bf61216841f59440e877cc0eeb424e834132492c721bd4faedc556</t>
+          <t>0x06a233f1b733d63cee459a37ac1beffad92b8f9ec21c414e0c26e2876b05eebd</t>
         </is>
       </c>
       <c r="M24" t="inlineStr">
@@ -2808,7 +2824,7 @@
       </c>
       <c r="R24" t="inlineStr">
         <is>
-          <t>1784984403</t>
+          <t>1784984431</t>
         </is>
       </c>
       <c r="S24" t="inlineStr">
@@ -2818,7 +2834,7 @@
       </c>
       <c r="T24" t="inlineStr">
         <is>
-          <t>4.444439</t>
+          <t>22.912332</t>
         </is>
       </c>
       <c r="U24" t="inlineStr">
@@ -2831,7 +2847,7 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>0x54a44d2ce4be4b546daee52057d4611c0f1d29571a9747f66b3462780e888ae0</t>
+          <t>0xa04fcfb1b689fd17d1c3c66ac2ed73a6e0b99d30bdfd296529ca6549b4642440</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
@@ -2846,12 +2862,12 @@
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>17.0</t>
+          <t>27.0</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>1.2988</t>
+          <t>1.4537</t>
         </is>
       </c>
       <c r="F25" t="inlineStr"/>
@@ -2878,7 +2894,7 @@
       </c>
       <c r="L25" t="inlineStr">
         <is>
-          <t>0x588a71865f90131e16b5b72dfef6ddb7cec8deb7df1f8102477a62eaa807cc71</t>
+          <t>0xd5ae8f2322bcc6adaca1c1bb1baf6a74afa50cc30131840c87632f67865c23d0</t>
         </is>
       </c>
       <c r="M25" t="inlineStr">
@@ -2908,7 +2924,7 @@
       </c>
       <c r="R25" t="inlineStr">
         <is>
-          <t>1784984402</t>
+          <t>1784984405</t>
         </is>
       </c>
       <c r="S25" t="inlineStr">
@@ -2918,7 +2934,7 @@
       </c>
       <c r="T25" t="inlineStr">
         <is>
-          <t>60.178243</t>
+          <t>60.187328</t>
         </is>
       </c>
       <c r="U25" t="inlineStr">
@@ -2931,7 +2947,7 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>0xf9d293335e6b1b3fd21eba9ec71cbbd6cbce398d5d606b38175d3776a077cb91</t>
+          <t>0xb07983b62c387b953f021bde51a561f510162701d56466ec78a20a598c01d8c4</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
@@ -2946,12 +2962,12 @@
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>41.0</t>
+          <t>35.0</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>1.685</t>
+          <t>1.595</t>
         </is>
       </c>
       <c r="F26" t="inlineStr"/>
@@ -2978,7 +2994,7 @@
       </c>
       <c r="L26" t="inlineStr">
         <is>
-          <t>0xaf0827308b557ecc964e4c608c6b71f345660fa965da2a0e02882ee62ce45e49</t>
+          <t>0xe1204c11efd43d8d3a0377591c468bba3ac169f58ab541c6d60665f2e0bbb051</t>
         </is>
       </c>
       <c r="M26" t="inlineStr">
@@ -3008,7 +3024,7 @@
       </c>
       <c r="R26" t="inlineStr">
         <is>
-          <t>1784984401</t>
+          <t>1784984404</t>
         </is>
       </c>
       <c r="S26" t="inlineStr">
@@ -3018,7 +3034,7 @@
       </c>
       <c r="T26" t="inlineStr">
         <is>
-          <t>60.189781</t>
+          <t>60.197529</t>
         </is>
       </c>
       <c r="U26" t="inlineStr">
@@ -3031,27 +3047,27 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>0x80f610f55e907d511b2c5a8d77d03f9aca143e4e50b6d7fba92997ba46481bde</t>
+          <t>0xc41db21ce0b5921299bba16424467dff9a9a6eb4d744a5aadf04422f8138f34f</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>0x47D0CE9b8d653c8884DB7E2a7F88d4849E0CD980</t>
+          <t>0x68E1818FF20BBe84F9be9E0A4A395FB11079Bd35</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>6.0</t>
+          <t>22.0</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>1.5537</t>
+          <t>1.7712</t>
         </is>
       </c>
       <c r="F27" t="inlineStr"/>
@@ -3078,7 +3094,7 @@
       </c>
       <c r="L27" t="inlineStr">
         <is>
-          <t>0x04fd78e33c10fb928e409323c26948f49fe4c81fcd47748d9153c9c611b38d0b</t>
+          <t>0x91a9ea8ebfd8b049218a8e072590d2f657e26fdb1f2a49b1016ae42171c68ef2</t>
         </is>
       </c>
       <c r="M27" t="inlineStr">
@@ -3108,7 +3124,7 @@
       </c>
       <c r="R27" t="inlineStr">
         <is>
-          <t>1784983849</t>
+          <t>1784984403</t>
         </is>
       </c>
       <c r="S27" t="inlineStr">
@@ -3118,7 +3134,7 @@
       </c>
       <c r="T27" t="inlineStr">
         <is>
-          <t>11.988786</t>
+          <t>29.185737</t>
         </is>
       </c>
       <c r="U27" t="inlineStr">
@@ -3131,7 +3147,7 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>0x6e3d6f822ebfe70f563004b4a5a4a6303f1d1cb9677e6e3a56324cda8cc92ba7</t>
+          <t>0x97d57842a441d56ad4d0172a6e2460bdd3644bd55476d419863d144ec4fb3f02</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
@@ -3141,17 +3157,17 @@
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>25.0</t>
+          <t>3.0</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>1.5513</t>
+          <t>1.775</t>
         </is>
       </c>
       <c r="F28" t="inlineStr"/>
@@ -3178,7 +3194,7 @@
       </c>
       <c r="L28" t="inlineStr">
         <is>
-          <t>0x04fd78e33c10fb928e409323c26948f49fe4c81fcd47748d9153c9c611b38d0b</t>
+          <t>0x2b00f05607bf61216841f59440e877cc0eeb424e834132492c721bd4faedc556</t>
         </is>
       </c>
       <c r="M28" t="inlineStr">
@@ -3208,7 +3224,7 @@
       </c>
       <c r="R28" t="inlineStr">
         <is>
-          <t>1784983797</t>
+          <t>1784984403</t>
         </is>
       </c>
       <c r="S28" t="inlineStr">
@@ -3218,7 +3234,7 @@
       </c>
       <c r="T28" t="inlineStr">
         <is>
-          <t>46.150404</t>
+          <t>4.444439</t>
         </is>
       </c>
       <c r="U28" t="inlineStr">
@@ -3231,27 +3247,27 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>0xc913b7104d801ceb0283dc9eefcce577969c93f7b16c1cc5515036561b5b8d8e</t>
+          <t>0x54a44d2ce4be4b546daee52057d4611c0f1d29571a9747f66b3462780e888ae0</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>0x68E1818FF20BBe84F9be9E0A4A395FB11079Bd35</t>
+          <t>0x4a09916b1325Eed50eE8973B13742a205B0B7c7E</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>1</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>4.0</t>
+          <t>17.0</t>
         </is>
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>1.7712</t>
+          <t>1.2988</t>
         </is>
       </c>
       <c r="F29" t="inlineStr"/>
@@ -3278,7 +3294,7 @@
       </c>
       <c r="L29" t="inlineStr">
         <is>
-          <t>0x91a9ea8ebfd8b049218a8e072590d2f657e26fdb1f2a49b1016ae42171c68ef2</t>
+          <t>0x588a71865f90131e16b5b72dfef6ddb7cec8deb7df1f8102477a62eaa807cc71</t>
         </is>
       </c>
       <c r="M29" t="inlineStr">
@@ -3308,7 +3324,7 @@
       </c>
       <c r="R29" t="inlineStr">
         <is>
-          <t>1784983703</t>
+          <t>1784984402</t>
         </is>
       </c>
       <c r="S29" t="inlineStr">
@@ -3318,7 +3334,7 @@
       </c>
       <c r="T29" t="inlineStr">
         <is>
-          <t>5.770489</t>
+          <t>60.178243</t>
         </is>
       </c>
       <c r="U29" t="inlineStr">
@@ -3331,12 +3347,12 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>0x78c593e23cd10a2517f77039f922e2d360ba0b6d4c89dc91bac22f6854ce01ea</t>
+          <t>0xf9d293335e6b1b3fd21eba9ec71cbbd6cbce398d5d606b38175d3776a077cb91</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>0x68E1818FF20BBe84F9be9E0A4A395FB11079Bd35</t>
+          <t>0x4a09916b1325Eed50eE8973B13742a205B0B7c7E</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
@@ -3346,12 +3362,12 @@
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>2.0</t>
+          <t>41.0</t>
         </is>
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>1.5513</t>
+          <t>1.685</t>
         </is>
       </c>
       <c r="F30" t="inlineStr"/>
@@ -3378,7 +3394,7 @@
       </c>
       <c r="L30" t="inlineStr">
         <is>
-          <t>0x04fd78e33c10fb928e409323c26948f49fe4c81fcd47748d9153c9c611b38d0b</t>
+          <t>0xaf0827308b557ecc964e4c608c6b71f345660fa965da2a0e02882ee62ce45e49</t>
         </is>
       </c>
       <c r="M30" t="inlineStr">
@@ -3408,7 +3424,7 @@
       </c>
       <c r="R30" t="inlineStr">
         <is>
-          <t>1784983703</t>
+          <t>1784984401</t>
         </is>
       </c>
       <c r="S30" t="inlineStr">
@@ -3418,7 +3434,7 @@
       </c>
       <c r="T30" t="inlineStr">
         <is>
-          <t>4.389968</t>
+          <t>60.189781</t>
         </is>
       </c>
       <c r="U30" t="inlineStr">
@@ -3431,12 +3447,12 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>0x589562dc55239bfc299045a0e5bbfed420cc8f286ee7326d34ed350f83ecdd45</t>
+          <t>0x80f610f55e907d511b2c5a8d77d03f9aca143e4e50b6d7fba92997ba46481bde</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>0x68E1818FF20BBe84F9be9E0A4A395FB11079Bd35</t>
+          <t>0x47D0CE9b8d653c8884DB7E2a7F88d4849E0CD980</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
@@ -3446,12 +3462,12 @@
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>12.0</t>
+          <t>6.0</t>
         </is>
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>1.5513</t>
+          <t>1.5537</t>
         </is>
       </c>
       <c r="F31" t="inlineStr"/>
@@ -3508,7 +3524,7 @@
       </c>
       <c r="R31" t="inlineStr">
         <is>
-          <t>1784983480</t>
+          <t>1784983849</t>
         </is>
       </c>
       <c r="S31" t="inlineStr">
@@ -3518,7 +3534,7 @@
       </c>
       <c r="T31" t="inlineStr">
         <is>
-          <t>22.284118</t>
+          <t>11.988786</t>
         </is>
       </c>
       <c r="U31" t="inlineStr">
@@ -3531,7 +3547,7 @@
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>0x629a7bab69ed2f6eae5804065863061a8e5f95bfbf35104c3a1d130585e021ca</t>
+          <t>0x6e3d6f822ebfe70f563004b4a5a4a6303f1d1cb9677e6e3a56324cda8cc92ba7</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
@@ -3546,7 +3562,7 @@
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>1.0</t>
+          <t>25.0</t>
         </is>
       </c>
       <c r="E32" t="inlineStr">
@@ -3608,7 +3624,7 @@
       </c>
       <c r="R32" t="inlineStr">
         <is>
-          <t>1784983361</t>
+          <t>1784983797</t>
         </is>
       </c>
       <c r="S32" t="inlineStr">
@@ -3618,7 +3634,7 @@
       </c>
       <c r="T32" t="inlineStr">
         <is>
-          <t>2.228408</t>
+          <t>46.150404</t>
         </is>
       </c>
       <c r="U32" t="inlineStr">
@@ -3631,27 +3647,27 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>0x888b7311174b291a1eeccf40a054d1599070da16bd2f2f7adea95d18002cc686</t>
+          <t>0xc913b7104d801ceb0283dc9eefcce577969c93f7b16c1cc5515036561b5b8d8e</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>0xB1854fc8aD8ce649EA80D007Fc67d318a239a5DA</t>
+          <t>0x68E1818FF20BBe84F9be9E0A4A395FB11079Bd35</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>0.0</t>
+          <t>4.0</t>
         </is>
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>1.215</t>
+          <t>1.7712</t>
         </is>
       </c>
       <c r="F33" t="inlineStr"/>
@@ -3708,7 +3724,7 @@
       </c>
       <c r="R33" t="inlineStr">
         <is>
-          <t>1784981088</t>
+          <t>1784983703</t>
         </is>
       </c>
       <c r="S33" t="inlineStr">
@@ -3718,7 +3734,7 @@
       </c>
       <c r="T33" t="inlineStr">
         <is>
-          <t>1.443442</t>
+          <t>5.770489</t>
         </is>
       </c>
       <c r="U33" t="inlineStr">
@@ -3731,7 +3747,7 @@
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>0x5d44678e836886d72dc3bddfca4b44d2be2bfa7f56096dbedd259cac92e30df3</t>
+          <t>0x78c593e23cd10a2517f77039f922e2d360ba0b6d4c89dc91bac22f6854ce01ea</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
@@ -3741,17 +3757,17 @@
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>1</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>16.0</t>
+          <t>2.0</t>
         </is>
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t>1.7712</t>
+          <t>1.5513</t>
         </is>
       </c>
       <c r="F34" t="inlineStr"/>
@@ -3778,7 +3794,7 @@
       </c>
       <c r="L34" t="inlineStr">
         <is>
-          <t>0x91a9ea8ebfd8b049218a8e072590d2f657e26fdb1f2a49b1016ae42171c68ef2</t>
+          <t>0x04fd78e33c10fb928e409323c26948f49fe4c81fcd47748d9153c9c611b38d0b</t>
         </is>
       </c>
       <c r="M34" t="inlineStr">
@@ -3808,7 +3824,7 @@
       </c>
       <c r="R34" t="inlineStr">
         <is>
-          <t>1784981082</t>
+          <t>1784983703</t>
         </is>
       </c>
       <c r="S34" t="inlineStr">
@@ -3818,7 +3834,7 @@
       </c>
       <c r="T34" t="inlineStr">
         <is>
-          <t>21.377037</t>
+          <t>4.389968</t>
         </is>
       </c>
       <c r="U34" t="inlineStr">
@@ -3831,7 +3847,7 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>0x5a96bb0ca1d506186a0e2c1c2e13d657784bbb03ad3f75e66db86da80f485bae</t>
+          <t>0x589562dc55239bfc299045a0e5bbfed420cc8f286ee7326d34ed350f83ecdd45</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
@@ -3846,7 +3862,7 @@
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>19.0</t>
+          <t>12.0</t>
         </is>
       </c>
       <c r="E35" t="inlineStr">
@@ -3908,7 +3924,7 @@
       </c>
       <c r="R35" t="inlineStr">
         <is>
-          <t>1784980847</t>
+          <t>1784983480</t>
         </is>
       </c>
       <c r="S35" t="inlineStr">
@@ -3918,7 +3934,7 @@
       </c>
       <c r="T35" t="inlineStr">
         <is>
-          <t>35.743728</t>
+          <t>22.284118</t>
         </is>
       </c>
       <c r="U35" t="inlineStr">
@@ -3931,12 +3947,12 @@
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>0xe6e61e0b4573e8e2199880691f7803f1943269d2b2b955ea7282a833c4dbc3c6</t>
+          <t>0x629a7bab69ed2f6eae5804065863061a8e5f95bfbf35104c3a1d130585e021ca</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>0x47D0CE9b8d653c8884DB7E2a7F88d4849E0CD980</t>
+          <t>0x68E1818FF20BBe84F9be9E0A4A395FB11079Bd35</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
@@ -3946,12 +3962,12 @@
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>22.0</t>
+          <t>1.0</t>
         </is>
       </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t>1.555</t>
+          <t>1.5513</t>
         </is>
       </c>
       <c r="F36" t="inlineStr"/>
@@ -4008,7 +4024,7 @@
       </c>
       <c r="R36" t="inlineStr">
         <is>
-          <t>1784977858</t>
+          <t>1784983361</t>
         </is>
       </c>
       <c r="S36" t="inlineStr">
@@ -4018,7 +4034,7 @@
       </c>
       <c r="T36" t="inlineStr">
         <is>
-          <t>39.775279</t>
+          <t>2.228408</t>
         </is>
       </c>
       <c r="U36" t="inlineStr">
@@ -4031,12 +4047,12 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>0x668fc309ba15ebe234fe9dd2d2bf696a9f4000c9ac85f8e7d55c998a052968dc</t>
+          <t>0x888b7311174b291a1eeccf40a054d1599070da16bd2f2f7adea95d18002cc686</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>0x47D0CE9b8d653c8884DB7E2a7F88d4849E0CD980</t>
+          <t>0xB1854fc8aD8ce649EA80D007Fc67d318a239a5DA</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
@@ -4046,12 +4062,12 @@
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>27.0</t>
+          <t>0.0</t>
         </is>
       </c>
       <c r="E37" t="inlineStr">
         <is>
-          <t>1.555</t>
+          <t>1.215</t>
         </is>
       </c>
       <c r="F37" t="inlineStr"/>
@@ -4078,7 +4094,7 @@
       </c>
       <c r="L37" t="inlineStr">
         <is>
-          <t>0x04fd78e33c10fb928e409323c26948f49fe4c81fcd47748d9153c9c611b38d0b</t>
+          <t>0x91a9ea8ebfd8b049218a8e072590d2f657e26fdb1f2a49b1016ae42171c68ef2</t>
         </is>
       </c>
       <c r="M37" t="inlineStr">
@@ -4108,7 +4124,7 @@
       </c>
       <c r="R37" t="inlineStr">
         <is>
-          <t>1784977853</t>
+          <t>1784981088</t>
         </is>
       </c>
       <c r="S37" t="inlineStr">
@@ -4118,7 +4134,7 @@
       </c>
       <c r="T37" t="inlineStr">
         <is>
-          <t>49.797748</t>
+          <t>1.443442</t>
         </is>
       </c>
       <c r="U37" t="inlineStr">
@@ -4131,12 +4147,12 @@
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>0xabcdef492212262464335967adbaa23c5214ede2fab0ea2a12bce6e0027067aa</t>
+          <t>0x5d44678e836886d72dc3bddfca4b44d2be2bfa7f56096dbedd259cac92e30df3</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>0xC88F614A48f8A705d7465b03aAF62ddaca0c3754</t>
+          <t>0x68E1818FF20BBe84F9be9E0A4A395FB11079Bd35</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
@@ -4146,12 +4162,12 @@
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>20.0</t>
+          <t>16.0</t>
         </is>
       </c>
       <c r="E38" t="inlineStr">
         <is>
-          <t>1.435</t>
+          <t>1.7712</t>
         </is>
       </c>
       <c r="F38" t="inlineStr"/>
@@ -4178,7 +4194,7 @@
       </c>
       <c r="L38" t="inlineStr">
         <is>
-          <t>0xef2cff3047642c7d3f79713526decc2ed1438c01d374590eb62929362f824801</t>
+          <t>0x91a9ea8ebfd8b049218a8e072590d2f657e26fdb1f2a49b1016ae42171c68ef2</t>
         </is>
       </c>
       <c r="M38" t="inlineStr">
@@ -4208,7 +4224,7 @@
       </c>
       <c r="R38" t="inlineStr">
         <is>
-          <t>1784968614</t>
+          <t>1784981082</t>
         </is>
       </c>
       <c r="S38" t="inlineStr">
@@ -4218,7 +4234,7 @@
       </c>
       <c r="T38" t="inlineStr">
         <is>
-          <t>47.149425</t>
+          <t>21.377037</t>
         </is>
       </c>
       <c r="U38" t="inlineStr">
@@ -4231,12 +4247,12 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>0xf7e34584abe1fc7da16770ad9dc2fe59e91a45480c1ff509d55070c7d811c7e2</t>
+          <t>0x5a96bb0ca1d506186a0e2c1c2e13d657784bbb03ad3f75e66db86da80f485bae</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>0x516bfc7CE57c0E1734388ECed5Bb9454aA6aeFae</t>
+          <t>0x68E1818FF20BBe84F9be9E0A4A395FB11079Bd35</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
@@ -4246,12 +4262,12 @@
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>10.0</t>
+          <t>19.0</t>
         </is>
       </c>
       <c r="E39" t="inlineStr">
         <is>
-          <t>1.56</t>
+          <t>1.5513</t>
         </is>
       </c>
       <c r="F39" t="inlineStr"/>
@@ -4278,7 +4294,7 @@
       </c>
       <c r="L39" t="inlineStr">
         <is>
-          <t>0xe1204c11efd43d8d3a0377591c468bba3ac169f58ab541c6d60665f2e0bbb051</t>
+          <t>0x04fd78e33c10fb928e409323c26948f49fe4c81fcd47748d9153c9c611b38d0b</t>
         </is>
       </c>
       <c r="M39" t="inlineStr">
@@ -4308,7 +4324,7 @@
       </c>
       <c r="R39" t="inlineStr">
         <is>
-          <t>1784907257</t>
+          <t>1784980847</t>
         </is>
       </c>
       <c r="S39" t="inlineStr">
@@ -4318,7 +4334,7 @@
       </c>
       <c r="T39" t="inlineStr">
         <is>
-          <t>17.857143</t>
+          <t>35.743728</t>
         </is>
       </c>
       <c r="U39" t="inlineStr">
@@ -4331,12 +4347,12 @@
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>0x030841d8eff7e23d98d8319e71f99f9eb17cb2a743343cfac134410b86f1178e</t>
+          <t>0xe6e61e0b4573e8e2199880691f7803f1943269d2b2b955ea7282a833c4dbc3c6</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>0xC88F614A48f8A705d7465b03aAF62ddaca0c3754</t>
+          <t>0x47D0CE9b8d653c8884DB7E2a7F88d4849E0CD980</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
@@ -4346,12 +4362,12 @@
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>26.0</t>
+          <t>22.0</t>
         </is>
       </c>
       <c r="E40" t="inlineStr">
         <is>
-          <t>1.5737</t>
+          <t>1.555</t>
         </is>
       </c>
       <c r="F40" t="inlineStr"/>
@@ -4378,7 +4394,7 @@
       </c>
       <c r="L40" t="inlineStr">
         <is>
-          <t>0xe1204c11efd43d8d3a0377591c468bba3ac169f58ab541c6d60665f2e0bbb051</t>
+          <t>0x04fd78e33c10fb928e409323c26948f49fe4c81fcd47748d9153c9c611b38d0b</t>
         </is>
       </c>
       <c r="M40" t="inlineStr">
@@ -4408,7 +4424,7 @@
       </c>
       <c r="R40" t="inlineStr">
         <is>
-          <t>1784907053</t>
+          <t>1784977858</t>
         </is>
       </c>
       <c r="S40" t="inlineStr">
@@ -4418,7 +4434,7 @@
       </c>
       <c r="T40" t="inlineStr">
         <is>
-          <t>46.28739</t>
+          <t>39.775279</t>
         </is>
       </c>
       <c r="U40" t="inlineStr">
@@ -4431,12 +4447,12 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>0xd486facb98ea7c7e7b67efb74b5231332788279dbd71dce40eea54aecf5d870e</t>
+          <t>0x668fc309ba15ebe234fe9dd2d2bf696a9f4000c9ac85f8e7d55c998a052968dc</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>0xC88F614A48f8A705d7465b03aAF62ddaca0c3754</t>
+          <t>0x47D0CE9b8d653c8884DB7E2a7F88d4849E0CD980</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
@@ -4446,12 +4462,12 @@
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t>14.0</t>
+          <t>27.0</t>
         </is>
       </c>
       <c r="E41" t="inlineStr">
         <is>
-          <t>1.315</t>
+          <t>1.555</t>
         </is>
       </c>
       <c r="F41" t="inlineStr"/>
@@ -4478,7 +4494,7 @@
       </c>
       <c r="L41" t="inlineStr">
         <is>
-          <t>0x588a71865f90131e16b5b72dfef6ddb7cec8deb7df1f8102477a62eaa807cc71</t>
+          <t>0x04fd78e33c10fb928e409323c26948f49fe4c81fcd47748d9153c9c611b38d0b</t>
         </is>
       </c>
       <c r="M41" t="inlineStr">
@@ -4508,7 +4524,7 @@
       </c>
       <c r="R41" t="inlineStr">
         <is>
-          <t>1784907041</t>
+          <t>1784977853</t>
         </is>
       </c>
       <c r="S41" t="inlineStr">
@@ -4518,7 +4534,7 @@
       </c>
       <c r="T41" t="inlineStr">
         <is>
-          <t>47.587302</t>
+          <t>49.797748</t>
         </is>
       </c>
       <c r="U41" t="inlineStr">
@@ -4531,7 +4547,7 @@
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>0x8a9596cb004924470885fe466db8f8d059fcb9d1b24e71490dd35bfeba65a98d</t>
+          <t>0xabcdef492212262464335967adbaa23c5214ede2fab0ea2a12bce6e0027067aa</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
@@ -4541,17 +4557,17 @@
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t>14.0</t>
+          <t>20.0</t>
         </is>
       </c>
       <c r="E42" t="inlineStr">
         <is>
-          <t>1.315</t>
+          <t>1.435</t>
         </is>
       </c>
       <c r="F42" t="inlineStr"/>
@@ -4578,7 +4594,7 @@
       </c>
       <c r="L42" t="inlineStr">
         <is>
-          <t>0x06a233f1b733d63cee459a37ac1beffad92b8f9ec21c414e0c26e2876b05eebd</t>
+          <t>0xef2cff3047642c7d3f79713526decc2ed1438c01d374590eb62929362f824801</t>
         </is>
       </c>
       <c r="M42" t="inlineStr">
@@ -4608,7 +4624,7 @@
       </c>
       <c r="R42" t="inlineStr">
         <is>
-          <t>1784907041</t>
+          <t>1784968614</t>
         </is>
       </c>
       <c r="S42" t="inlineStr">
@@ -4618,7 +4634,7 @@
       </c>
       <c r="T42" t="inlineStr">
         <is>
-          <t>47.555556</t>
+          <t>47.149425</t>
         </is>
       </c>
       <c r="U42" t="inlineStr">
@@ -4631,12 +4647,12 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>0xdaf8fe8a287cecb340987a0eebd287e9d8e007af24d015fcadd720fceba485cd</t>
+          <t>0xf7e34584abe1fc7da16770ad9dc2fe59e91a45480c1ff509d55070c7d811c7e2</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>0xC88F614A48f8A705d7465b03aAF62ddaca0c3754</t>
+          <t>0x516bfc7CE57c0E1734388ECed5Bb9454aA6aeFae</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
@@ -4646,12 +4662,12 @@
       </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t>26.0</t>
+          <t>10.0</t>
         </is>
       </c>
       <c r="E43" t="inlineStr">
         <is>
-          <t>1.57</t>
+          <t>1.56</t>
         </is>
       </c>
       <c r="F43" t="inlineStr"/>
@@ -4708,7 +4724,7 @@
       </c>
       <c r="R43" t="inlineStr">
         <is>
-          <t>1784907040</t>
+          <t>1784907257</t>
         </is>
       </c>
       <c r="S43" t="inlineStr">
@@ -4718,7 +4734,7 @@
       </c>
       <c r="T43" t="inlineStr">
         <is>
-          <t>47.046509</t>
+          <t>17.857143</t>
         </is>
       </c>
       <c r="U43" t="inlineStr">
@@ -4731,7 +4747,7 @@
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>0x3f981c0415a637d3cb9137ae5b4b0b4b0c50f1a3af5d4e42f65e682f80daadba</t>
+          <t>0x030841d8eff7e23d98d8319e71f99f9eb17cb2a743343cfac134410b86f1178e</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
@@ -4746,12 +4762,12 @@
       </c>
       <c r="D44" t="inlineStr">
         <is>
-          <t>22.0</t>
+          <t>26.0</t>
         </is>
       </c>
       <c r="E44" t="inlineStr">
         <is>
-          <t>1.4625</t>
+          <t>1.5737</t>
         </is>
       </c>
       <c r="F44" t="inlineStr"/>
@@ -4778,55 +4794,455 @@
       </c>
       <c r="L44" t="inlineStr">
         <is>
+          <t>0xe1204c11efd43d8d3a0377591c468bba3ac169f58ab541c6d60665f2e0bbb051</t>
+        </is>
+      </c>
+      <c r="M44" t="inlineStr">
+        <is>
+          <t>L19520873</t>
+        </is>
+      </c>
+      <c r="N44" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="O44" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="P44" t="inlineStr">
+        <is>
+          <t>SUCCESS</t>
+        </is>
+      </c>
+      <c r="Q44" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="R44" t="inlineStr">
+        <is>
+          <t>1784907053</t>
+        </is>
+      </c>
+      <c r="S44" t="inlineStr">
+        <is>
+          <t>1784988000</t>
+        </is>
+      </c>
+      <c r="T44" t="inlineStr">
+        <is>
+          <t>46.28739</t>
+        </is>
+      </c>
+      <c r="U44" t="inlineStr">
+        <is>
+          <t>SXR</t>
+        </is>
+      </c>
+      <c r="V44" t="inlineStr"/>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>0xd486facb98ea7c7e7b67efb74b5231332788279dbd71dce40eea54aecf5d870e</t>
+        </is>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>0xC88F614A48f8A705d7465b03aAF62ddaca0c3754</t>
+        </is>
+      </c>
+      <c r="C45" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="D45" t="inlineStr">
+        <is>
+          <t>14.0</t>
+        </is>
+      </c>
+      <c r="E45" t="inlineStr">
+        <is>
+          <t>1.315</t>
+        </is>
+      </c>
+      <c r="F45" t="inlineStr"/>
+      <c r="G45" t="inlineStr"/>
+      <c r="H45" t="inlineStr">
+        <is>
+          <t>Besta Deild Karla</t>
+        </is>
+      </c>
+      <c r="I45" t="inlineStr">
+        <is>
+          <t>IR Reykjavik vs Fylkir</t>
+        </is>
+      </c>
+      <c r="J45" t="inlineStr">
+        <is>
+          <t>IR Reykjavik</t>
+        </is>
+      </c>
+      <c r="K45" t="inlineStr">
+        <is>
+          <t>Fylkir</t>
+        </is>
+      </c>
+      <c r="L45" t="inlineStr">
+        <is>
+          <t>0x588a71865f90131e16b5b72dfef6ddb7cec8deb7df1f8102477a62eaa807cc71</t>
+        </is>
+      </c>
+      <c r="M45" t="inlineStr">
+        <is>
+          <t>L19520873</t>
+        </is>
+      </c>
+      <c r="N45" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="O45" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="P45" t="inlineStr">
+        <is>
+          <t>SUCCESS</t>
+        </is>
+      </c>
+      <c r="Q45" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="R45" t="inlineStr">
+        <is>
+          <t>1784907041</t>
+        </is>
+      </c>
+      <c r="S45" t="inlineStr">
+        <is>
+          <t>1784988000</t>
+        </is>
+      </c>
+      <c r="T45" t="inlineStr">
+        <is>
+          <t>47.587302</t>
+        </is>
+      </c>
+      <c r="U45" t="inlineStr">
+        <is>
+          <t>SXR</t>
+        </is>
+      </c>
+      <c r="V45" t="inlineStr"/>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>0x8a9596cb004924470885fe466db8f8d059fcb9d1b24e71490dd35bfeba65a98d</t>
+        </is>
+      </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>0xC88F614A48f8A705d7465b03aAF62ddaca0c3754</t>
+        </is>
+      </c>
+      <c r="C46" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="D46" t="inlineStr">
+        <is>
+          <t>14.0</t>
+        </is>
+      </c>
+      <c r="E46" t="inlineStr">
+        <is>
+          <t>1.315</t>
+        </is>
+      </c>
+      <c r="F46" t="inlineStr"/>
+      <c r="G46" t="inlineStr"/>
+      <c r="H46" t="inlineStr">
+        <is>
+          <t>Besta Deild Karla</t>
+        </is>
+      </c>
+      <c r="I46" t="inlineStr">
+        <is>
+          <t>IR Reykjavik vs Fylkir</t>
+        </is>
+      </c>
+      <c r="J46" t="inlineStr">
+        <is>
+          <t>IR Reykjavik</t>
+        </is>
+      </c>
+      <c r="K46" t="inlineStr">
+        <is>
+          <t>Fylkir</t>
+        </is>
+      </c>
+      <c r="L46" t="inlineStr">
+        <is>
+          <t>0x06a233f1b733d63cee459a37ac1beffad92b8f9ec21c414e0c26e2876b05eebd</t>
+        </is>
+      </c>
+      <c r="M46" t="inlineStr">
+        <is>
+          <t>L19520873</t>
+        </is>
+      </c>
+      <c r="N46" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="O46" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="P46" t="inlineStr">
+        <is>
+          <t>SUCCESS</t>
+        </is>
+      </c>
+      <c r="Q46" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="R46" t="inlineStr">
+        <is>
+          <t>1784907041</t>
+        </is>
+      </c>
+      <c r="S46" t="inlineStr">
+        <is>
+          <t>1784988000</t>
+        </is>
+      </c>
+      <c r="T46" t="inlineStr">
+        <is>
+          <t>47.555556</t>
+        </is>
+      </c>
+      <c r="U46" t="inlineStr">
+        <is>
+          <t>SXR</t>
+        </is>
+      </c>
+      <c r="V46" t="inlineStr"/>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>0xdaf8fe8a287cecb340987a0eebd287e9d8e007af24d015fcadd720fceba485cd</t>
+        </is>
+      </c>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>0xC88F614A48f8A705d7465b03aAF62ddaca0c3754</t>
+        </is>
+      </c>
+      <c r="C47" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="D47" t="inlineStr">
+        <is>
+          <t>26.0</t>
+        </is>
+      </c>
+      <c r="E47" t="inlineStr">
+        <is>
+          <t>1.57</t>
+        </is>
+      </c>
+      <c r="F47" t="inlineStr"/>
+      <c r="G47" t="inlineStr"/>
+      <c r="H47" t="inlineStr">
+        <is>
+          <t>Besta Deild Karla</t>
+        </is>
+      </c>
+      <c r="I47" t="inlineStr">
+        <is>
+          <t>IR Reykjavik vs Fylkir</t>
+        </is>
+      </c>
+      <c r="J47" t="inlineStr">
+        <is>
+          <t>IR Reykjavik</t>
+        </is>
+      </c>
+      <c r="K47" t="inlineStr">
+        <is>
+          <t>Fylkir</t>
+        </is>
+      </c>
+      <c r="L47" t="inlineStr">
+        <is>
+          <t>0xe1204c11efd43d8d3a0377591c468bba3ac169f58ab541c6d60665f2e0bbb051</t>
+        </is>
+      </c>
+      <c r="M47" t="inlineStr">
+        <is>
+          <t>L19520873</t>
+        </is>
+      </c>
+      <c r="N47" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="O47" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="P47" t="inlineStr">
+        <is>
+          <t>SUCCESS</t>
+        </is>
+      </c>
+      <c r="Q47" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="R47" t="inlineStr">
+        <is>
+          <t>1784907040</t>
+        </is>
+      </c>
+      <c r="S47" t="inlineStr">
+        <is>
+          <t>1784988000</t>
+        </is>
+      </c>
+      <c r="T47" t="inlineStr">
+        <is>
+          <t>47.046509</t>
+        </is>
+      </c>
+      <c r="U47" t="inlineStr">
+        <is>
+          <t>SXR</t>
+        </is>
+      </c>
+      <c r="V47" t="inlineStr"/>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>0x3f981c0415a637d3cb9137ae5b4b0b4b0c50f1a3af5d4e42f65e682f80daadba</t>
+        </is>
+      </c>
+      <c r="B48" t="inlineStr">
+        <is>
+          <t>0xC88F614A48f8A705d7465b03aAF62ddaca0c3754</t>
+        </is>
+      </c>
+      <c r="C48" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="D48" t="inlineStr">
+        <is>
+          <t>22.0</t>
+        </is>
+      </c>
+      <c r="E48" t="inlineStr">
+        <is>
+          <t>1.4625</t>
+        </is>
+      </c>
+      <c r="F48" t="inlineStr"/>
+      <c r="G48" t="inlineStr"/>
+      <c r="H48" t="inlineStr">
+        <is>
+          <t>Besta Deild Karla</t>
+        </is>
+      </c>
+      <c r="I48" t="inlineStr">
+        <is>
+          <t>IR Reykjavik vs Fylkir</t>
+        </is>
+      </c>
+      <c r="J48" t="inlineStr">
+        <is>
+          <t>IR Reykjavik</t>
+        </is>
+      </c>
+      <c r="K48" t="inlineStr">
+        <is>
+          <t>Fylkir</t>
+        </is>
+      </c>
+      <c r="L48" t="inlineStr">
+        <is>
           <t>0xd5ae8f2322bcc6adaca1c1bb1baf6a74afa50cc30131840c87632f67865c23d0</t>
         </is>
       </c>
-      <c r="M44" t="inlineStr">
+      <c r="M48" t="inlineStr">
         <is>
           <t>L19520873</t>
         </is>
       </c>
-      <c r="N44" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="O44" t="inlineStr">
+      <c r="N48" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="O48" t="inlineStr">
         <is>
           <t>0</t>
         </is>
       </c>
-      <c r="P44" t="inlineStr">
+      <c r="P48" t="inlineStr">
         <is>
           <t>SUCCESS</t>
         </is>
       </c>
-      <c r="Q44" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="R44" t="inlineStr">
+      <c r="Q48" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="R48" t="inlineStr">
         <is>
           <t>1784907040</t>
         </is>
       </c>
-      <c r="S44" t="inlineStr">
+      <c r="S48" t="inlineStr">
         <is>
           <t>1784988000</t>
         </is>
       </c>
-      <c r="T44" t="inlineStr">
+      <c r="T48" t="inlineStr">
         <is>
           <t>47.589189</t>
         </is>
       </c>
-      <c r="U44" t="inlineStr">
+      <c r="U48" t="inlineStr">
         <is>
           <t>SXR</t>
         </is>
       </c>
-      <c r="V44" t="inlineStr"/>
+      <c r="V48" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Update soccer trades 2026-07-29 01:01:13 UTC
</commit_message>
<xml_diff>
--- a/data/sxbet/ligas/Besta Deild Karla/trades.xlsx
+++ b/data/sxbet/ligas/Besta Deild Karla/trades.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:V48"/>
+  <dimension ref="A1:V52"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -531,31 +531,39 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>0x79c1f616b380c93f42fe785c942a2cc39edc55c4cdd4d5b6a09024c926a74f60</t>
+          <t>0xda116ce959332ba41194293702cd84c233a1aa5dc72f06cf3a812e3b16c89f50</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>0x97EC1C9682F70091efB04e97b0B34698cF815EE1</t>
-        </is>
-      </c>
-      <c r="C2" t="inlineStr"/>
+          <t>0x5A76a26f838Ff5430Fd53E61CD8Bd76D895c946E</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>11.22999</t>
+          <t>1.45</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>1.5413</t>
+          <t>1.5088</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>Under/Over (4)</t>
-        </is>
-      </c>
-      <c r="G2" t="inlineStr"/>
+          <t>1X2</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>Throttur Reykjavik</t>
+        </is>
+      </c>
       <c r="H2" t="inlineStr">
         <is>
           <t>Besta Deild Karla</t>
@@ -563,27 +571,27 @@
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>Aegir vs Njardvik</t>
+          <t>Throttur Reykjavik vs Afturelding Mosfellsbaer</t>
         </is>
       </c>
       <c r="J2" t="inlineStr">
         <is>
-          <t>Aegir</t>
+          <t>Throttur Reykjavik</t>
         </is>
       </c>
       <c r="K2" t="inlineStr">
         <is>
-          <t>Njardvik</t>
+          <t>Afturelding Mosfellsbaer</t>
         </is>
       </c>
       <c r="L2" t="inlineStr">
         <is>
-          <t>0xde9c2677ae0e84c01c06a23050c75f29399db6bd766b2ef90484b73f8e0bbaed</t>
+          <t>0x7a5019973da533d172cf682264ba4b7ae8b6e65bb7591585a6fce73a807f64b0</t>
         </is>
       </c>
       <c r="M2" t="inlineStr">
         <is>
-          <t>L19548408</t>
+          <t>L19558554</t>
         </is>
       </c>
       <c r="N2" t="inlineStr">
@@ -608,17 +616,17 @@
       </c>
       <c r="R2" t="inlineStr">
         <is>
-          <t>1785237449</t>
+          <t>1785267812</t>
         </is>
       </c>
       <c r="S2" t="inlineStr">
         <is>
-          <t>1785266100</t>
+          <t>1785352500</t>
         </is>
       </c>
       <c r="T2" t="inlineStr">
         <is>
-          <t>20.748249</t>
+          <t>2.850123</t>
         </is>
       </c>
       <c r="U2" t="inlineStr">
@@ -635,31 +643,39 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>0xce612ac2221331f875649902eb6a0cde4b9db2f0f597bbc86e7caced63d25b99</t>
+          <t>0xf8236e3ab62a3112d2d962ecd3674bb25592395a1e4e2b076102954ddd699eb7</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>0x97EC1C9682F70091efB04e97b0B34698cF815EE1</t>
-        </is>
-      </c>
-      <c r="C3" t="inlineStr"/>
+          <t>0x5A76a26f838Ff5430Fd53E61CD8Bd76D895c946E</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>11.73</t>
+          <t>1.45</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>1.4412</t>
+          <t>1.5088</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>Under/Over (3.5)</t>
-        </is>
-      </c>
-      <c r="G3" t="inlineStr"/>
+          <t>1X2</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>Throttur Reykjavik</t>
+        </is>
+      </c>
       <c r="H3" t="inlineStr">
         <is>
           <t>Besta Deild Karla</t>
@@ -667,27 +683,27 @@
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>Aegir vs Njardvik</t>
+          <t>Throttur Reykjavik vs Afturelding Mosfellsbaer</t>
         </is>
       </c>
       <c r="J3" t="inlineStr">
         <is>
-          <t>Aegir</t>
+          <t>Throttur Reykjavik</t>
         </is>
       </c>
       <c r="K3" t="inlineStr">
         <is>
-          <t>Njardvik</t>
+          <t>Afturelding Mosfellsbaer</t>
         </is>
       </c>
       <c r="L3" t="inlineStr">
         <is>
-          <t>0x0825c99784fd72c055ffaeeb62e8e792f152ccd5a39c675722acf968b754f571</t>
+          <t>0x7a5019973da533d172cf682264ba4b7ae8b6e65bb7591585a6fce73a807f64b0</t>
         </is>
       </c>
       <c r="M3" t="inlineStr">
         <is>
-          <t>L19548408</t>
+          <t>L19558554</t>
         </is>
       </c>
       <c r="N3" t="inlineStr">
@@ -712,17 +728,17 @@
       </c>
       <c r="R3" t="inlineStr">
         <is>
-          <t>1785236520</t>
+          <t>1785267777</t>
         </is>
       </c>
       <c r="S3" t="inlineStr">
         <is>
-          <t>1785266100</t>
+          <t>1785352500</t>
         </is>
       </c>
       <c r="T3" t="inlineStr">
         <is>
-          <t>26.583569</t>
+          <t>2.850123</t>
         </is>
       </c>
       <c r="U3" t="inlineStr">
@@ -739,31 +755,39 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>0x7ae96391e38cfe39539922631da2025b36f57f1831d5f35ec6338463f27cb2a2</t>
+          <t>0x9c098bbf30f27adf5fb61d9dc7cffe685f61dacbc06ffd60f2ab0ab57bf9a296</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>0x5D69C3af95Ff47088b415B25F41b1fFDc8571063</t>
-        </is>
-      </c>
-      <c r="C4" t="inlineStr"/>
+          <t>0x5A76a26f838Ff5430Fd53E61CD8Bd76D895c946E</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>1.03</t>
+          <t>1.45</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>1.5525</t>
+          <t>1.5088</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>Under/Over (4)</t>
-        </is>
-      </c>
-      <c r="G4" t="inlineStr"/>
+          <t>1X2</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>Throttur Reykjavik</t>
+        </is>
+      </c>
       <c r="H4" t="inlineStr">
         <is>
           <t>Besta Deild Karla</t>
@@ -771,27 +795,27 @@
       </c>
       <c r="I4" t="inlineStr">
         <is>
-          <t>Aegir vs Njardvik</t>
+          <t>Throttur Reykjavik vs Afturelding Mosfellsbaer</t>
         </is>
       </c>
       <c r="J4" t="inlineStr">
         <is>
-          <t>Aegir</t>
+          <t>Throttur Reykjavik</t>
         </is>
       </c>
       <c r="K4" t="inlineStr">
         <is>
-          <t>Njardvik</t>
+          <t>Afturelding Mosfellsbaer</t>
         </is>
       </c>
       <c r="L4" t="inlineStr">
         <is>
-          <t>0xde9c2677ae0e84c01c06a23050c75f29399db6bd766b2ef90484b73f8e0bbaed</t>
+          <t>0x7a5019973da533d172cf682264ba4b7ae8b6e65bb7591585a6fce73a807f64b0</t>
         </is>
       </c>
       <c r="M4" t="inlineStr">
         <is>
-          <t>L19548408</t>
+          <t>L19558554</t>
         </is>
       </c>
       <c r="N4" t="inlineStr">
@@ -816,17 +840,17 @@
       </c>
       <c r="R4" t="inlineStr">
         <is>
-          <t>1785236069</t>
+          <t>1785267742</t>
         </is>
       </c>
       <c r="S4" t="inlineStr">
         <is>
-          <t>1785266100</t>
+          <t>1785352500</t>
         </is>
       </c>
       <c r="T4" t="inlineStr">
         <is>
-          <t>1.864253</t>
+          <t>2.850123</t>
         </is>
       </c>
       <c r="U4" t="inlineStr">
@@ -843,31 +867,39 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>0xc979cd389b2d4ca831b9a44b7738a2ae46abf46b1bd95d0fbe5b654a09413b1e</t>
+          <t>0x4c622a3a303c2e364803ca8b5f2417b149396b0a5a454b59e42697e254ae9315</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>0x97EC1C9682F70091efB04e97b0B34698cF815EE1</t>
-        </is>
-      </c>
-      <c r="C5" t="inlineStr"/>
+          <t>0x5A76a26f838Ff5430Fd53E61CD8Bd76D895c946E</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>5.59</t>
+          <t>1.45</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>1.4525</t>
+          <t>1.5088</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>Under/Over (3.5)</t>
-        </is>
-      </c>
-      <c r="G5" t="inlineStr"/>
+          <t>1X2</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>Throttur Reykjavik</t>
+        </is>
+      </c>
       <c r="H5" t="inlineStr">
         <is>
           <t>Besta Deild Karla</t>
@@ -875,27 +907,27 @@
       </c>
       <c r="I5" t="inlineStr">
         <is>
-          <t>Aegir vs Njardvik</t>
+          <t>Throttur Reykjavik vs Afturelding Mosfellsbaer</t>
         </is>
       </c>
       <c r="J5" t="inlineStr">
         <is>
-          <t>Aegir</t>
+          <t>Throttur Reykjavik</t>
         </is>
       </c>
       <c r="K5" t="inlineStr">
         <is>
-          <t>Njardvik</t>
+          <t>Afturelding Mosfellsbaer</t>
         </is>
       </c>
       <c r="L5" t="inlineStr">
         <is>
-          <t>0x0825c99784fd72c055ffaeeb62e8e792f152ccd5a39c675722acf968b754f571</t>
+          <t>0x7a5019973da533d172cf682264ba4b7ae8b6e65bb7591585a6fce73a807f64b0</t>
         </is>
       </c>
       <c r="M5" t="inlineStr">
         <is>
-          <t>L19548408</t>
+          <t>L19558554</t>
         </is>
       </c>
       <c r="N5" t="inlineStr">
@@ -920,17 +952,17 @@
       </c>
       <c r="R5" t="inlineStr">
         <is>
-          <t>1785235526</t>
+          <t>1785267709</t>
         </is>
       </c>
       <c r="S5" t="inlineStr">
         <is>
-          <t>1785266100</t>
+          <t>1785352500</t>
         </is>
       </c>
       <c r="T5" t="inlineStr">
         <is>
-          <t>12.353591</t>
+          <t>2.850123</t>
         </is>
       </c>
       <c r="U5" t="inlineStr">
@@ -947,30 +979,30 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>0x65bc0b70a6148d6f136b1552723c33dcf058e2ee7e6097ad6d18a39367f4821b</t>
+          <t>0x79c1f616b380c93f42fe785c942a2cc39edc55c4cdd4d5b6a09024c926a74f60</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>0x4a09916b1325Eed50eE8973B13742a205B0B7c7E</t>
-        </is>
-      </c>
-      <c r="C6" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
+          <t>0x97EC1C9682F70091efB04e97b0B34698cF815EE1</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr"/>
       <c r="D6" t="inlineStr">
         <is>
-          <t>35.0</t>
+          <t>11.22999</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>1.5987</t>
-        </is>
-      </c>
-      <c r="F6" t="inlineStr"/>
+          <t>1.5413</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>Under/Over (4)</t>
+        </is>
+      </c>
       <c r="G6" t="inlineStr"/>
       <c r="H6" t="inlineStr">
         <is>
@@ -979,32 +1011,32 @@
       </c>
       <c r="I6" t="inlineStr">
         <is>
-          <t>IR Reykjavik vs Fylkir</t>
+          <t>Aegir vs Njardvik</t>
         </is>
       </c>
       <c r="J6" t="inlineStr">
         <is>
-          <t>IR Reykjavik</t>
+          <t>Aegir</t>
         </is>
       </c>
       <c r="K6" t="inlineStr">
         <is>
-          <t>Fylkir</t>
+          <t>Njardvik</t>
         </is>
       </c>
       <c r="L6" t="inlineStr">
         <is>
-          <t>0xef2cff3047642c7d3f79713526decc2ed1438c01d374590eb62929362f824801</t>
+          <t>0xde9c2677ae0e84c01c06a23050c75f29399db6bd766b2ef90484b73f8e0bbaed</t>
         </is>
       </c>
       <c r="M6" t="inlineStr">
         <is>
-          <t>L19520873</t>
+          <t>L19548408</t>
         </is>
       </c>
       <c r="N6" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>0</t>
         </is>
       </c>
       <c r="O6" t="inlineStr">
@@ -1024,17 +1056,17 @@
       </c>
       <c r="R6" t="inlineStr">
         <is>
-          <t>1784987195</t>
+          <t>1785237449</t>
         </is>
       </c>
       <c r="S6" t="inlineStr">
         <is>
-          <t>1784988000</t>
+          <t>1785266100</t>
         </is>
       </c>
       <c r="T6" t="inlineStr">
         <is>
-          <t>59.090338</t>
+          <t>20.748249</t>
         </is>
       </c>
       <c r="U6" t="inlineStr">
@@ -1042,35 +1074,39 @@
           <t>SXR</t>
         </is>
       </c>
-      <c r="V6" t="inlineStr"/>
+      <c r="V6" t="inlineStr">
+        <is>
+          <t>0x6629Ce1Cf35Cc1329ebB4F63202F3f197b3F050B</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>0xd5e3b95bd82e0d7627a9203f0fe8fdd3b068e15fd373a543e05b207e66faf2a0</t>
+          <t>0xce612ac2221331f875649902eb6a0cde4b9db2f0f597bbc86e7caced63d25b99</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>0x68E1818FF20BBe84F9be9E0A4A395FB11079Bd35</t>
-        </is>
-      </c>
-      <c r="C7" t="inlineStr">
-        <is>
-          <t>2</t>
-        </is>
-      </c>
+          <t>0x97EC1C9682F70091efB04e97b0B34698cF815EE1</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr"/>
       <c r="D7" t="inlineStr">
         <is>
-          <t>12.0</t>
+          <t>11.73</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>1.7862</t>
-        </is>
-      </c>
-      <c r="F7" t="inlineStr"/>
+          <t>1.4412</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>Under/Over (3.5)</t>
+        </is>
+      </c>
       <c r="G7" t="inlineStr"/>
       <c r="H7" t="inlineStr">
         <is>
@@ -1079,32 +1115,32 @@
       </c>
       <c r="I7" t="inlineStr">
         <is>
-          <t>IR Reykjavik vs Fylkir</t>
+          <t>Aegir vs Njardvik</t>
         </is>
       </c>
       <c r="J7" t="inlineStr">
         <is>
-          <t>IR Reykjavik</t>
+          <t>Aegir</t>
         </is>
       </c>
       <c r="K7" t="inlineStr">
         <is>
-          <t>Fylkir</t>
+          <t>Njardvik</t>
         </is>
       </c>
       <c r="L7" t="inlineStr">
         <is>
-          <t>0x2b00f05607bf61216841f59440e877cc0eeb424e834132492c721bd4faedc556</t>
+          <t>0x0825c99784fd72c055ffaeeb62e8e792f152ccd5a39c675722acf968b754f571</t>
         </is>
       </c>
       <c r="M7" t="inlineStr">
         <is>
-          <t>L19520873</t>
+          <t>L19548408</t>
         </is>
       </c>
       <c r="N7" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>0</t>
         </is>
       </c>
       <c r="O7" t="inlineStr">
@@ -1124,17 +1160,17 @@
       </c>
       <c r="R7" t="inlineStr">
         <is>
-          <t>1784986980</t>
+          <t>1785236520</t>
         </is>
       </c>
       <c r="S7" t="inlineStr">
         <is>
-          <t>1784988000</t>
+          <t>1785266100</t>
         </is>
       </c>
       <c r="T7" t="inlineStr">
         <is>
-          <t>16.327479</t>
+          <t>26.583569</t>
         </is>
       </c>
       <c r="U7" t="inlineStr">
@@ -1142,35 +1178,39 @@
           <t>SXR</t>
         </is>
       </c>
-      <c r="V7" t="inlineStr"/>
+      <c r="V7" t="inlineStr">
+        <is>
+          <t>0x6629Ce1Cf35Cc1329ebB4F63202F3f197b3F050B</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>0xbfc0a906e601c3195b374e6d33b07e4c0b0dcbf09e05e45b8bd53226678d5d88</t>
+          <t>0x7ae96391e38cfe39539922631da2025b36f57f1831d5f35ec6338463f27cb2a2</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>0x68E1818FF20BBe84F9be9E0A4A395FB11079Bd35</t>
-        </is>
-      </c>
-      <c r="C8" t="inlineStr">
-        <is>
-          <t>2</t>
-        </is>
-      </c>
+          <t>0x5D69C3af95Ff47088b415B25F41b1fFDc8571063</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr"/>
       <c r="D8" t="inlineStr">
         <is>
-          <t>37.0</t>
+          <t>1.03</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>1.7875</t>
-        </is>
-      </c>
-      <c r="F8" t="inlineStr"/>
+          <t>1.5525</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>Under/Over (4)</t>
+        </is>
+      </c>
       <c r="G8" t="inlineStr"/>
       <c r="H8" t="inlineStr">
         <is>
@@ -1179,32 +1219,32 @@
       </c>
       <c r="I8" t="inlineStr">
         <is>
-          <t>IR Reykjavik vs Fylkir</t>
+          <t>Aegir vs Njardvik</t>
         </is>
       </c>
       <c r="J8" t="inlineStr">
         <is>
-          <t>IR Reykjavik</t>
+          <t>Aegir</t>
         </is>
       </c>
       <c r="K8" t="inlineStr">
         <is>
-          <t>Fylkir</t>
+          <t>Njardvik</t>
         </is>
       </c>
       <c r="L8" t="inlineStr">
         <is>
-          <t>0x2b00f05607bf61216841f59440e877cc0eeb424e834132492c721bd4faedc556</t>
+          <t>0xde9c2677ae0e84c01c06a23050c75f29399db6bd766b2ef90484b73f8e0bbaed</t>
         </is>
       </c>
       <c r="M8" t="inlineStr">
         <is>
-          <t>L19520873</t>
+          <t>L19548408</t>
         </is>
       </c>
       <c r="N8" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>0</t>
         </is>
       </c>
       <c r="O8" t="inlineStr">
@@ -1224,17 +1264,17 @@
       </c>
       <c r="R8" t="inlineStr">
         <is>
-          <t>1784986980</t>
+          <t>1785236069</t>
         </is>
       </c>
       <c r="S8" t="inlineStr">
         <is>
-          <t>1784988000</t>
+          <t>1785266100</t>
         </is>
       </c>
       <c r="T8" t="inlineStr">
         <is>
-          <t>47.105879</t>
+          <t>1.864253</t>
         </is>
       </c>
       <c r="U8" t="inlineStr">
@@ -1242,35 +1282,39 @@
           <t>SXR</t>
         </is>
       </c>
-      <c r="V8" t="inlineStr"/>
+      <c r="V8" t="inlineStr">
+        <is>
+          <t>0x6629Ce1Cf35Cc1329ebB4F63202F3f197b3F050B</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>0x5724a3badfc2012619fbf8e1a14ab0e7f4c66de896315371280c186505e86b85</t>
+          <t>0xc979cd389b2d4ca831b9a44b7738a2ae46abf46b1bd95d0fbe5b654a09413b1e</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>0xe2C68b7ef85645e47F9b94382c3Db59b046945a2</t>
-        </is>
-      </c>
-      <c r="C9" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
+          <t>0x97EC1C9682F70091efB04e97b0B34698cF815EE1</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr"/>
       <c r="D9" t="inlineStr">
         <is>
-          <t>69.0</t>
+          <t>5.59</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>1.6012</t>
-        </is>
-      </c>
-      <c r="F9" t="inlineStr"/>
+          <t>1.4525</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>Under/Over (3.5)</t>
+        </is>
+      </c>
       <c r="G9" t="inlineStr"/>
       <c r="H9" t="inlineStr">
         <is>
@@ -1279,32 +1323,32 @@
       </c>
       <c r="I9" t="inlineStr">
         <is>
-          <t>IR Reykjavik vs Fylkir</t>
+          <t>Aegir vs Njardvik</t>
         </is>
       </c>
       <c r="J9" t="inlineStr">
         <is>
-          <t>IR Reykjavik</t>
+          <t>Aegir</t>
         </is>
       </c>
       <c r="K9" t="inlineStr">
         <is>
-          <t>Fylkir</t>
+          <t>Njardvik</t>
         </is>
       </c>
       <c r="L9" t="inlineStr">
         <is>
-          <t>0x04fd78e33c10fb928e409323c26948f49fe4c81fcd47748d9153c9c611b38d0b</t>
+          <t>0x0825c99784fd72c055ffaeeb62e8e792f152ccd5a39c675722acf968b754f571</t>
         </is>
       </c>
       <c r="M9" t="inlineStr">
         <is>
-          <t>L19520873</t>
+          <t>L19548408</t>
         </is>
       </c>
       <c r="N9" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>0</t>
         </is>
       </c>
       <c r="O9" t="inlineStr">
@@ -1324,17 +1368,17 @@
       </c>
       <c r="R9" t="inlineStr">
         <is>
-          <t>1784986978</t>
+          <t>1785235526</t>
         </is>
       </c>
       <c r="S9" t="inlineStr">
         <is>
-          <t>1784988000</t>
+          <t>1785266100</t>
         </is>
       </c>
       <c r="T9" t="inlineStr">
         <is>
-          <t>114.884008</t>
+          <t>12.353591</t>
         </is>
       </c>
       <c r="U9" t="inlineStr">
@@ -1342,12 +1386,16 @@
           <t>SXR</t>
         </is>
       </c>
-      <c r="V9" t="inlineStr"/>
+      <c r="V9" t="inlineStr">
+        <is>
+          <t>0x6629Ce1Cf35Cc1329ebB4F63202F3f197b3F050B</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>0xf825a9ec3149d5a232253fd07078e2ed75a62b287df75e59fbb6c1546f6912a3</t>
+          <t>0x65bc0b70a6148d6f136b1552723c33dcf058e2ee7e6097ad6d18a39367f4821b</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
@@ -1362,12 +1410,12 @@
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>15.0</t>
+          <t>35.0</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>1.2712</t>
+          <t>1.5987</t>
         </is>
       </c>
       <c r="F10" t="inlineStr"/>
@@ -1394,7 +1442,7 @@
       </c>
       <c r="L10" t="inlineStr">
         <is>
-          <t>0x06a233f1b733d63cee459a37ac1beffad92b8f9ec21c414e0c26e2876b05eebd</t>
+          <t>0xef2cff3047642c7d3f79713526decc2ed1438c01d374590eb62929362f824801</t>
         </is>
       </c>
       <c r="M10" t="inlineStr">
@@ -1424,7 +1472,7 @@
       </c>
       <c r="R10" t="inlineStr">
         <is>
-          <t>1784984833</t>
+          <t>1784987195</t>
         </is>
       </c>
       <c r="S10" t="inlineStr">
@@ -1434,7 +1482,7 @@
       </c>
       <c r="T10" t="inlineStr">
         <is>
-          <t>58.211982</t>
+          <t>59.090338</t>
         </is>
       </c>
       <c r="U10" t="inlineStr">
@@ -1447,7 +1495,7 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>0x832d570bfcb61240d74893710e1758118ea62888a2bf55921f3190b9a71f4561</t>
+          <t>0xd5e3b95bd82e0d7627a9203f0fe8fdd3b068e15fd373a543e05b207e66faf2a0</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
@@ -1462,12 +1510,12 @@
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>3.0</t>
+          <t>12.0</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>1.7887</t>
+          <t>1.7862</t>
         </is>
       </c>
       <c r="F11" t="inlineStr"/>
@@ -1494,7 +1542,7 @@
       </c>
       <c r="L11" t="inlineStr">
         <is>
-          <t>0x91a9ea8ebfd8b049218a8e072590d2f657e26fdb1f2a49b1016ae42171c68ef2</t>
+          <t>0x2b00f05607bf61216841f59440e877cc0eeb424e834132492c721bd4faedc556</t>
         </is>
       </c>
       <c r="M11" t="inlineStr">
@@ -1524,7 +1572,7 @@
       </c>
       <c r="R11" t="inlineStr">
         <is>
-          <t>1784984812</t>
+          <t>1784986980</t>
         </is>
       </c>
       <c r="S11" t="inlineStr">
@@ -1534,7 +1582,7 @@
       </c>
       <c r="T11" t="inlineStr">
         <is>
-          <t>4.733718</t>
+          <t>16.327479</t>
         </is>
       </c>
       <c r="U11" t="inlineStr">
@@ -1547,7 +1595,7 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>0x78e73a1fbc4bce58e1469ba84a7a75afedee1c817a9927ff72cae6f55f5b4a58</t>
+          <t>0xbfc0a906e601c3195b374e6d33b07e4c0b0dcbf09e05e45b8bd53226678d5d88</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
@@ -1562,12 +1610,12 @@
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>8.0</t>
+          <t>37.0</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>1.7887</t>
+          <t>1.7875</t>
         </is>
       </c>
       <c r="F12" t="inlineStr"/>
@@ -1594,7 +1642,7 @@
       </c>
       <c r="L12" t="inlineStr">
         <is>
-          <t>0x91a9ea8ebfd8b049218a8e072590d2f657e26fdb1f2a49b1016ae42171c68ef2</t>
+          <t>0x2b00f05607bf61216841f59440e877cc0eeb424e834132492c721bd4faedc556</t>
         </is>
       </c>
       <c r="M12" t="inlineStr">
@@ -1624,7 +1672,7 @@
       </c>
       <c r="R12" t="inlineStr">
         <is>
-          <t>1784984812</t>
+          <t>1784986980</t>
         </is>
       </c>
       <c r="S12" t="inlineStr">
@@ -1634,7 +1682,7 @@
       </c>
       <c r="T12" t="inlineStr">
         <is>
-          <t>10.745559</t>
+          <t>47.105879</t>
         </is>
       </c>
       <c r="U12" t="inlineStr">
@@ -1647,12 +1695,12 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>0x02053d570c2ec6485bf734b3e9d25cb6962b678b5212cc142c9b62d371752a01</t>
+          <t>0x5724a3badfc2012619fbf8e1a14ab0e7f4c66de896315371280c186505e86b85</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>0x68E1818FF20BBe84F9be9E0A4A395FB11079Bd35</t>
+          <t>0xe2C68b7ef85645e47F9b94382c3Db59b046945a2</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
@@ -1662,12 +1710,12 @@
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>13.0</t>
+          <t>69.0</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>1.5737</t>
+          <t>1.6012</t>
         </is>
       </c>
       <c r="F13" t="inlineStr"/>
@@ -1724,7 +1772,7 @@
       </c>
       <c r="R13" t="inlineStr">
         <is>
-          <t>1784984812</t>
+          <t>1784986978</t>
         </is>
       </c>
       <c r="S13" t="inlineStr">
@@ -1734,7 +1782,7 @@
       </c>
       <c r="T13" t="inlineStr">
         <is>
-          <t>23.46041</t>
+          <t>114.884008</t>
         </is>
       </c>
       <c r="U13" t="inlineStr">
@@ -1747,7 +1795,7 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>0x6c8964e487e133d59a699205a9a6514d54217a61ad5ca3887aa005a89c8cbdfa</t>
+          <t>0xf825a9ec3149d5a232253fd07078e2ed75a62b287df75e59fbb6c1546f6912a3</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
@@ -1824,7 +1872,7 @@
       </c>
       <c r="R14" t="inlineStr">
         <is>
-          <t>1784984810</t>
+          <t>1784984833</t>
         </is>
       </c>
       <c r="S14" t="inlineStr">
@@ -1834,7 +1882,7 @@
       </c>
       <c r="T14" t="inlineStr">
         <is>
-          <t>58.209253</t>
+          <t>58.211982</t>
         </is>
       </c>
       <c r="U14" t="inlineStr">
@@ -1847,27 +1895,27 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>0xb8b680dda4305fed43c95dc6dbc059c9678abe5f31da65b83ac57ecd5c8d3903</t>
+          <t>0x832d570bfcb61240d74893710e1758118ea62888a2bf55921f3190b9a71f4561</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>0x4a09916b1325Eed50eE8973B13742a205B0B7c7E</t>
+          <t>0x68E1818FF20BBe84F9be9E0A4A395FB11079Bd35</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>16.0</t>
+          <t>3.0</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>1.2712</t>
+          <t>1.7887</t>
         </is>
       </c>
       <c r="F15" t="inlineStr"/>
@@ -1894,7 +1942,7 @@
       </c>
       <c r="L15" t="inlineStr">
         <is>
-          <t>0x06a233f1b733d63cee459a37ac1beffad92b8f9ec21c414e0c26e2876b05eebd</t>
+          <t>0x91a9ea8ebfd8b049218a8e072590d2f657e26fdb1f2a49b1016ae42171c68ef2</t>
         </is>
       </c>
       <c r="M15" t="inlineStr">
@@ -1924,7 +1972,7 @@
       </c>
       <c r="R15" t="inlineStr">
         <is>
-          <t>1784984670</t>
+          <t>1784984812</t>
         </is>
       </c>
       <c r="S15" t="inlineStr">
@@ -1934,7 +1982,7 @@
       </c>
       <c r="T15" t="inlineStr">
         <is>
-          <t>60.198968</t>
+          <t>4.733718</t>
         </is>
       </c>
       <c r="U15" t="inlineStr">
@@ -1947,27 +1995,27 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>0x374cde0708e064be0b99fea4bb71434540b7ca7bbd1a444cb12a8b14c6aa3c48</t>
+          <t>0x78e73a1fbc4bce58e1469ba84a7a75afedee1c817a9927ff72cae6f55f5b4a58</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>0x4a09916b1325Eed50eE8973B13742a205B0B7c7E</t>
+          <t>0x68E1818FF20BBe84F9be9E0A4A395FB11079Bd35</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>16.0</t>
+          <t>8.0</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>1.2712</t>
+          <t>1.7887</t>
         </is>
       </c>
       <c r="F16" t="inlineStr"/>
@@ -1994,7 +2042,7 @@
       </c>
       <c r="L16" t="inlineStr">
         <is>
-          <t>0x06a233f1b733d63cee459a37ac1beffad92b8f9ec21c414e0c26e2876b05eebd</t>
+          <t>0x91a9ea8ebfd8b049218a8e072590d2f657e26fdb1f2a49b1016ae42171c68ef2</t>
         </is>
       </c>
       <c r="M16" t="inlineStr">
@@ -2024,7 +2072,7 @@
       </c>
       <c r="R16" t="inlineStr">
         <is>
-          <t>1784984617</t>
+          <t>1784984812</t>
         </is>
       </c>
       <c r="S16" t="inlineStr">
@@ -2034,7 +2082,7 @@
       </c>
       <c r="T16" t="inlineStr">
         <is>
-          <t>60.198968</t>
+          <t>10.745559</t>
         </is>
       </c>
       <c r="U16" t="inlineStr">
@@ -2047,12 +2095,12 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>0x4c094ddc4f89a7cbd768baf6a26f7e686ead028a4b15ee75fd8f4927e1ad7989</t>
+          <t>0x02053d570c2ec6485bf734b3e9d25cb6962b678b5212cc142c9b62d371752a01</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>0x4a09916b1325Eed50eE8973B13742a205B0B7c7E</t>
+          <t>0x68E1818FF20BBe84F9be9E0A4A395FB11079Bd35</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
@@ -2062,12 +2110,12 @@
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>16.0</t>
+          <t>13.0</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>1.2712</t>
+          <t>1.5737</t>
         </is>
       </c>
       <c r="F17" t="inlineStr"/>
@@ -2094,7 +2142,7 @@
       </c>
       <c r="L17" t="inlineStr">
         <is>
-          <t>0x06a233f1b733d63cee459a37ac1beffad92b8f9ec21c414e0c26e2876b05eebd</t>
+          <t>0x04fd78e33c10fb928e409323c26948f49fe4c81fcd47748d9153c9c611b38d0b</t>
         </is>
       </c>
       <c r="M17" t="inlineStr">
@@ -2124,7 +2172,7 @@
       </c>
       <c r="R17" t="inlineStr">
         <is>
-          <t>1784984581</t>
+          <t>1784984812</t>
         </is>
       </c>
       <c r="S17" t="inlineStr">
@@ -2134,7 +2182,7 @@
       </c>
       <c r="T17" t="inlineStr">
         <is>
-          <t>60.198968</t>
+          <t>23.46041</t>
         </is>
       </c>
       <c r="U17" t="inlineStr">
@@ -2147,7 +2195,7 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>0x7dd8d48e4f9e00707e79d58d5900292571189d9de19bd23c6c6a9a433ea96f72</t>
+          <t>0x6c8964e487e133d59a699205a9a6514d54217a61ad5ca3887aa005a89c8cbdfa</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
@@ -2162,7 +2210,7 @@
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>16.0</t>
+          <t>15.0</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
@@ -2224,7 +2272,7 @@
       </c>
       <c r="R18" t="inlineStr">
         <is>
-          <t>1784984563</t>
+          <t>1784984810</t>
         </is>
       </c>
       <c r="S18" t="inlineStr">
@@ -2234,7 +2282,7 @@
       </c>
       <c r="T18" t="inlineStr">
         <is>
-          <t>60.198968</t>
+          <t>58.209253</t>
         </is>
       </c>
       <c r="U18" t="inlineStr">
@@ -2247,7 +2295,7 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>0x7354c940dd56ae7caca9fa9b1a548dcf53e1a3516f531216c677cf582affb4fe</t>
+          <t>0xb8b680dda4305fed43c95dc6dbc059c9678abe5f31da65b83ac57ecd5c8d3903</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
@@ -2262,12 +2310,12 @@
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>9.0</t>
+          <t>16.0</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>1.3013</t>
+          <t>1.2712</t>
         </is>
       </c>
       <c r="F19" t="inlineStr"/>
@@ -2324,7 +2372,7 @@
       </c>
       <c r="R19" t="inlineStr">
         <is>
-          <t>1784984538</t>
+          <t>1784984670</t>
         </is>
       </c>
       <c r="S19" t="inlineStr">
@@ -2334,7 +2382,7 @@
       </c>
       <c r="T19" t="inlineStr">
         <is>
-          <t>31.184232</t>
+          <t>60.198968</t>
         </is>
       </c>
       <c r="U19" t="inlineStr">
@@ -2347,12 +2395,12 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>0xdc3c1508859b265a9cc7ea3dadc58bb672f939bf46cde2c06081ec2891a03946</t>
+          <t>0x374cde0708e064be0b99fea4bb71434540b7ca7bbd1a444cb12a8b14c6aa3c48</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>0xC88F614A48f8A705d7465b03aAF62ddaca0c3754</t>
+          <t>0x4a09916b1325Eed50eE8973B13742a205B0B7c7E</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
@@ -2362,12 +2410,12 @@
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>21.0</t>
+          <t>16.0</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>1.4363</t>
+          <t>1.2712</t>
         </is>
       </c>
       <c r="F20" t="inlineStr"/>
@@ -2394,7 +2442,7 @@
       </c>
       <c r="L20" t="inlineStr">
         <is>
-          <t>0xd5ae8f2322bcc6adaca1c1bb1baf6a74afa50cc30131840c87632f67865c23d0</t>
+          <t>0x06a233f1b733d63cee459a37ac1beffad92b8f9ec21c414e0c26e2876b05eebd</t>
         </is>
       </c>
       <c r="M20" t="inlineStr">
@@ -2424,7 +2472,7 @@
       </c>
       <c r="R20" t="inlineStr">
         <is>
-          <t>1784984537</t>
+          <t>1784984617</t>
         </is>
       </c>
       <c r="S20" t="inlineStr">
@@ -2434,7 +2482,7 @@
       </c>
       <c r="T20" t="inlineStr">
         <is>
-          <t>48.297994</t>
+          <t>60.198968</t>
         </is>
       </c>
       <c r="U20" t="inlineStr">
@@ -2447,12 +2495,12 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>0x0bf6c8f6ea5d7452bf543eb72d99a66c1b6ff74a5e56b4ad9449b6870f225d2d</t>
+          <t>0x4c094ddc4f89a7cbd768baf6a26f7e686ead028a4b15ee75fd8f4927e1ad7989</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>0x47D0CE9b8d653c8884DB7E2a7F88d4849E0CD980</t>
+          <t>0x4a09916b1325Eed50eE8973B13742a205B0B7c7E</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
@@ -2462,12 +2510,12 @@
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>38.0</t>
+          <t>16.0</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>1.5537</t>
+          <t>1.2712</t>
         </is>
       </c>
       <c r="F21" t="inlineStr"/>
@@ -2494,7 +2542,7 @@
       </c>
       <c r="L21" t="inlineStr">
         <is>
-          <t>0x04fd78e33c10fb928e409323c26948f49fe4c81fcd47748d9153c9c611b38d0b</t>
+          <t>0x06a233f1b733d63cee459a37ac1beffad92b8f9ec21c414e0c26e2876b05eebd</t>
         </is>
       </c>
       <c r="M21" t="inlineStr">
@@ -2524,7 +2572,7 @@
       </c>
       <c r="R21" t="inlineStr">
         <is>
-          <t>1784984536</t>
+          <t>1784984581</t>
         </is>
       </c>
       <c r="S21" t="inlineStr">
@@ -2534,7 +2582,7 @@
       </c>
       <c r="T21" t="inlineStr">
         <is>
-          <t>68.833427</t>
+          <t>60.198968</t>
         </is>
       </c>
       <c r="U21" t="inlineStr">
@@ -2547,12 +2595,12 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>0xa4b5b4c3c3766e7d708b5373412745aa0b0d5f4c097f5451a2210d6d019269c6</t>
+          <t>0x7dd8d48e4f9e00707e79d58d5900292571189d9de19bd23c6c6a9a433ea96f72</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>0x47D0CE9b8d653c8884DB7E2a7F88d4849E0CD980</t>
+          <t>0x4a09916b1325Eed50eE8973B13742a205B0B7c7E</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
@@ -2562,12 +2610,12 @@
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>29.0</t>
+          <t>16.0</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>1.5537</t>
+          <t>1.2712</t>
         </is>
       </c>
       <c r="F22" t="inlineStr"/>
@@ -2594,7 +2642,7 @@
       </c>
       <c r="L22" t="inlineStr">
         <is>
-          <t>0x04fd78e33c10fb928e409323c26948f49fe4c81fcd47748d9153c9c611b38d0b</t>
+          <t>0x06a233f1b733d63cee459a37ac1beffad92b8f9ec21c414e0c26e2876b05eebd</t>
         </is>
       </c>
       <c r="M22" t="inlineStr">
@@ -2624,7 +2672,7 @@
       </c>
       <c r="R22" t="inlineStr">
         <is>
-          <t>1784984502</t>
+          <t>1784984563</t>
         </is>
       </c>
       <c r="S22" t="inlineStr">
@@ -2634,7 +2682,7 @@
       </c>
       <c r="T22" t="inlineStr">
         <is>
-          <t>53.355738</t>
+          <t>60.198968</t>
         </is>
       </c>
       <c r="U22" t="inlineStr">
@@ -2647,12 +2695,12 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>0xfac3960037b540d1b0b49f14ff5313d7db5bd6320c356e510ef3e6bdaca6d1ff</t>
+          <t>0x7354c940dd56ae7caca9fa9b1a548dcf53e1a3516f531216c677cf582affb4fe</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>0x47D0CE9b8d653c8884DB7E2a7F88d4849E0CD980</t>
+          <t>0x4a09916b1325Eed50eE8973B13742a205B0B7c7E</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
@@ -2662,12 +2710,12 @@
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>25.0</t>
+          <t>9.0</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>1.5537</t>
+          <t>1.3013</t>
         </is>
       </c>
       <c r="F23" t="inlineStr"/>
@@ -2694,7 +2742,7 @@
       </c>
       <c r="L23" t="inlineStr">
         <is>
-          <t>0x04fd78e33c10fb928e409323c26948f49fe4c81fcd47748d9153c9c611b38d0b</t>
+          <t>0x06a233f1b733d63cee459a37ac1beffad92b8f9ec21c414e0c26e2876b05eebd</t>
         </is>
       </c>
       <c r="M23" t="inlineStr">
@@ -2724,7 +2772,7 @@
       </c>
       <c r="R23" t="inlineStr">
         <is>
-          <t>1784984501</t>
+          <t>1784984538</t>
         </is>
       </c>
       <c r="S23" t="inlineStr">
@@ -2734,7 +2782,7 @@
       </c>
       <c r="T23" t="inlineStr">
         <is>
-          <t>46.408957</t>
+          <t>31.184232</t>
         </is>
       </c>
       <c r="U23" t="inlineStr">
@@ -2747,12 +2795,12 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>0xf3b65016998beda20548812c7503abc20be0fa3abedc59c3ac7e08e6b82c70f1</t>
+          <t>0xdc3c1508859b265a9cc7ea3dadc58bb672f939bf46cde2c06081ec2891a03946</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>0x4a09916b1325Eed50eE8973B13742a205B0B7c7E</t>
+          <t>0xC88F614A48f8A705d7465b03aAF62ddaca0c3754</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
@@ -2762,12 +2810,12 @@
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>6.0</t>
+          <t>21.0</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>1.3013</t>
+          <t>1.4363</t>
         </is>
       </c>
       <c r="F24" t="inlineStr"/>
@@ -2794,7 +2842,7 @@
       </c>
       <c r="L24" t="inlineStr">
         <is>
-          <t>0x06a233f1b733d63cee459a37ac1beffad92b8f9ec21c414e0c26e2876b05eebd</t>
+          <t>0xd5ae8f2322bcc6adaca1c1bb1baf6a74afa50cc30131840c87632f67865c23d0</t>
         </is>
       </c>
       <c r="M24" t="inlineStr">
@@ -2824,7 +2872,7 @@
       </c>
       <c r="R24" t="inlineStr">
         <is>
-          <t>1784984431</t>
+          <t>1784984537</t>
         </is>
       </c>
       <c r="S24" t="inlineStr">
@@ -2834,7 +2882,7 @@
       </c>
       <c r="T24" t="inlineStr">
         <is>
-          <t>22.912332</t>
+          <t>48.297994</t>
         </is>
       </c>
       <c r="U24" t="inlineStr">
@@ -2847,12 +2895,12 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>0xa04fcfb1b689fd17d1c3c66ac2ed73a6e0b99d30bdfd296529ca6549b4642440</t>
+          <t>0x0bf6c8f6ea5d7452bf543eb72d99a66c1b6ff74a5e56b4ad9449b6870f225d2d</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>0x4a09916b1325Eed50eE8973B13742a205B0B7c7E</t>
+          <t>0x47D0CE9b8d653c8884DB7E2a7F88d4849E0CD980</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
@@ -2862,12 +2910,12 @@
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>27.0</t>
+          <t>38.0</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>1.4537</t>
+          <t>1.5537</t>
         </is>
       </c>
       <c r="F25" t="inlineStr"/>
@@ -2894,7 +2942,7 @@
       </c>
       <c r="L25" t="inlineStr">
         <is>
-          <t>0xd5ae8f2322bcc6adaca1c1bb1baf6a74afa50cc30131840c87632f67865c23d0</t>
+          <t>0x04fd78e33c10fb928e409323c26948f49fe4c81fcd47748d9153c9c611b38d0b</t>
         </is>
       </c>
       <c r="M25" t="inlineStr">
@@ -2924,7 +2972,7 @@
       </c>
       <c r="R25" t="inlineStr">
         <is>
-          <t>1784984405</t>
+          <t>1784984536</t>
         </is>
       </c>
       <c r="S25" t="inlineStr">
@@ -2934,7 +2982,7 @@
       </c>
       <c r="T25" t="inlineStr">
         <is>
-          <t>60.187328</t>
+          <t>68.833427</t>
         </is>
       </c>
       <c r="U25" t="inlineStr">
@@ -2947,12 +2995,12 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>0xb07983b62c387b953f021bde51a561f510162701d56466ec78a20a598c01d8c4</t>
+          <t>0xa4b5b4c3c3766e7d708b5373412745aa0b0d5f4c097f5451a2210d6d019269c6</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>0x4a09916b1325Eed50eE8973B13742a205B0B7c7E</t>
+          <t>0x47D0CE9b8d653c8884DB7E2a7F88d4849E0CD980</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
@@ -2962,12 +3010,12 @@
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>35.0</t>
+          <t>29.0</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>1.595</t>
+          <t>1.5537</t>
         </is>
       </c>
       <c r="F26" t="inlineStr"/>
@@ -2994,7 +3042,7 @@
       </c>
       <c r="L26" t="inlineStr">
         <is>
-          <t>0xe1204c11efd43d8d3a0377591c468bba3ac169f58ab541c6d60665f2e0bbb051</t>
+          <t>0x04fd78e33c10fb928e409323c26948f49fe4c81fcd47748d9153c9c611b38d0b</t>
         </is>
       </c>
       <c r="M26" t="inlineStr">
@@ -3024,7 +3072,7 @@
       </c>
       <c r="R26" t="inlineStr">
         <is>
-          <t>1784984404</t>
+          <t>1784984502</t>
         </is>
       </c>
       <c r="S26" t="inlineStr">
@@ -3034,7 +3082,7 @@
       </c>
       <c r="T26" t="inlineStr">
         <is>
-          <t>60.197529</t>
+          <t>53.355738</t>
         </is>
       </c>
       <c r="U26" t="inlineStr">
@@ -3047,27 +3095,27 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>0xc41db21ce0b5921299bba16424467dff9a9a6eb4d744a5aadf04422f8138f34f</t>
+          <t>0xfac3960037b540d1b0b49f14ff5313d7db5bd6320c356e510ef3e6bdaca6d1ff</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>0x68E1818FF20BBe84F9be9E0A4A395FB11079Bd35</t>
+          <t>0x47D0CE9b8d653c8884DB7E2a7F88d4849E0CD980</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>1</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>22.0</t>
+          <t>25.0</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>1.7712</t>
+          <t>1.5537</t>
         </is>
       </c>
       <c r="F27" t="inlineStr"/>
@@ -3094,7 +3142,7 @@
       </c>
       <c r="L27" t="inlineStr">
         <is>
-          <t>0x91a9ea8ebfd8b049218a8e072590d2f657e26fdb1f2a49b1016ae42171c68ef2</t>
+          <t>0x04fd78e33c10fb928e409323c26948f49fe4c81fcd47748d9153c9c611b38d0b</t>
         </is>
       </c>
       <c r="M27" t="inlineStr">
@@ -3124,7 +3172,7 @@
       </c>
       <c r="R27" t="inlineStr">
         <is>
-          <t>1784984403</t>
+          <t>1784984501</t>
         </is>
       </c>
       <c r="S27" t="inlineStr">
@@ -3134,7 +3182,7 @@
       </c>
       <c r="T27" t="inlineStr">
         <is>
-          <t>29.185737</t>
+          <t>46.408957</t>
         </is>
       </c>
       <c r="U27" t="inlineStr">
@@ -3147,27 +3195,27 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>0x97d57842a441d56ad4d0172a6e2460bdd3644bd55476d419863d144ec4fb3f02</t>
+          <t>0xf3b65016998beda20548812c7503abc20be0fa3abedc59c3ac7e08e6b82c70f1</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>0x68E1818FF20BBe84F9be9E0A4A395FB11079Bd35</t>
+          <t>0x4a09916b1325Eed50eE8973B13742a205B0B7c7E</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>1</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>3.0</t>
+          <t>6.0</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>1.775</t>
+          <t>1.3013</t>
         </is>
       </c>
       <c r="F28" t="inlineStr"/>
@@ -3194,7 +3242,7 @@
       </c>
       <c r="L28" t="inlineStr">
         <is>
-          <t>0x2b00f05607bf61216841f59440e877cc0eeb424e834132492c721bd4faedc556</t>
+          <t>0x06a233f1b733d63cee459a37ac1beffad92b8f9ec21c414e0c26e2876b05eebd</t>
         </is>
       </c>
       <c r="M28" t="inlineStr">
@@ -3224,7 +3272,7 @@
       </c>
       <c r="R28" t="inlineStr">
         <is>
-          <t>1784984403</t>
+          <t>1784984431</t>
         </is>
       </c>
       <c r="S28" t="inlineStr">
@@ -3234,7 +3282,7 @@
       </c>
       <c r="T28" t="inlineStr">
         <is>
-          <t>4.444439</t>
+          <t>22.912332</t>
         </is>
       </c>
       <c r="U28" t="inlineStr">
@@ -3247,7 +3295,7 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>0x54a44d2ce4be4b546daee52057d4611c0f1d29571a9747f66b3462780e888ae0</t>
+          <t>0xa04fcfb1b689fd17d1c3c66ac2ed73a6e0b99d30bdfd296529ca6549b4642440</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
@@ -3262,12 +3310,12 @@
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>17.0</t>
+          <t>27.0</t>
         </is>
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>1.2988</t>
+          <t>1.4537</t>
         </is>
       </c>
       <c r="F29" t="inlineStr"/>
@@ -3294,7 +3342,7 @@
       </c>
       <c r="L29" t="inlineStr">
         <is>
-          <t>0x588a71865f90131e16b5b72dfef6ddb7cec8deb7df1f8102477a62eaa807cc71</t>
+          <t>0xd5ae8f2322bcc6adaca1c1bb1baf6a74afa50cc30131840c87632f67865c23d0</t>
         </is>
       </c>
       <c r="M29" t="inlineStr">
@@ -3324,7 +3372,7 @@
       </c>
       <c r="R29" t="inlineStr">
         <is>
-          <t>1784984402</t>
+          <t>1784984405</t>
         </is>
       </c>
       <c r="S29" t="inlineStr">
@@ -3334,7 +3382,7 @@
       </c>
       <c r="T29" t="inlineStr">
         <is>
-          <t>60.178243</t>
+          <t>60.187328</t>
         </is>
       </c>
       <c r="U29" t="inlineStr">
@@ -3347,7 +3395,7 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>0xf9d293335e6b1b3fd21eba9ec71cbbd6cbce398d5d606b38175d3776a077cb91</t>
+          <t>0xb07983b62c387b953f021bde51a561f510162701d56466ec78a20a598c01d8c4</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
@@ -3362,12 +3410,12 @@
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>41.0</t>
+          <t>35.0</t>
         </is>
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>1.685</t>
+          <t>1.595</t>
         </is>
       </c>
       <c r="F30" t="inlineStr"/>
@@ -3394,7 +3442,7 @@
       </c>
       <c r="L30" t="inlineStr">
         <is>
-          <t>0xaf0827308b557ecc964e4c608c6b71f345660fa965da2a0e02882ee62ce45e49</t>
+          <t>0xe1204c11efd43d8d3a0377591c468bba3ac169f58ab541c6d60665f2e0bbb051</t>
         </is>
       </c>
       <c r="M30" t="inlineStr">
@@ -3424,7 +3472,7 @@
       </c>
       <c r="R30" t="inlineStr">
         <is>
-          <t>1784984401</t>
+          <t>1784984404</t>
         </is>
       </c>
       <c r="S30" t="inlineStr">
@@ -3434,7 +3482,7 @@
       </c>
       <c r="T30" t="inlineStr">
         <is>
-          <t>60.189781</t>
+          <t>60.197529</t>
         </is>
       </c>
       <c r="U30" t="inlineStr">
@@ -3447,27 +3495,27 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>0x80f610f55e907d511b2c5a8d77d03f9aca143e4e50b6d7fba92997ba46481bde</t>
+          <t>0xc41db21ce0b5921299bba16424467dff9a9a6eb4d744a5aadf04422f8138f34f</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>0x47D0CE9b8d653c8884DB7E2a7F88d4849E0CD980</t>
+          <t>0x68E1818FF20BBe84F9be9E0A4A395FB11079Bd35</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>6.0</t>
+          <t>22.0</t>
         </is>
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>1.5537</t>
+          <t>1.7712</t>
         </is>
       </c>
       <c r="F31" t="inlineStr"/>
@@ -3494,7 +3542,7 @@
       </c>
       <c r="L31" t="inlineStr">
         <is>
-          <t>0x04fd78e33c10fb928e409323c26948f49fe4c81fcd47748d9153c9c611b38d0b</t>
+          <t>0x91a9ea8ebfd8b049218a8e072590d2f657e26fdb1f2a49b1016ae42171c68ef2</t>
         </is>
       </c>
       <c r="M31" t="inlineStr">
@@ -3524,7 +3572,7 @@
       </c>
       <c r="R31" t="inlineStr">
         <is>
-          <t>1784983849</t>
+          <t>1784984403</t>
         </is>
       </c>
       <c r="S31" t="inlineStr">
@@ -3534,7 +3582,7 @@
       </c>
       <c r="T31" t="inlineStr">
         <is>
-          <t>11.988786</t>
+          <t>29.185737</t>
         </is>
       </c>
       <c r="U31" t="inlineStr">
@@ -3547,7 +3595,7 @@
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>0x6e3d6f822ebfe70f563004b4a5a4a6303f1d1cb9677e6e3a56324cda8cc92ba7</t>
+          <t>0x97d57842a441d56ad4d0172a6e2460bdd3644bd55476d419863d144ec4fb3f02</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
@@ -3557,17 +3605,17 @@
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>25.0</t>
+          <t>3.0</t>
         </is>
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>1.5513</t>
+          <t>1.775</t>
         </is>
       </c>
       <c r="F32" t="inlineStr"/>
@@ -3594,7 +3642,7 @@
       </c>
       <c r="L32" t="inlineStr">
         <is>
-          <t>0x04fd78e33c10fb928e409323c26948f49fe4c81fcd47748d9153c9c611b38d0b</t>
+          <t>0x2b00f05607bf61216841f59440e877cc0eeb424e834132492c721bd4faedc556</t>
         </is>
       </c>
       <c r="M32" t="inlineStr">
@@ -3624,7 +3672,7 @@
       </c>
       <c r="R32" t="inlineStr">
         <is>
-          <t>1784983797</t>
+          <t>1784984403</t>
         </is>
       </c>
       <c r="S32" t="inlineStr">
@@ -3634,7 +3682,7 @@
       </c>
       <c r="T32" t="inlineStr">
         <is>
-          <t>46.150404</t>
+          <t>4.444439</t>
         </is>
       </c>
       <c r="U32" t="inlineStr">
@@ -3647,27 +3695,27 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>0xc913b7104d801ceb0283dc9eefcce577969c93f7b16c1cc5515036561b5b8d8e</t>
+          <t>0x54a44d2ce4be4b546daee52057d4611c0f1d29571a9747f66b3462780e888ae0</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>0x68E1818FF20BBe84F9be9E0A4A395FB11079Bd35</t>
+          <t>0x4a09916b1325Eed50eE8973B13742a205B0B7c7E</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>1</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>4.0</t>
+          <t>17.0</t>
         </is>
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>1.7712</t>
+          <t>1.2988</t>
         </is>
       </c>
       <c r="F33" t="inlineStr"/>
@@ -3694,7 +3742,7 @@
       </c>
       <c r="L33" t="inlineStr">
         <is>
-          <t>0x91a9ea8ebfd8b049218a8e072590d2f657e26fdb1f2a49b1016ae42171c68ef2</t>
+          <t>0x588a71865f90131e16b5b72dfef6ddb7cec8deb7df1f8102477a62eaa807cc71</t>
         </is>
       </c>
       <c r="M33" t="inlineStr">
@@ -3724,7 +3772,7 @@
       </c>
       <c r="R33" t="inlineStr">
         <is>
-          <t>1784983703</t>
+          <t>1784984402</t>
         </is>
       </c>
       <c r="S33" t="inlineStr">
@@ -3734,7 +3782,7 @@
       </c>
       <c r="T33" t="inlineStr">
         <is>
-          <t>5.770489</t>
+          <t>60.178243</t>
         </is>
       </c>
       <c r="U33" t="inlineStr">
@@ -3747,12 +3795,12 @@
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>0x78c593e23cd10a2517f77039f922e2d360ba0b6d4c89dc91bac22f6854ce01ea</t>
+          <t>0xf9d293335e6b1b3fd21eba9ec71cbbd6cbce398d5d606b38175d3776a077cb91</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>0x68E1818FF20BBe84F9be9E0A4A395FB11079Bd35</t>
+          <t>0x4a09916b1325Eed50eE8973B13742a205B0B7c7E</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
@@ -3762,12 +3810,12 @@
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>2.0</t>
+          <t>41.0</t>
         </is>
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t>1.5513</t>
+          <t>1.685</t>
         </is>
       </c>
       <c r="F34" t="inlineStr"/>
@@ -3794,7 +3842,7 @@
       </c>
       <c r="L34" t="inlineStr">
         <is>
-          <t>0x04fd78e33c10fb928e409323c26948f49fe4c81fcd47748d9153c9c611b38d0b</t>
+          <t>0xaf0827308b557ecc964e4c608c6b71f345660fa965da2a0e02882ee62ce45e49</t>
         </is>
       </c>
       <c r="M34" t="inlineStr">
@@ -3824,7 +3872,7 @@
       </c>
       <c r="R34" t="inlineStr">
         <is>
-          <t>1784983703</t>
+          <t>1784984401</t>
         </is>
       </c>
       <c r="S34" t="inlineStr">
@@ -3834,7 +3882,7 @@
       </c>
       <c r="T34" t="inlineStr">
         <is>
-          <t>4.389968</t>
+          <t>60.189781</t>
         </is>
       </c>
       <c r="U34" t="inlineStr">
@@ -3847,12 +3895,12 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>0x589562dc55239bfc299045a0e5bbfed420cc8f286ee7326d34ed350f83ecdd45</t>
+          <t>0x80f610f55e907d511b2c5a8d77d03f9aca143e4e50b6d7fba92997ba46481bde</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>0x68E1818FF20BBe84F9be9E0A4A395FB11079Bd35</t>
+          <t>0x47D0CE9b8d653c8884DB7E2a7F88d4849E0CD980</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
@@ -3862,12 +3910,12 @@
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>12.0</t>
+          <t>6.0</t>
         </is>
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>1.5513</t>
+          <t>1.5537</t>
         </is>
       </c>
       <c r="F35" t="inlineStr"/>
@@ -3924,7 +3972,7 @@
       </c>
       <c r="R35" t="inlineStr">
         <is>
-          <t>1784983480</t>
+          <t>1784983849</t>
         </is>
       </c>
       <c r="S35" t="inlineStr">
@@ -3934,7 +3982,7 @@
       </c>
       <c r="T35" t="inlineStr">
         <is>
-          <t>22.284118</t>
+          <t>11.988786</t>
         </is>
       </c>
       <c r="U35" t="inlineStr">
@@ -3947,7 +3995,7 @@
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>0x629a7bab69ed2f6eae5804065863061a8e5f95bfbf35104c3a1d130585e021ca</t>
+          <t>0x6e3d6f822ebfe70f563004b4a5a4a6303f1d1cb9677e6e3a56324cda8cc92ba7</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
@@ -3962,7 +4010,7 @@
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>1.0</t>
+          <t>25.0</t>
         </is>
       </c>
       <c r="E36" t="inlineStr">
@@ -4024,7 +4072,7 @@
       </c>
       <c r="R36" t="inlineStr">
         <is>
-          <t>1784983361</t>
+          <t>1784983797</t>
         </is>
       </c>
       <c r="S36" t="inlineStr">
@@ -4034,7 +4082,7 @@
       </c>
       <c r="T36" t="inlineStr">
         <is>
-          <t>2.228408</t>
+          <t>46.150404</t>
         </is>
       </c>
       <c r="U36" t="inlineStr">
@@ -4047,27 +4095,27 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>0x888b7311174b291a1eeccf40a054d1599070da16bd2f2f7adea95d18002cc686</t>
+          <t>0xc913b7104d801ceb0283dc9eefcce577969c93f7b16c1cc5515036561b5b8d8e</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>0xB1854fc8aD8ce649EA80D007Fc67d318a239a5DA</t>
+          <t>0x68E1818FF20BBe84F9be9E0A4A395FB11079Bd35</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>0.0</t>
+          <t>4.0</t>
         </is>
       </c>
       <c r="E37" t="inlineStr">
         <is>
-          <t>1.215</t>
+          <t>1.7712</t>
         </is>
       </c>
       <c r="F37" t="inlineStr"/>
@@ -4124,7 +4172,7 @@
       </c>
       <c r="R37" t="inlineStr">
         <is>
-          <t>1784981088</t>
+          <t>1784983703</t>
         </is>
       </c>
       <c r="S37" t="inlineStr">
@@ -4134,7 +4182,7 @@
       </c>
       <c r="T37" t="inlineStr">
         <is>
-          <t>1.443442</t>
+          <t>5.770489</t>
         </is>
       </c>
       <c r="U37" t="inlineStr">
@@ -4147,7 +4195,7 @@
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>0x5d44678e836886d72dc3bddfca4b44d2be2bfa7f56096dbedd259cac92e30df3</t>
+          <t>0x78c593e23cd10a2517f77039f922e2d360ba0b6d4c89dc91bac22f6854ce01ea</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
@@ -4157,17 +4205,17 @@
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>1</t>
         </is>
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>16.0</t>
+          <t>2.0</t>
         </is>
       </c>
       <c r="E38" t="inlineStr">
         <is>
-          <t>1.7712</t>
+          <t>1.5513</t>
         </is>
       </c>
       <c r="F38" t="inlineStr"/>
@@ -4194,7 +4242,7 @@
       </c>
       <c r="L38" t="inlineStr">
         <is>
-          <t>0x91a9ea8ebfd8b049218a8e072590d2f657e26fdb1f2a49b1016ae42171c68ef2</t>
+          <t>0x04fd78e33c10fb928e409323c26948f49fe4c81fcd47748d9153c9c611b38d0b</t>
         </is>
       </c>
       <c r="M38" t="inlineStr">
@@ -4224,7 +4272,7 @@
       </c>
       <c r="R38" t="inlineStr">
         <is>
-          <t>1784981082</t>
+          <t>1784983703</t>
         </is>
       </c>
       <c r="S38" t="inlineStr">
@@ -4234,7 +4282,7 @@
       </c>
       <c r="T38" t="inlineStr">
         <is>
-          <t>21.377037</t>
+          <t>4.389968</t>
         </is>
       </c>
       <c r="U38" t="inlineStr">
@@ -4247,7 +4295,7 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>0x5a96bb0ca1d506186a0e2c1c2e13d657784bbb03ad3f75e66db86da80f485bae</t>
+          <t>0x589562dc55239bfc299045a0e5bbfed420cc8f286ee7326d34ed350f83ecdd45</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
@@ -4262,7 +4310,7 @@
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>19.0</t>
+          <t>12.0</t>
         </is>
       </c>
       <c r="E39" t="inlineStr">
@@ -4324,7 +4372,7 @@
       </c>
       <c r="R39" t="inlineStr">
         <is>
-          <t>1784980847</t>
+          <t>1784983480</t>
         </is>
       </c>
       <c r="S39" t="inlineStr">
@@ -4334,7 +4382,7 @@
       </c>
       <c r="T39" t="inlineStr">
         <is>
-          <t>35.743728</t>
+          <t>22.284118</t>
         </is>
       </c>
       <c r="U39" t="inlineStr">
@@ -4347,12 +4395,12 @@
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>0xe6e61e0b4573e8e2199880691f7803f1943269d2b2b955ea7282a833c4dbc3c6</t>
+          <t>0x629a7bab69ed2f6eae5804065863061a8e5f95bfbf35104c3a1d130585e021ca</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>0x47D0CE9b8d653c8884DB7E2a7F88d4849E0CD980</t>
+          <t>0x68E1818FF20BBe84F9be9E0A4A395FB11079Bd35</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
@@ -4362,12 +4410,12 @@
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>22.0</t>
+          <t>1.0</t>
         </is>
       </c>
       <c r="E40" t="inlineStr">
         <is>
-          <t>1.555</t>
+          <t>1.5513</t>
         </is>
       </c>
       <c r="F40" t="inlineStr"/>
@@ -4424,7 +4472,7 @@
       </c>
       <c r="R40" t="inlineStr">
         <is>
-          <t>1784977858</t>
+          <t>1784983361</t>
         </is>
       </c>
       <c r="S40" t="inlineStr">
@@ -4434,7 +4482,7 @@
       </c>
       <c r="T40" t="inlineStr">
         <is>
-          <t>39.775279</t>
+          <t>2.228408</t>
         </is>
       </c>
       <c r="U40" t="inlineStr">
@@ -4447,12 +4495,12 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>0x668fc309ba15ebe234fe9dd2d2bf696a9f4000c9ac85f8e7d55c998a052968dc</t>
+          <t>0x888b7311174b291a1eeccf40a054d1599070da16bd2f2f7adea95d18002cc686</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>0x47D0CE9b8d653c8884DB7E2a7F88d4849E0CD980</t>
+          <t>0xB1854fc8aD8ce649EA80D007Fc67d318a239a5DA</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
@@ -4462,12 +4510,12 @@
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t>27.0</t>
+          <t>0.0</t>
         </is>
       </c>
       <c r="E41" t="inlineStr">
         <is>
-          <t>1.555</t>
+          <t>1.215</t>
         </is>
       </c>
       <c r="F41" t="inlineStr"/>
@@ -4494,7 +4542,7 @@
       </c>
       <c r="L41" t="inlineStr">
         <is>
-          <t>0x04fd78e33c10fb928e409323c26948f49fe4c81fcd47748d9153c9c611b38d0b</t>
+          <t>0x91a9ea8ebfd8b049218a8e072590d2f657e26fdb1f2a49b1016ae42171c68ef2</t>
         </is>
       </c>
       <c r="M41" t="inlineStr">
@@ -4524,7 +4572,7 @@
       </c>
       <c r="R41" t="inlineStr">
         <is>
-          <t>1784977853</t>
+          <t>1784981088</t>
         </is>
       </c>
       <c r="S41" t="inlineStr">
@@ -4534,7 +4582,7 @@
       </c>
       <c r="T41" t="inlineStr">
         <is>
-          <t>49.797748</t>
+          <t>1.443442</t>
         </is>
       </c>
       <c r="U41" t="inlineStr">
@@ -4547,12 +4595,12 @@
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>0xabcdef492212262464335967adbaa23c5214ede2fab0ea2a12bce6e0027067aa</t>
+          <t>0x5d44678e836886d72dc3bddfca4b44d2be2bfa7f56096dbedd259cac92e30df3</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>0xC88F614A48f8A705d7465b03aAF62ddaca0c3754</t>
+          <t>0x68E1818FF20BBe84F9be9E0A4A395FB11079Bd35</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
@@ -4562,12 +4610,12 @@
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t>20.0</t>
+          <t>16.0</t>
         </is>
       </c>
       <c r="E42" t="inlineStr">
         <is>
-          <t>1.435</t>
+          <t>1.7712</t>
         </is>
       </c>
       <c r="F42" t="inlineStr"/>
@@ -4594,7 +4642,7 @@
       </c>
       <c r="L42" t="inlineStr">
         <is>
-          <t>0xef2cff3047642c7d3f79713526decc2ed1438c01d374590eb62929362f824801</t>
+          <t>0x91a9ea8ebfd8b049218a8e072590d2f657e26fdb1f2a49b1016ae42171c68ef2</t>
         </is>
       </c>
       <c r="M42" t="inlineStr">
@@ -4624,7 +4672,7 @@
       </c>
       <c r="R42" t="inlineStr">
         <is>
-          <t>1784968614</t>
+          <t>1784981082</t>
         </is>
       </c>
       <c r="S42" t="inlineStr">
@@ -4634,7 +4682,7 @@
       </c>
       <c r="T42" t="inlineStr">
         <is>
-          <t>47.149425</t>
+          <t>21.377037</t>
         </is>
       </c>
       <c r="U42" t="inlineStr">
@@ -4647,12 +4695,12 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>0xf7e34584abe1fc7da16770ad9dc2fe59e91a45480c1ff509d55070c7d811c7e2</t>
+          <t>0x5a96bb0ca1d506186a0e2c1c2e13d657784bbb03ad3f75e66db86da80f485bae</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>0x516bfc7CE57c0E1734388ECed5Bb9454aA6aeFae</t>
+          <t>0x68E1818FF20BBe84F9be9E0A4A395FB11079Bd35</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
@@ -4662,12 +4710,12 @@
       </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t>10.0</t>
+          <t>19.0</t>
         </is>
       </c>
       <c r="E43" t="inlineStr">
         <is>
-          <t>1.56</t>
+          <t>1.5513</t>
         </is>
       </c>
       <c r="F43" t="inlineStr"/>
@@ -4694,7 +4742,7 @@
       </c>
       <c r="L43" t="inlineStr">
         <is>
-          <t>0xe1204c11efd43d8d3a0377591c468bba3ac169f58ab541c6d60665f2e0bbb051</t>
+          <t>0x04fd78e33c10fb928e409323c26948f49fe4c81fcd47748d9153c9c611b38d0b</t>
         </is>
       </c>
       <c r="M43" t="inlineStr">
@@ -4724,7 +4772,7 @@
       </c>
       <c r="R43" t="inlineStr">
         <is>
-          <t>1784907257</t>
+          <t>1784980847</t>
         </is>
       </c>
       <c r="S43" t="inlineStr">
@@ -4734,7 +4782,7 @@
       </c>
       <c r="T43" t="inlineStr">
         <is>
-          <t>17.857143</t>
+          <t>35.743728</t>
         </is>
       </c>
       <c r="U43" t="inlineStr">
@@ -4747,12 +4795,12 @@
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>0x030841d8eff7e23d98d8319e71f99f9eb17cb2a743343cfac134410b86f1178e</t>
+          <t>0xe6e61e0b4573e8e2199880691f7803f1943269d2b2b955ea7282a833c4dbc3c6</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>0xC88F614A48f8A705d7465b03aAF62ddaca0c3754</t>
+          <t>0x47D0CE9b8d653c8884DB7E2a7F88d4849E0CD980</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
@@ -4762,12 +4810,12 @@
       </c>
       <c r="D44" t="inlineStr">
         <is>
-          <t>26.0</t>
+          <t>22.0</t>
         </is>
       </c>
       <c r="E44" t="inlineStr">
         <is>
-          <t>1.5737</t>
+          <t>1.555</t>
         </is>
       </c>
       <c r="F44" t="inlineStr"/>
@@ -4794,7 +4842,7 @@
       </c>
       <c r="L44" t="inlineStr">
         <is>
-          <t>0xe1204c11efd43d8d3a0377591c468bba3ac169f58ab541c6d60665f2e0bbb051</t>
+          <t>0x04fd78e33c10fb928e409323c26948f49fe4c81fcd47748d9153c9c611b38d0b</t>
         </is>
       </c>
       <c r="M44" t="inlineStr">
@@ -4824,7 +4872,7 @@
       </c>
       <c r="R44" t="inlineStr">
         <is>
-          <t>1784907053</t>
+          <t>1784977858</t>
         </is>
       </c>
       <c r="S44" t="inlineStr">
@@ -4834,7 +4882,7 @@
       </c>
       <c r="T44" t="inlineStr">
         <is>
-          <t>46.28739</t>
+          <t>39.775279</t>
         </is>
       </c>
       <c r="U44" t="inlineStr">
@@ -4847,12 +4895,12 @@
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>0xd486facb98ea7c7e7b67efb74b5231332788279dbd71dce40eea54aecf5d870e</t>
+          <t>0x668fc309ba15ebe234fe9dd2d2bf696a9f4000c9ac85f8e7d55c998a052968dc</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>0xC88F614A48f8A705d7465b03aAF62ddaca0c3754</t>
+          <t>0x47D0CE9b8d653c8884DB7E2a7F88d4849E0CD980</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
@@ -4862,12 +4910,12 @@
       </c>
       <c r="D45" t="inlineStr">
         <is>
-          <t>14.0</t>
+          <t>27.0</t>
         </is>
       </c>
       <c r="E45" t="inlineStr">
         <is>
-          <t>1.315</t>
+          <t>1.555</t>
         </is>
       </c>
       <c r="F45" t="inlineStr"/>
@@ -4894,7 +4942,7 @@
       </c>
       <c r="L45" t="inlineStr">
         <is>
-          <t>0x588a71865f90131e16b5b72dfef6ddb7cec8deb7df1f8102477a62eaa807cc71</t>
+          <t>0x04fd78e33c10fb928e409323c26948f49fe4c81fcd47748d9153c9c611b38d0b</t>
         </is>
       </c>
       <c r="M45" t="inlineStr">
@@ -4924,7 +4972,7 @@
       </c>
       <c r="R45" t="inlineStr">
         <is>
-          <t>1784907041</t>
+          <t>1784977853</t>
         </is>
       </c>
       <c r="S45" t="inlineStr">
@@ -4934,7 +4982,7 @@
       </c>
       <c r="T45" t="inlineStr">
         <is>
-          <t>47.587302</t>
+          <t>49.797748</t>
         </is>
       </c>
       <c r="U45" t="inlineStr">
@@ -4947,7 +4995,7 @@
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>0x8a9596cb004924470885fe466db8f8d059fcb9d1b24e71490dd35bfeba65a98d</t>
+          <t>0xabcdef492212262464335967adbaa23c5214ede2fab0ea2a12bce6e0027067aa</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
@@ -4957,17 +5005,17 @@
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
       <c r="D46" t="inlineStr">
         <is>
-          <t>14.0</t>
+          <t>20.0</t>
         </is>
       </c>
       <c r="E46" t="inlineStr">
         <is>
-          <t>1.315</t>
+          <t>1.435</t>
         </is>
       </c>
       <c r="F46" t="inlineStr"/>
@@ -4994,7 +5042,7 @@
       </c>
       <c r="L46" t="inlineStr">
         <is>
-          <t>0x06a233f1b733d63cee459a37ac1beffad92b8f9ec21c414e0c26e2876b05eebd</t>
+          <t>0xef2cff3047642c7d3f79713526decc2ed1438c01d374590eb62929362f824801</t>
         </is>
       </c>
       <c r="M46" t="inlineStr">
@@ -5024,7 +5072,7 @@
       </c>
       <c r="R46" t="inlineStr">
         <is>
-          <t>1784907041</t>
+          <t>1784968614</t>
         </is>
       </c>
       <c r="S46" t="inlineStr">
@@ -5034,7 +5082,7 @@
       </c>
       <c r="T46" t="inlineStr">
         <is>
-          <t>47.555556</t>
+          <t>47.149425</t>
         </is>
       </c>
       <c r="U46" t="inlineStr">
@@ -5047,12 +5095,12 @@
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>0xdaf8fe8a287cecb340987a0eebd287e9d8e007af24d015fcadd720fceba485cd</t>
+          <t>0xf7e34584abe1fc7da16770ad9dc2fe59e91a45480c1ff509d55070c7d811c7e2</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>0xC88F614A48f8A705d7465b03aAF62ddaca0c3754</t>
+          <t>0x516bfc7CE57c0E1734388ECed5Bb9454aA6aeFae</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
@@ -5062,12 +5110,12 @@
       </c>
       <c r="D47" t="inlineStr">
         <is>
-          <t>26.0</t>
+          <t>10.0</t>
         </is>
       </c>
       <c r="E47" t="inlineStr">
         <is>
-          <t>1.57</t>
+          <t>1.56</t>
         </is>
       </c>
       <c r="F47" t="inlineStr"/>
@@ -5124,7 +5172,7 @@
       </c>
       <c r="R47" t="inlineStr">
         <is>
-          <t>1784907040</t>
+          <t>1784907257</t>
         </is>
       </c>
       <c r="S47" t="inlineStr">
@@ -5134,7 +5182,7 @@
       </c>
       <c r="T47" t="inlineStr">
         <is>
-          <t>47.046509</t>
+          <t>17.857143</t>
         </is>
       </c>
       <c r="U47" t="inlineStr">
@@ -5147,7 +5195,7 @@
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>0x3f981c0415a637d3cb9137ae5b4b0b4b0c50f1a3af5d4e42f65e682f80daadba</t>
+          <t>0x030841d8eff7e23d98d8319e71f99f9eb17cb2a743343cfac134410b86f1178e</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
@@ -5162,12 +5210,12 @@
       </c>
       <c r="D48" t="inlineStr">
         <is>
-          <t>22.0</t>
+          <t>26.0</t>
         </is>
       </c>
       <c r="E48" t="inlineStr">
         <is>
-          <t>1.4625</t>
+          <t>1.5737</t>
         </is>
       </c>
       <c r="F48" t="inlineStr"/>
@@ -5194,55 +5242,455 @@
       </c>
       <c r="L48" t="inlineStr">
         <is>
+          <t>0xe1204c11efd43d8d3a0377591c468bba3ac169f58ab541c6d60665f2e0bbb051</t>
+        </is>
+      </c>
+      <c r="M48" t="inlineStr">
+        <is>
+          <t>L19520873</t>
+        </is>
+      </c>
+      <c r="N48" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="O48" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="P48" t="inlineStr">
+        <is>
+          <t>SUCCESS</t>
+        </is>
+      </c>
+      <c r="Q48" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="R48" t="inlineStr">
+        <is>
+          <t>1784907053</t>
+        </is>
+      </c>
+      <c r="S48" t="inlineStr">
+        <is>
+          <t>1784988000</t>
+        </is>
+      </c>
+      <c r="T48" t="inlineStr">
+        <is>
+          <t>46.28739</t>
+        </is>
+      </c>
+      <c r="U48" t="inlineStr">
+        <is>
+          <t>SXR</t>
+        </is>
+      </c>
+      <c r="V48" t="inlineStr"/>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>0xd486facb98ea7c7e7b67efb74b5231332788279dbd71dce40eea54aecf5d870e</t>
+        </is>
+      </c>
+      <c r="B49" t="inlineStr">
+        <is>
+          <t>0xC88F614A48f8A705d7465b03aAF62ddaca0c3754</t>
+        </is>
+      </c>
+      <c r="C49" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="D49" t="inlineStr">
+        <is>
+          <t>14.0</t>
+        </is>
+      </c>
+      <c r="E49" t="inlineStr">
+        <is>
+          <t>1.315</t>
+        </is>
+      </c>
+      <c r="F49" t="inlineStr"/>
+      <c r="G49" t="inlineStr"/>
+      <c r="H49" t="inlineStr">
+        <is>
+          <t>Besta Deild Karla</t>
+        </is>
+      </c>
+      <c r="I49" t="inlineStr">
+        <is>
+          <t>IR Reykjavik vs Fylkir</t>
+        </is>
+      </c>
+      <c r="J49" t="inlineStr">
+        <is>
+          <t>IR Reykjavik</t>
+        </is>
+      </c>
+      <c r="K49" t="inlineStr">
+        <is>
+          <t>Fylkir</t>
+        </is>
+      </c>
+      <c r="L49" t="inlineStr">
+        <is>
+          <t>0x588a71865f90131e16b5b72dfef6ddb7cec8deb7df1f8102477a62eaa807cc71</t>
+        </is>
+      </c>
+      <c r="M49" t="inlineStr">
+        <is>
+          <t>L19520873</t>
+        </is>
+      </c>
+      <c r="N49" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="O49" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="P49" t="inlineStr">
+        <is>
+          <t>SUCCESS</t>
+        </is>
+      </c>
+      <c r="Q49" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="R49" t="inlineStr">
+        <is>
+          <t>1784907041</t>
+        </is>
+      </c>
+      <c r="S49" t="inlineStr">
+        <is>
+          <t>1784988000</t>
+        </is>
+      </c>
+      <c r="T49" t="inlineStr">
+        <is>
+          <t>47.587302</t>
+        </is>
+      </c>
+      <c r="U49" t="inlineStr">
+        <is>
+          <t>SXR</t>
+        </is>
+      </c>
+      <c r="V49" t="inlineStr"/>
+    </row>
+    <row r="50">
+      <c r="A50" t="inlineStr">
+        <is>
+          <t>0x8a9596cb004924470885fe466db8f8d059fcb9d1b24e71490dd35bfeba65a98d</t>
+        </is>
+      </c>
+      <c r="B50" t="inlineStr">
+        <is>
+          <t>0xC88F614A48f8A705d7465b03aAF62ddaca0c3754</t>
+        </is>
+      </c>
+      <c r="C50" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="D50" t="inlineStr">
+        <is>
+          <t>14.0</t>
+        </is>
+      </c>
+      <c r="E50" t="inlineStr">
+        <is>
+          <t>1.315</t>
+        </is>
+      </c>
+      <c r="F50" t="inlineStr"/>
+      <c r="G50" t="inlineStr"/>
+      <c r="H50" t="inlineStr">
+        <is>
+          <t>Besta Deild Karla</t>
+        </is>
+      </c>
+      <c r="I50" t="inlineStr">
+        <is>
+          <t>IR Reykjavik vs Fylkir</t>
+        </is>
+      </c>
+      <c r="J50" t="inlineStr">
+        <is>
+          <t>IR Reykjavik</t>
+        </is>
+      </c>
+      <c r="K50" t="inlineStr">
+        <is>
+          <t>Fylkir</t>
+        </is>
+      </c>
+      <c r="L50" t="inlineStr">
+        <is>
+          <t>0x06a233f1b733d63cee459a37ac1beffad92b8f9ec21c414e0c26e2876b05eebd</t>
+        </is>
+      </c>
+      <c r="M50" t="inlineStr">
+        <is>
+          <t>L19520873</t>
+        </is>
+      </c>
+      <c r="N50" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="O50" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="P50" t="inlineStr">
+        <is>
+          <t>SUCCESS</t>
+        </is>
+      </c>
+      <c r="Q50" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="R50" t="inlineStr">
+        <is>
+          <t>1784907041</t>
+        </is>
+      </c>
+      <c r="S50" t="inlineStr">
+        <is>
+          <t>1784988000</t>
+        </is>
+      </c>
+      <c r="T50" t="inlineStr">
+        <is>
+          <t>47.555556</t>
+        </is>
+      </c>
+      <c r="U50" t="inlineStr">
+        <is>
+          <t>SXR</t>
+        </is>
+      </c>
+      <c r="V50" t="inlineStr"/>
+    </row>
+    <row r="51">
+      <c r="A51" t="inlineStr">
+        <is>
+          <t>0xdaf8fe8a287cecb340987a0eebd287e9d8e007af24d015fcadd720fceba485cd</t>
+        </is>
+      </c>
+      <c r="B51" t="inlineStr">
+        <is>
+          <t>0xC88F614A48f8A705d7465b03aAF62ddaca0c3754</t>
+        </is>
+      </c>
+      <c r="C51" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="D51" t="inlineStr">
+        <is>
+          <t>26.0</t>
+        </is>
+      </c>
+      <c r="E51" t="inlineStr">
+        <is>
+          <t>1.57</t>
+        </is>
+      </c>
+      <c r="F51" t="inlineStr"/>
+      <c r="G51" t="inlineStr"/>
+      <c r="H51" t="inlineStr">
+        <is>
+          <t>Besta Deild Karla</t>
+        </is>
+      </c>
+      <c r="I51" t="inlineStr">
+        <is>
+          <t>IR Reykjavik vs Fylkir</t>
+        </is>
+      </c>
+      <c r="J51" t="inlineStr">
+        <is>
+          <t>IR Reykjavik</t>
+        </is>
+      </c>
+      <c r="K51" t="inlineStr">
+        <is>
+          <t>Fylkir</t>
+        </is>
+      </c>
+      <c r="L51" t="inlineStr">
+        <is>
+          <t>0xe1204c11efd43d8d3a0377591c468bba3ac169f58ab541c6d60665f2e0bbb051</t>
+        </is>
+      </c>
+      <c r="M51" t="inlineStr">
+        <is>
+          <t>L19520873</t>
+        </is>
+      </c>
+      <c r="N51" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="O51" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="P51" t="inlineStr">
+        <is>
+          <t>SUCCESS</t>
+        </is>
+      </c>
+      <c r="Q51" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="R51" t="inlineStr">
+        <is>
+          <t>1784907040</t>
+        </is>
+      </c>
+      <c r="S51" t="inlineStr">
+        <is>
+          <t>1784988000</t>
+        </is>
+      </c>
+      <c r="T51" t="inlineStr">
+        <is>
+          <t>47.046509</t>
+        </is>
+      </c>
+      <c r="U51" t="inlineStr">
+        <is>
+          <t>SXR</t>
+        </is>
+      </c>
+      <c r="V51" t="inlineStr"/>
+    </row>
+    <row r="52">
+      <c r="A52" t="inlineStr">
+        <is>
+          <t>0x3f981c0415a637d3cb9137ae5b4b0b4b0c50f1a3af5d4e42f65e682f80daadba</t>
+        </is>
+      </c>
+      <c r="B52" t="inlineStr">
+        <is>
+          <t>0xC88F614A48f8A705d7465b03aAF62ddaca0c3754</t>
+        </is>
+      </c>
+      <c r="C52" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="D52" t="inlineStr">
+        <is>
+          <t>22.0</t>
+        </is>
+      </c>
+      <c r="E52" t="inlineStr">
+        <is>
+          <t>1.4625</t>
+        </is>
+      </c>
+      <c r="F52" t="inlineStr"/>
+      <c r="G52" t="inlineStr"/>
+      <c r="H52" t="inlineStr">
+        <is>
+          <t>Besta Deild Karla</t>
+        </is>
+      </c>
+      <c r="I52" t="inlineStr">
+        <is>
+          <t>IR Reykjavik vs Fylkir</t>
+        </is>
+      </c>
+      <c r="J52" t="inlineStr">
+        <is>
+          <t>IR Reykjavik</t>
+        </is>
+      </c>
+      <c r="K52" t="inlineStr">
+        <is>
+          <t>Fylkir</t>
+        </is>
+      </c>
+      <c r="L52" t="inlineStr">
+        <is>
           <t>0xd5ae8f2322bcc6adaca1c1bb1baf6a74afa50cc30131840c87632f67865c23d0</t>
         </is>
       </c>
-      <c r="M48" t="inlineStr">
+      <c r="M52" t="inlineStr">
         <is>
           <t>L19520873</t>
         </is>
       </c>
-      <c r="N48" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="O48" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="P48" t="inlineStr">
+      <c r="N52" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="O52" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="P52" t="inlineStr">
         <is>
           <t>SUCCESS</t>
         </is>
       </c>
-      <c r="Q48" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="R48" t="inlineStr">
+      <c r="Q52" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="R52" t="inlineStr">
         <is>
           <t>1784907040</t>
         </is>
       </c>
-      <c r="S48" t="inlineStr">
+      <c r="S52" t="inlineStr">
         <is>
           <t>1784988000</t>
         </is>
       </c>
-      <c r="T48" t="inlineStr">
+      <c r="T52" t="inlineStr">
         <is>
           <t>47.589189</t>
         </is>
       </c>
-      <c r="U48" t="inlineStr">
+      <c r="U52" t="inlineStr">
         <is>
           <t>SXR</t>
         </is>
       </c>
-      <c r="V48" t="inlineStr"/>
+      <c r="V52" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Update soccer trades 2026-07-29 06:01:08 UTC
</commit_message>
<xml_diff>
--- a/data/sxbet/ligas/Besta Deild Karla/trades.xlsx
+++ b/data/sxbet/ligas/Besta Deild Karla/trades.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:V52"/>
+  <dimension ref="A1:V54"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -531,12 +531,12 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>0xda116ce959332ba41194293702cd84c233a1aa5dc72f06cf3a812e3b16c89f50</t>
+          <t>0xa9c4c39c3003eff066c3a4586da774f5987355742d4863d64aa5984bf9a94e7e</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>0x5A76a26f838Ff5430Fd53E61CD8Bd76D895c946E</t>
+          <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
@@ -546,12 +546,12 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>1.45</t>
+          <t>1</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>1.5088</t>
+          <t>1.3375</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
@@ -561,7 +561,7 @@
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>Throttur Reykjavik</t>
+          <t>Leiknir Reykjavik</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">
@@ -571,27 +571,27 @@
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>Throttur Reykjavik vs Afturelding Mosfellsbaer</t>
+          <t>Grindavík vs Leiknir Reykjavik</t>
         </is>
       </c>
       <c r="J2" t="inlineStr">
         <is>
-          <t>Throttur Reykjavik</t>
+          <t>Grindavík</t>
         </is>
       </c>
       <c r="K2" t="inlineStr">
         <is>
-          <t>Afturelding Mosfellsbaer</t>
+          <t>Leiknir Reykjavik</t>
         </is>
       </c>
       <c r="L2" t="inlineStr">
         <is>
-          <t>0x7a5019973da533d172cf682264ba4b7ae8b6e65bb7591585a6fce73a807f64b0</t>
+          <t>0xa483946547c248863e7e21964d2b27f06ba27a90ee1332f03f91f58c894d0ab5</t>
         </is>
       </c>
       <c r="M2" t="inlineStr">
         <is>
-          <t>L19558554</t>
+          <t>L19558553</t>
         </is>
       </c>
       <c r="N2" t="inlineStr">
@@ -616,7 +616,7 @@
       </c>
       <c r="R2" t="inlineStr">
         <is>
-          <t>1785267812</t>
+          <t>1785298455</t>
         </is>
       </c>
       <c r="S2" t="inlineStr">
@@ -626,7 +626,7 @@
       </c>
       <c r="T2" t="inlineStr">
         <is>
-          <t>2.850123</t>
+          <t>2.962963</t>
         </is>
       </c>
       <c r="U2" t="inlineStr">
@@ -643,12 +643,12 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>0xf8236e3ab62a3112d2d962ecd3674bb25592395a1e4e2b076102954ddd699eb7</t>
+          <t>0xee5e46dfcd55125e8c178c7b7ec5808cbc3059b6cb7c8b8db7ac3eed5d7918bc</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>0x5A76a26f838Ff5430Fd53E61CD8Bd76D895c946E</t>
+          <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -658,12 +658,12 @@
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>1.45</t>
+          <t>0.00209</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>1.5088</t>
+          <t>1.3375</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
@@ -673,7 +673,7 @@
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>Throttur Reykjavik</t>
+          <t>Leiknir Reykjavik</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
@@ -683,27 +683,27 @@
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>Throttur Reykjavik vs Afturelding Mosfellsbaer</t>
+          <t>Grindavík vs Leiknir Reykjavik</t>
         </is>
       </c>
       <c r="J3" t="inlineStr">
         <is>
-          <t>Throttur Reykjavik</t>
+          <t>Grindavík</t>
         </is>
       </c>
       <c r="K3" t="inlineStr">
         <is>
-          <t>Afturelding Mosfellsbaer</t>
+          <t>Leiknir Reykjavik</t>
         </is>
       </c>
       <c r="L3" t="inlineStr">
         <is>
-          <t>0x7a5019973da533d172cf682264ba4b7ae8b6e65bb7591585a6fce73a807f64b0</t>
+          <t>0xa483946547c248863e7e21964d2b27f06ba27a90ee1332f03f91f58c894d0ab5</t>
         </is>
       </c>
       <c r="M3" t="inlineStr">
         <is>
-          <t>L19558554</t>
+          <t>L19558553</t>
         </is>
       </c>
       <c r="N3" t="inlineStr">
@@ -728,7 +728,7 @@
       </c>
       <c r="R3" t="inlineStr">
         <is>
-          <t>1785267777</t>
+          <t>1785298146</t>
         </is>
       </c>
       <c r="S3" t="inlineStr">
@@ -738,7 +738,7 @@
       </c>
       <c r="T3" t="inlineStr">
         <is>
-          <t>2.850123</t>
+          <t>0.006193</t>
         </is>
       </c>
       <c r="U3" t="inlineStr">
@@ -755,7 +755,7 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>0x9c098bbf30f27adf5fb61d9dc7cffe685f61dacbc06ffd60f2ab0ab57bf9a296</t>
+          <t>0xda116ce959332ba41194293702cd84c233a1aa5dc72f06cf3a812e3b16c89f50</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -840,7 +840,7 @@
       </c>
       <c r="R4" t="inlineStr">
         <is>
-          <t>1785267742</t>
+          <t>1785267812</t>
         </is>
       </c>
       <c r="S4" t="inlineStr">
@@ -867,7 +867,7 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>0x4c622a3a303c2e364803ca8b5f2417b149396b0a5a454b59e42697e254ae9315</t>
+          <t>0xf8236e3ab62a3112d2d962ecd3674bb25592395a1e4e2b076102954ddd699eb7</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
@@ -952,7 +952,7 @@
       </c>
       <c r="R5" t="inlineStr">
         <is>
-          <t>1785267709</t>
+          <t>1785267777</t>
         </is>
       </c>
       <c r="S5" t="inlineStr">
@@ -979,31 +979,39 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>0x79c1f616b380c93f42fe785c942a2cc39edc55c4cdd4d5b6a09024c926a74f60</t>
+          <t>0x9c098bbf30f27adf5fb61d9dc7cffe685f61dacbc06ffd60f2ab0ab57bf9a296</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>0x97EC1C9682F70091efB04e97b0B34698cF815EE1</t>
-        </is>
-      </c>
-      <c r="C6" t="inlineStr"/>
+          <t>0x5A76a26f838Ff5430Fd53E61CD8Bd76D895c946E</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>11.22999</t>
+          <t>1.45</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>1.5413</t>
+          <t>1.5088</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>Under/Over (4)</t>
-        </is>
-      </c>
-      <c r="G6" t="inlineStr"/>
+          <t>1X2</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>Throttur Reykjavik</t>
+        </is>
+      </c>
       <c r="H6" t="inlineStr">
         <is>
           <t>Besta Deild Karla</t>
@@ -1011,27 +1019,27 @@
       </c>
       <c r="I6" t="inlineStr">
         <is>
-          <t>Aegir vs Njardvik</t>
+          <t>Throttur Reykjavik vs Afturelding Mosfellsbaer</t>
         </is>
       </c>
       <c r="J6" t="inlineStr">
         <is>
-          <t>Aegir</t>
+          <t>Throttur Reykjavik</t>
         </is>
       </c>
       <c r="K6" t="inlineStr">
         <is>
-          <t>Njardvik</t>
+          <t>Afturelding Mosfellsbaer</t>
         </is>
       </c>
       <c r="L6" t="inlineStr">
         <is>
-          <t>0xde9c2677ae0e84c01c06a23050c75f29399db6bd766b2ef90484b73f8e0bbaed</t>
+          <t>0x7a5019973da533d172cf682264ba4b7ae8b6e65bb7591585a6fce73a807f64b0</t>
         </is>
       </c>
       <c r="M6" t="inlineStr">
         <is>
-          <t>L19548408</t>
+          <t>L19558554</t>
         </is>
       </c>
       <c r="N6" t="inlineStr">
@@ -1056,17 +1064,17 @@
       </c>
       <c r="R6" t="inlineStr">
         <is>
-          <t>1785237449</t>
+          <t>1785267742</t>
         </is>
       </c>
       <c r="S6" t="inlineStr">
         <is>
-          <t>1785266100</t>
+          <t>1785352500</t>
         </is>
       </c>
       <c r="T6" t="inlineStr">
         <is>
-          <t>20.748249</t>
+          <t>2.850123</t>
         </is>
       </c>
       <c r="U6" t="inlineStr">
@@ -1083,31 +1091,39 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>0xce612ac2221331f875649902eb6a0cde4b9db2f0f597bbc86e7caced63d25b99</t>
+          <t>0x4c622a3a303c2e364803ca8b5f2417b149396b0a5a454b59e42697e254ae9315</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>0x97EC1C9682F70091efB04e97b0B34698cF815EE1</t>
-        </is>
-      </c>
-      <c r="C7" t="inlineStr"/>
+          <t>0x5A76a26f838Ff5430Fd53E61CD8Bd76D895c946E</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>11.73</t>
+          <t>1.45</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>1.4412</t>
+          <t>1.5088</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>Under/Over (3.5)</t>
-        </is>
-      </c>
-      <c r="G7" t="inlineStr"/>
+          <t>1X2</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>Throttur Reykjavik</t>
+        </is>
+      </c>
       <c r="H7" t="inlineStr">
         <is>
           <t>Besta Deild Karla</t>
@@ -1115,27 +1131,27 @@
       </c>
       <c r="I7" t="inlineStr">
         <is>
-          <t>Aegir vs Njardvik</t>
+          <t>Throttur Reykjavik vs Afturelding Mosfellsbaer</t>
         </is>
       </c>
       <c r="J7" t="inlineStr">
         <is>
-          <t>Aegir</t>
+          <t>Throttur Reykjavik</t>
         </is>
       </c>
       <c r="K7" t="inlineStr">
         <is>
-          <t>Njardvik</t>
+          <t>Afturelding Mosfellsbaer</t>
         </is>
       </c>
       <c r="L7" t="inlineStr">
         <is>
-          <t>0x0825c99784fd72c055ffaeeb62e8e792f152ccd5a39c675722acf968b754f571</t>
+          <t>0x7a5019973da533d172cf682264ba4b7ae8b6e65bb7591585a6fce73a807f64b0</t>
         </is>
       </c>
       <c r="M7" t="inlineStr">
         <is>
-          <t>L19548408</t>
+          <t>L19558554</t>
         </is>
       </c>
       <c r="N7" t="inlineStr">
@@ -1160,17 +1176,17 @@
       </c>
       <c r="R7" t="inlineStr">
         <is>
-          <t>1785236520</t>
+          <t>1785267709</t>
         </is>
       </c>
       <c r="S7" t="inlineStr">
         <is>
-          <t>1785266100</t>
+          <t>1785352500</t>
         </is>
       </c>
       <c r="T7" t="inlineStr">
         <is>
-          <t>26.583569</t>
+          <t>2.850123</t>
         </is>
       </c>
       <c r="U7" t="inlineStr">
@@ -1187,23 +1203,23 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>0x7ae96391e38cfe39539922631da2025b36f57f1831d5f35ec6338463f27cb2a2</t>
+          <t>0x79c1f616b380c93f42fe785c942a2cc39edc55c4cdd4d5b6a09024c926a74f60</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>0x5D69C3af95Ff47088b415B25F41b1fFDc8571063</t>
+          <t>0x97EC1C9682F70091efB04e97b0B34698cF815EE1</t>
         </is>
       </c>
       <c r="C8" t="inlineStr"/>
       <c r="D8" t="inlineStr">
         <is>
-          <t>1.03</t>
+          <t>11.22999</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>1.5525</t>
+          <t>1.5413</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
@@ -1264,7 +1280,7 @@
       </c>
       <c r="R8" t="inlineStr">
         <is>
-          <t>1785236069</t>
+          <t>1785237449</t>
         </is>
       </c>
       <c r="S8" t="inlineStr">
@@ -1274,7 +1290,7 @@
       </c>
       <c r="T8" t="inlineStr">
         <is>
-          <t>1.864253</t>
+          <t>20.748249</t>
         </is>
       </c>
       <c r="U8" t="inlineStr">
@@ -1291,7 +1307,7 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>0xc979cd389b2d4ca831b9a44b7738a2ae46abf46b1bd95d0fbe5b654a09413b1e</t>
+          <t>0xce612ac2221331f875649902eb6a0cde4b9db2f0f597bbc86e7caced63d25b99</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
@@ -1302,12 +1318,12 @@
       <c r="C9" t="inlineStr"/>
       <c r="D9" t="inlineStr">
         <is>
-          <t>5.59</t>
+          <t>11.73</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>1.4525</t>
+          <t>1.4412</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
@@ -1368,7 +1384,7 @@
       </c>
       <c r="R9" t="inlineStr">
         <is>
-          <t>1785235526</t>
+          <t>1785236520</t>
         </is>
       </c>
       <c r="S9" t="inlineStr">
@@ -1378,7 +1394,7 @@
       </c>
       <c r="T9" t="inlineStr">
         <is>
-          <t>12.353591</t>
+          <t>26.583569</t>
         </is>
       </c>
       <c r="U9" t="inlineStr">
@@ -1395,30 +1411,30 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>0x65bc0b70a6148d6f136b1552723c33dcf058e2ee7e6097ad6d18a39367f4821b</t>
+          <t>0x7ae96391e38cfe39539922631da2025b36f57f1831d5f35ec6338463f27cb2a2</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>0x4a09916b1325Eed50eE8973B13742a205B0B7c7E</t>
-        </is>
-      </c>
-      <c r="C10" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
+          <t>0x5D69C3af95Ff47088b415B25F41b1fFDc8571063</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr"/>
       <c r="D10" t="inlineStr">
         <is>
-          <t>35.0</t>
+          <t>1.03</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>1.5987</t>
-        </is>
-      </c>
-      <c r="F10" t="inlineStr"/>
+          <t>1.5525</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>Under/Over (4)</t>
+        </is>
+      </c>
       <c r="G10" t="inlineStr"/>
       <c r="H10" t="inlineStr">
         <is>
@@ -1427,32 +1443,32 @@
       </c>
       <c r="I10" t="inlineStr">
         <is>
-          <t>IR Reykjavik vs Fylkir</t>
+          <t>Aegir vs Njardvik</t>
         </is>
       </c>
       <c r="J10" t="inlineStr">
         <is>
-          <t>IR Reykjavik</t>
+          <t>Aegir</t>
         </is>
       </c>
       <c r="K10" t="inlineStr">
         <is>
-          <t>Fylkir</t>
+          <t>Njardvik</t>
         </is>
       </c>
       <c r="L10" t="inlineStr">
         <is>
-          <t>0xef2cff3047642c7d3f79713526decc2ed1438c01d374590eb62929362f824801</t>
+          <t>0xde9c2677ae0e84c01c06a23050c75f29399db6bd766b2ef90484b73f8e0bbaed</t>
         </is>
       </c>
       <c r="M10" t="inlineStr">
         <is>
-          <t>L19520873</t>
+          <t>L19548408</t>
         </is>
       </c>
       <c r="N10" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>0</t>
         </is>
       </c>
       <c r="O10" t="inlineStr">
@@ -1472,17 +1488,17 @@
       </c>
       <c r="R10" t="inlineStr">
         <is>
-          <t>1784987195</t>
+          <t>1785236069</t>
         </is>
       </c>
       <c r="S10" t="inlineStr">
         <is>
-          <t>1784988000</t>
+          <t>1785266100</t>
         </is>
       </c>
       <c r="T10" t="inlineStr">
         <is>
-          <t>59.090338</t>
+          <t>1.864253</t>
         </is>
       </c>
       <c r="U10" t="inlineStr">
@@ -1490,35 +1506,39 @@
           <t>SXR</t>
         </is>
       </c>
-      <c r="V10" t="inlineStr"/>
+      <c r="V10" t="inlineStr">
+        <is>
+          <t>0x6629Ce1Cf35Cc1329ebB4F63202F3f197b3F050B</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>0xd5e3b95bd82e0d7627a9203f0fe8fdd3b068e15fd373a543e05b207e66faf2a0</t>
+          <t>0xc979cd389b2d4ca831b9a44b7738a2ae46abf46b1bd95d0fbe5b654a09413b1e</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>0x68E1818FF20BBe84F9be9E0A4A395FB11079Bd35</t>
-        </is>
-      </c>
-      <c r="C11" t="inlineStr">
-        <is>
-          <t>2</t>
-        </is>
-      </c>
+          <t>0x97EC1C9682F70091efB04e97b0B34698cF815EE1</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr"/>
       <c r="D11" t="inlineStr">
         <is>
-          <t>12.0</t>
+          <t>5.59</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>1.7862</t>
-        </is>
-      </c>
-      <c r="F11" t="inlineStr"/>
+          <t>1.4525</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>Under/Over (3.5)</t>
+        </is>
+      </c>
       <c r="G11" t="inlineStr"/>
       <c r="H11" t="inlineStr">
         <is>
@@ -1527,32 +1547,32 @@
       </c>
       <c r="I11" t="inlineStr">
         <is>
-          <t>IR Reykjavik vs Fylkir</t>
+          <t>Aegir vs Njardvik</t>
         </is>
       </c>
       <c r="J11" t="inlineStr">
         <is>
-          <t>IR Reykjavik</t>
+          <t>Aegir</t>
         </is>
       </c>
       <c r="K11" t="inlineStr">
         <is>
-          <t>Fylkir</t>
+          <t>Njardvik</t>
         </is>
       </c>
       <c r="L11" t="inlineStr">
         <is>
-          <t>0x2b00f05607bf61216841f59440e877cc0eeb424e834132492c721bd4faedc556</t>
+          <t>0x0825c99784fd72c055ffaeeb62e8e792f152ccd5a39c675722acf968b754f571</t>
         </is>
       </c>
       <c r="M11" t="inlineStr">
         <is>
-          <t>L19520873</t>
+          <t>L19548408</t>
         </is>
       </c>
       <c r="N11" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>0</t>
         </is>
       </c>
       <c r="O11" t="inlineStr">
@@ -1572,17 +1592,17 @@
       </c>
       <c r="R11" t="inlineStr">
         <is>
-          <t>1784986980</t>
+          <t>1785235526</t>
         </is>
       </c>
       <c r="S11" t="inlineStr">
         <is>
-          <t>1784988000</t>
+          <t>1785266100</t>
         </is>
       </c>
       <c r="T11" t="inlineStr">
         <is>
-          <t>16.327479</t>
+          <t>12.353591</t>
         </is>
       </c>
       <c r="U11" t="inlineStr">
@@ -1590,32 +1610,36 @@
           <t>SXR</t>
         </is>
       </c>
-      <c r="V11" t="inlineStr"/>
+      <c r="V11" t="inlineStr">
+        <is>
+          <t>0x6629Ce1Cf35Cc1329ebB4F63202F3f197b3F050B</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>0xbfc0a906e601c3195b374e6d33b07e4c0b0dcbf09e05e45b8bd53226678d5d88</t>
+          <t>0x65bc0b70a6148d6f136b1552723c33dcf058e2ee7e6097ad6d18a39367f4821b</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>0x68E1818FF20BBe84F9be9E0A4A395FB11079Bd35</t>
+          <t>0x4a09916b1325Eed50eE8973B13742a205B0B7c7E</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>1</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>37.0</t>
+          <t>35.0</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>1.7875</t>
+          <t>1.5987</t>
         </is>
       </c>
       <c r="F12" t="inlineStr"/>
@@ -1642,7 +1666,7 @@
       </c>
       <c r="L12" t="inlineStr">
         <is>
-          <t>0x2b00f05607bf61216841f59440e877cc0eeb424e834132492c721bd4faedc556</t>
+          <t>0xef2cff3047642c7d3f79713526decc2ed1438c01d374590eb62929362f824801</t>
         </is>
       </c>
       <c r="M12" t="inlineStr">
@@ -1672,7 +1696,7 @@
       </c>
       <c r="R12" t="inlineStr">
         <is>
-          <t>1784986980</t>
+          <t>1784987195</t>
         </is>
       </c>
       <c r="S12" t="inlineStr">
@@ -1682,7 +1706,7 @@
       </c>
       <c r="T12" t="inlineStr">
         <is>
-          <t>47.105879</t>
+          <t>59.090338</t>
         </is>
       </c>
       <c r="U12" t="inlineStr">
@@ -1695,27 +1719,27 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>0x5724a3badfc2012619fbf8e1a14ab0e7f4c66de896315371280c186505e86b85</t>
+          <t>0xd5e3b95bd82e0d7627a9203f0fe8fdd3b068e15fd373a543e05b207e66faf2a0</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>0xe2C68b7ef85645e47F9b94382c3Db59b046945a2</t>
+          <t>0x68E1818FF20BBe84F9be9E0A4A395FB11079Bd35</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>69.0</t>
+          <t>12.0</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>1.6012</t>
+          <t>1.7862</t>
         </is>
       </c>
       <c r="F13" t="inlineStr"/>
@@ -1742,7 +1766,7 @@
       </c>
       <c r="L13" t="inlineStr">
         <is>
-          <t>0x04fd78e33c10fb928e409323c26948f49fe4c81fcd47748d9153c9c611b38d0b</t>
+          <t>0x2b00f05607bf61216841f59440e877cc0eeb424e834132492c721bd4faedc556</t>
         </is>
       </c>
       <c r="M13" t="inlineStr">
@@ -1772,7 +1796,7 @@
       </c>
       <c r="R13" t="inlineStr">
         <is>
-          <t>1784986978</t>
+          <t>1784986980</t>
         </is>
       </c>
       <c r="S13" t="inlineStr">
@@ -1782,7 +1806,7 @@
       </c>
       <c r="T13" t="inlineStr">
         <is>
-          <t>114.884008</t>
+          <t>16.327479</t>
         </is>
       </c>
       <c r="U13" t="inlineStr">
@@ -1795,27 +1819,27 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>0xf825a9ec3149d5a232253fd07078e2ed75a62b287df75e59fbb6c1546f6912a3</t>
+          <t>0xbfc0a906e601c3195b374e6d33b07e4c0b0dcbf09e05e45b8bd53226678d5d88</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>0x4a09916b1325Eed50eE8973B13742a205B0B7c7E</t>
+          <t>0x68E1818FF20BBe84F9be9E0A4A395FB11079Bd35</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>15.0</t>
+          <t>37.0</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>1.2712</t>
+          <t>1.7875</t>
         </is>
       </c>
       <c r="F14" t="inlineStr"/>
@@ -1842,7 +1866,7 @@
       </c>
       <c r="L14" t="inlineStr">
         <is>
-          <t>0x06a233f1b733d63cee459a37ac1beffad92b8f9ec21c414e0c26e2876b05eebd</t>
+          <t>0x2b00f05607bf61216841f59440e877cc0eeb424e834132492c721bd4faedc556</t>
         </is>
       </c>
       <c r="M14" t="inlineStr">
@@ -1872,7 +1896,7 @@
       </c>
       <c r="R14" t="inlineStr">
         <is>
-          <t>1784984833</t>
+          <t>1784986980</t>
         </is>
       </c>
       <c r="S14" t="inlineStr">
@@ -1882,7 +1906,7 @@
       </c>
       <c r="T14" t="inlineStr">
         <is>
-          <t>58.211982</t>
+          <t>47.105879</t>
         </is>
       </c>
       <c r="U14" t="inlineStr">
@@ -1895,27 +1919,27 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>0x832d570bfcb61240d74893710e1758118ea62888a2bf55921f3190b9a71f4561</t>
+          <t>0x5724a3badfc2012619fbf8e1a14ab0e7f4c66de896315371280c186505e86b85</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>0x68E1818FF20BBe84F9be9E0A4A395FB11079Bd35</t>
+          <t>0xe2C68b7ef85645e47F9b94382c3Db59b046945a2</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>1</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>3.0</t>
+          <t>69.0</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>1.7887</t>
+          <t>1.6012</t>
         </is>
       </c>
       <c r="F15" t="inlineStr"/>
@@ -1942,7 +1966,7 @@
       </c>
       <c r="L15" t="inlineStr">
         <is>
-          <t>0x91a9ea8ebfd8b049218a8e072590d2f657e26fdb1f2a49b1016ae42171c68ef2</t>
+          <t>0x04fd78e33c10fb928e409323c26948f49fe4c81fcd47748d9153c9c611b38d0b</t>
         </is>
       </c>
       <c r="M15" t="inlineStr">
@@ -1972,7 +1996,7 @@
       </c>
       <c r="R15" t="inlineStr">
         <is>
-          <t>1784984812</t>
+          <t>1784986978</t>
         </is>
       </c>
       <c r="S15" t="inlineStr">
@@ -1982,7 +2006,7 @@
       </c>
       <c r="T15" t="inlineStr">
         <is>
-          <t>4.733718</t>
+          <t>114.884008</t>
         </is>
       </c>
       <c r="U15" t="inlineStr">
@@ -1995,27 +2019,27 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>0x78e73a1fbc4bce58e1469ba84a7a75afedee1c817a9927ff72cae6f55f5b4a58</t>
+          <t>0xf825a9ec3149d5a232253fd07078e2ed75a62b287df75e59fbb6c1546f6912a3</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>0x68E1818FF20BBe84F9be9E0A4A395FB11079Bd35</t>
+          <t>0x4a09916b1325Eed50eE8973B13742a205B0B7c7E</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>1</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>8.0</t>
+          <t>15.0</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>1.7887</t>
+          <t>1.2712</t>
         </is>
       </c>
       <c r="F16" t="inlineStr"/>
@@ -2042,7 +2066,7 @@
       </c>
       <c r="L16" t="inlineStr">
         <is>
-          <t>0x91a9ea8ebfd8b049218a8e072590d2f657e26fdb1f2a49b1016ae42171c68ef2</t>
+          <t>0x06a233f1b733d63cee459a37ac1beffad92b8f9ec21c414e0c26e2876b05eebd</t>
         </is>
       </c>
       <c r="M16" t="inlineStr">
@@ -2072,7 +2096,7 @@
       </c>
       <c r="R16" t="inlineStr">
         <is>
-          <t>1784984812</t>
+          <t>1784984833</t>
         </is>
       </c>
       <c r="S16" t="inlineStr">
@@ -2082,7 +2106,7 @@
       </c>
       <c r="T16" t="inlineStr">
         <is>
-          <t>10.745559</t>
+          <t>58.211982</t>
         </is>
       </c>
       <c r="U16" t="inlineStr">
@@ -2095,7 +2119,7 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>0x02053d570c2ec6485bf734b3e9d25cb6962b678b5212cc142c9b62d371752a01</t>
+          <t>0x832d570bfcb61240d74893710e1758118ea62888a2bf55921f3190b9a71f4561</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
@@ -2105,17 +2129,17 @@
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>13.0</t>
+          <t>3.0</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>1.5737</t>
+          <t>1.7887</t>
         </is>
       </c>
       <c r="F17" t="inlineStr"/>
@@ -2142,7 +2166,7 @@
       </c>
       <c r="L17" t="inlineStr">
         <is>
-          <t>0x04fd78e33c10fb928e409323c26948f49fe4c81fcd47748d9153c9c611b38d0b</t>
+          <t>0x91a9ea8ebfd8b049218a8e072590d2f657e26fdb1f2a49b1016ae42171c68ef2</t>
         </is>
       </c>
       <c r="M17" t="inlineStr">
@@ -2182,7 +2206,7 @@
       </c>
       <c r="T17" t="inlineStr">
         <is>
-          <t>23.46041</t>
+          <t>4.733718</t>
         </is>
       </c>
       <c r="U17" t="inlineStr">
@@ -2195,27 +2219,27 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>0x6c8964e487e133d59a699205a9a6514d54217a61ad5ca3887aa005a89c8cbdfa</t>
+          <t>0x78e73a1fbc4bce58e1469ba84a7a75afedee1c817a9927ff72cae6f55f5b4a58</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>0x4a09916b1325Eed50eE8973B13742a205B0B7c7E</t>
+          <t>0x68E1818FF20BBe84F9be9E0A4A395FB11079Bd35</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>15.0</t>
+          <t>8.0</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>1.2712</t>
+          <t>1.7887</t>
         </is>
       </c>
       <c r="F18" t="inlineStr"/>
@@ -2242,7 +2266,7 @@
       </c>
       <c r="L18" t="inlineStr">
         <is>
-          <t>0x06a233f1b733d63cee459a37ac1beffad92b8f9ec21c414e0c26e2876b05eebd</t>
+          <t>0x91a9ea8ebfd8b049218a8e072590d2f657e26fdb1f2a49b1016ae42171c68ef2</t>
         </is>
       </c>
       <c r="M18" t="inlineStr">
@@ -2272,7 +2296,7 @@
       </c>
       <c r="R18" t="inlineStr">
         <is>
-          <t>1784984810</t>
+          <t>1784984812</t>
         </is>
       </c>
       <c r="S18" t="inlineStr">
@@ -2282,7 +2306,7 @@
       </c>
       <c r="T18" t="inlineStr">
         <is>
-          <t>58.209253</t>
+          <t>10.745559</t>
         </is>
       </c>
       <c r="U18" t="inlineStr">
@@ -2295,12 +2319,12 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>0xb8b680dda4305fed43c95dc6dbc059c9678abe5f31da65b83ac57ecd5c8d3903</t>
+          <t>0x02053d570c2ec6485bf734b3e9d25cb6962b678b5212cc142c9b62d371752a01</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>0x4a09916b1325Eed50eE8973B13742a205B0B7c7E</t>
+          <t>0x68E1818FF20BBe84F9be9E0A4A395FB11079Bd35</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
@@ -2310,12 +2334,12 @@
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>16.0</t>
+          <t>13.0</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>1.2712</t>
+          <t>1.5737</t>
         </is>
       </c>
       <c r="F19" t="inlineStr"/>
@@ -2342,7 +2366,7 @@
       </c>
       <c r="L19" t="inlineStr">
         <is>
-          <t>0x06a233f1b733d63cee459a37ac1beffad92b8f9ec21c414e0c26e2876b05eebd</t>
+          <t>0x04fd78e33c10fb928e409323c26948f49fe4c81fcd47748d9153c9c611b38d0b</t>
         </is>
       </c>
       <c r="M19" t="inlineStr">
@@ -2372,7 +2396,7 @@
       </c>
       <c r="R19" t="inlineStr">
         <is>
-          <t>1784984670</t>
+          <t>1784984812</t>
         </is>
       </c>
       <c r="S19" t="inlineStr">
@@ -2382,7 +2406,7 @@
       </c>
       <c r="T19" t="inlineStr">
         <is>
-          <t>60.198968</t>
+          <t>23.46041</t>
         </is>
       </c>
       <c r="U19" t="inlineStr">
@@ -2395,7 +2419,7 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>0x374cde0708e064be0b99fea4bb71434540b7ca7bbd1a444cb12a8b14c6aa3c48</t>
+          <t>0x6c8964e487e133d59a699205a9a6514d54217a61ad5ca3887aa005a89c8cbdfa</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
@@ -2410,7 +2434,7 @@
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>16.0</t>
+          <t>15.0</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
@@ -2472,7 +2496,7 @@
       </c>
       <c r="R20" t="inlineStr">
         <is>
-          <t>1784984617</t>
+          <t>1784984810</t>
         </is>
       </c>
       <c r="S20" t="inlineStr">
@@ -2482,7 +2506,7 @@
       </c>
       <c r="T20" t="inlineStr">
         <is>
-          <t>60.198968</t>
+          <t>58.209253</t>
         </is>
       </c>
       <c r="U20" t="inlineStr">
@@ -2495,7 +2519,7 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>0x4c094ddc4f89a7cbd768baf6a26f7e686ead028a4b15ee75fd8f4927e1ad7989</t>
+          <t>0xb8b680dda4305fed43c95dc6dbc059c9678abe5f31da65b83ac57ecd5c8d3903</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
@@ -2572,7 +2596,7 @@
       </c>
       <c r="R21" t="inlineStr">
         <is>
-          <t>1784984581</t>
+          <t>1784984670</t>
         </is>
       </c>
       <c r="S21" t="inlineStr">
@@ -2595,7 +2619,7 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>0x7dd8d48e4f9e00707e79d58d5900292571189d9de19bd23c6c6a9a433ea96f72</t>
+          <t>0x374cde0708e064be0b99fea4bb71434540b7ca7bbd1a444cb12a8b14c6aa3c48</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
@@ -2672,7 +2696,7 @@
       </c>
       <c r="R22" t="inlineStr">
         <is>
-          <t>1784984563</t>
+          <t>1784984617</t>
         </is>
       </c>
       <c r="S22" t="inlineStr">
@@ -2695,7 +2719,7 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>0x7354c940dd56ae7caca9fa9b1a548dcf53e1a3516f531216c677cf582affb4fe</t>
+          <t>0x4c094ddc4f89a7cbd768baf6a26f7e686ead028a4b15ee75fd8f4927e1ad7989</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
@@ -2710,12 +2734,12 @@
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>9.0</t>
+          <t>16.0</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>1.3013</t>
+          <t>1.2712</t>
         </is>
       </c>
       <c r="F23" t="inlineStr"/>
@@ -2772,7 +2796,7 @@
       </c>
       <c r="R23" t="inlineStr">
         <is>
-          <t>1784984538</t>
+          <t>1784984581</t>
         </is>
       </c>
       <c r="S23" t="inlineStr">
@@ -2782,7 +2806,7 @@
       </c>
       <c r="T23" t="inlineStr">
         <is>
-          <t>31.184232</t>
+          <t>60.198968</t>
         </is>
       </c>
       <c r="U23" t="inlineStr">
@@ -2795,12 +2819,12 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>0xdc3c1508859b265a9cc7ea3dadc58bb672f939bf46cde2c06081ec2891a03946</t>
+          <t>0x7dd8d48e4f9e00707e79d58d5900292571189d9de19bd23c6c6a9a433ea96f72</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>0xC88F614A48f8A705d7465b03aAF62ddaca0c3754</t>
+          <t>0x4a09916b1325Eed50eE8973B13742a205B0B7c7E</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
@@ -2810,12 +2834,12 @@
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>21.0</t>
+          <t>16.0</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>1.4363</t>
+          <t>1.2712</t>
         </is>
       </c>
       <c r="F24" t="inlineStr"/>
@@ -2842,7 +2866,7 @@
       </c>
       <c r="L24" t="inlineStr">
         <is>
-          <t>0xd5ae8f2322bcc6adaca1c1bb1baf6a74afa50cc30131840c87632f67865c23d0</t>
+          <t>0x06a233f1b733d63cee459a37ac1beffad92b8f9ec21c414e0c26e2876b05eebd</t>
         </is>
       </c>
       <c r="M24" t="inlineStr">
@@ -2872,7 +2896,7 @@
       </c>
       <c r="R24" t="inlineStr">
         <is>
-          <t>1784984537</t>
+          <t>1784984563</t>
         </is>
       </c>
       <c r="S24" t="inlineStr">
@@ -2882,7 +2906,7 @@
       </c>
       <c r="T24" t="inlineStr">
         <is>
-          <t>48.297994</t>
+          <t>60.198968</t>
         </is>
       </c>
       <c r="U24" t="inlineStr">
@@ -2895,12 +2919,12 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>0x0bf6c8f6ea5d7452bf543eb72d99a66c1b6ff74a5e56b4ad9449b6870f225d2d</t>
+          <t>0x7354c940dd56ae7caca9fa9b1a548dcf53e1a3516f531216c677cf582affb4fe</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>0x47D0CE9b8d653c8884DB7E2a7F88d4849E0CD980</t>
+          <t>0x4a09916b1325Eed50eE8973B13742a205B0B7c7E</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
@@ -2910,12 +2934,12 @@
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>38.0</t>
+          <t>9.0</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>1.5537</t>
+          <t>1.3013</t>
         </is>
       </c>
       <c r="F25" t="inlineStr"/>
@@ -2942,7 +2966,7 @@
       </c>
       <c r="L25" t="inlineStr">
         <is>
-          <t>0x04fd78e33c10fb928e409323c26948f49fe4c81fcd47748d9153c9c611b38d0b</t>
+          <t>0x06a233f1b733d63cee459a37ac1beffad92b8f9ec21c414e0c26e2876b05eebd</t>
         </is>
       </c>
       <c r="M25" t="inlineStr">
@@ -2972,7 +2996,7 @@
       </c>
       <c r="R25" t="inlineStr">
         <is>
-          <t>1784984536</t>
+          <t>1784984538</t>
         </is>
       </c>
       <c r="S25" t="inlineStr">
@@ -2982,7 +3006,7 @@
       </c>
       <c r="T25" t="inlineStr">
         <is>
-          <t>68.833427</t>
+          <t>31.184232</t>
         </is>
       </c>
       <c r="U25" t="inlineStr">
@@ -2995,12 +3019,12 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>0xa4b5b4c3c3766e7d708b5373412745aa0b0d5f4c097f5451a2210d6d019269c6</t>
+          <t>0xdc3c1508859b265a9cc7ea3dadc58bb672f939bf46cde2c06081ec2891a03946</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>0x47D0CE9b8d653c8884DB7E2a7F88d4849E0CD980</t>
+          <t>0xC88F614A48f8A705d7465b03aAF62ddaca0c3754</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
@@ -3010,12 +3034,12 @@
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>29.0</t>
+          <t>21.0</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>1.5537</t>
+          <t>1.4363</t>
         </is>
       </c>
       <c r="F26" t="inlineStr"/>
@@ -3042,7 +3066,7 @@
       </c>
       <c r="L26" t="inlineStr">
         <is>
-          <t>0x04fd78e33c10fb928e409323c26948f49fe4c81fcd47748d9153c9c611b38d0b</t>
+          <t>0xd5ae8f2322bcc6adaca1c1bb1baf6a74afa50cc30131840c87632f67865c23d0</t>
         </is>
       </c>
       <c r="M26" t="inlineStr">
@@ -3072,7 +3096,7 @@
       </c>
       <c r="R26" t="inlineStr">
         <is>
-          <t>1784984502</t>
+          <t>1784984537</t>
         </is>
       </c>
       <c r="S26" t="inlineStr">
@@ -3082,7 +3106,7 @@
       </c>
       <c r="T26" t="inlineStr">
         <is>
-          <t>53.355738</t>
+          <t>48.297994</t>
         </is>
       </c>
       <c r="U26" t="inlineStr">
@@ -3095,7 +3119,7 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>0xfac3960037b540d1b0b49f14ff5313d7db5bd6320c356e510ef3e6bdaca6d1ff</t>
+          <t>0x0bf6c8f6ea5d7452bf543eb72d99a66c1b6ff74a5e56b4ad9449b6870f225d2d</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
@@ -3110,7 +3134,7 @@
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>25.0</t>
+          <t>38.0</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
@@ -3172,7 +3196,7 @@
       </c>
       <c r="R27" t="inlineStr">
         <is>
-          <t>1784984501</t>
+          <t>1784984536</t>
         </is>
       </c>
       <c r="S27" t="inlineStr">
@@ -3182,7 +3206,7 @@
       </c>
       <c r="T27" t="inlineStr">
         <is>
-          <t>46.408957</t>
+          <t>68.833427</t>
         </is>
       </c>
       <c r="U27" t="inlineStr">
@@ -3195,12 +3219,12 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>0xf3b65016998beda20548812c7503abc20be0fa3abedc59c3ac7e08e6b82c70f1</t>
+          <t>0xa4b5b4c3c3766e7d708b5373412745aa0b0d5f4c097f5451a2210d6d019269c6</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>0x4a09916b1325Eed50eE8973B13742a205B0B7c7E</t>
+          <t>0x47D0CE9b8d653c8884DB7E2a7F88d4849E0CD980</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
@@ -3210,12 +3234,12 @@
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>6.0</t>
+          <t>29.0</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>1.3013</t>
+          <t>1.5537</t>
         </is>
       </c>
       <c r="F28" t="inlineStr"/>
@@ -3242,7 +3266,7 @@
       </c>
       <c r="L28" t="inlineStr">
         <is>
-          <t>0x06a233f1b733d63cee459a37ac1beffad92b8f9ec21c414e0c26e2876b05eebd</t>
+          <t>0x04fd78e33c10fb928e409323c26948f49fe4c81fcd47748d9153c9c611b38d0b</t>
         </is>
       </c>
       <c r="M28" t="inlineStr">
@@ -3272,7 +3296,7 @@
       </c>
       <c r="R28" t="inlineStr">
         <is>
-          <t>1784984431</t>
+          <t>1784984502</t>
         </is>
       </c>
       <c r="S28" t="inlineStr">
@@ -3282,7 +3306,7 @@
       </c>
       <c r="T28" t="inlineStr">
         <is>
-          <t>22.912332</t>
+          <t>53.355738</t>
         </is>
       </c>
       <c r="U28" t="inlineStr">
@@ -3295,12 +3319,12 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>0xa04fcfb1b689fd17d1c3c66ac2ed73a6e0b99d30bdfd296529ca6549b4642440</t>
+          <t>0xfac3960037b540d1b0b49f14ff5313d7db5bd6320c356e510ef3e6bdaca6d1ff</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>0x4a09916b1325Eed50eE8973B13742a205B0B7c7E</t>
+          <t>0x47D0CE9b8d653c8884DB7E2a7F88d4849E0CD980</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
@@ -3310,12 +3334,12 @@
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>27.0</t>
+          <t>25.0</t>
         </is>
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>1.4537</t>
+          <t>1.5537</t>
         </is>
       </c>
       <c r="F29" t="inlineStr"/>
@@ -3342,7 +3366,7 @@
       </c>
       <c r="L29" t="inlineStr">
         <is>
-          <t>0xd5ae8f2322bcc6adaca1c1bb1baf6a74afa50cc30131840c87632f67865c23d0</t>
+          <t>0x04fd78e33c10fb928e409323c26948f49fe4c81fcd47748d9153c9c611b38d0b</t>
         </is>
       </c>
       <c r="M29" t="inlineStr">
@@ -3372,7 +3396,7 @@
       </c>
       <c r="R29" t="inlineStr">
         <is>
-          <t>1784984405</t>
+          <t>1784984501</t>
         </is>
       </c>
       <c r="S29" t="inlineStr">
@@ -3382,7 +3406,7 @@
       </c>
       <c r="T29" t="inlineStr">
         <is>
-          <t>60.187328</t>
+          <t>46.408957</t>
         </is>
       </c>
       <c r="U29" t="inlineStr">
@@ -3395,7 +3419,7 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>0xb07983b62c387b953f021bde51a561f510162701d56466ec78a20a598c01d8c4</t>
+          <t>0xf3b65016998beda20548812c7503abc20be0fa3abedc59c3ac7e08e6b82c70f1</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
@@ -3410,12 +3434,12 @@
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>35.0</t>
+          <t>6.0</t>
         </is>
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>1.595</t>
+          <t>1.3013</t>
         </is>
       </c>
       <c r="F30" t="inlineStr"/>
@@ -3442,7 +3466,7 @@
       </c>
       <c r="L30" t="inlineStr">
         <is>
-          <t>0xe1204c11efd43d8d3a0377591c468bba3ac169f58ab541c6d60665f2e0bbb051</t>
+          <t>0x06a233f1b733d63cee459a37ac1beffad92b8f9ec21c414e0c26e2876b05eebd</t>
         </is>
       </c>
       <c r="M30" t="inlineStr">
@@ -3472,7 +3496,7 @@
       </c>
       <c r="R30" t="inlineStr">
         <is>
-          <t>1784984404</t>
+          <t>1784984431</t>
         </is>
       </c>
       <c r="S30" t="inlineStr">
@@ -3482,7 +3506,7 @@
       </c>
       <c r="T30" t="inlineStr">
         <is>
-          <t>60.197529</t>
+          <t>22.912332</t>
         </is>
       </c>
       <c r="U30" t="inlineStr">
@@ -3495,27 +3519,27 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>0xc41db21ce0b5921299bba16424467dff9a9a6eb4d744a5aadf04422f8138f34f</t>
+          <t>0xa04fcfb1b689fd17d1c3c66ac2ed73a6e0b99d30bdfd296529ca6549b4642440</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>0x68E1818FF20BBe84F9be9E0A4A395FB11079Bd35</t>
+          <t>0x4a09916b1325Eed50eE8973B13742a205B0B7c7E</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>1</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>22.0</t>
+          <t>27.0</t>
         </is>
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>1.7712</t>
+          <t>1.4537</t>
         </is>
       </c>
       <c r="F31" t="inlineStr"/>
@@ -3542,7 +3566,7 @@
       </c>
       <c r="L31" t="inlineStr">
         <is>
-          <t>0x91a9ea8ebfd8b049218a8e072590d2f657e26fdb1f2a49b1016ae42171c68ef2</t>
+          <t>0xd5ae8f2322bcc6adaca1c1bb1baf6a74afa50cc30131840c87632f67865c23d0</t>
         </is>
       </c>
       <c r="M31" t="inlineStr">
@@ -3572,7 +3596,7 @@
       </c>
       <c r="R31" t="inlineStr">
         <is>
-          <t>1784984403</t>
+          <t>1784984405</t>
         </is>
       </c>
       <c r="S31" t="inlineStr">
@@ -3582,7 +3606,7 @@
       </c>
       <c r="T31" t="inlineStr">
         <is>
-          <t>29.185737</t>
+          <t>60.187328</t>
         </is>
       </c>
       <c r="U31" t="inlineStr">
@@ -3595,27 +3619,27 @@
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>0x97d57842a441d56ad4d0172a6e2460bdd3644bd55476d419863d144ec4fb3f02</t>
+          <t>0xb07983b62c387b953f021bde51a561f510162701d56466ec78a20a598c01d8c4</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>0x68E1818FF20BBe84F9be9E0A4A395FB11079Bd35</t>
+          <t>0x4a09916b1325Eed50eE8973B13742a205B0B7c7E</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>1</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>3.0</t>
+          <t>35.0</t>
         </is>
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>1.775</t>
+          <t>1.595</t>
         </is>
       </c>
       <c r="F32" t="inlineStr"/>
@@ -3642,7 +3666,7 @@
       </c>
       <c r="L32" t="inlineStr">
         <is>
-          <t>0x2b00f05607bf61216841f59440e877cc0eeb424e834132492c721bd4faedc556</t>
+          <t>0xe1204c11efd43d8d3a0377591c468bba3ac169f58ab541c6d60665f2e0bbb051</t>
         </is>
       </c>
       <c r="M32" t="inlineStr">
@@ -3672,7 +3696,7 @@
       </c>
       <c r="R32" t="inlineStr">
         <is>
-          <t>1784984403</t>
+          <t>1784984404</t>
         </is>
       </c>
       <c r="S32" t="inlineStr">
@@ -3682,7 +3706,7 @@
       </c>
       <c r="T32" t="inlineStr">
         <is>
-          <t>4.444439</t>
+          <t>60.197529</t>
         </is>
       </c>
       <c r="U32" t="inlineStr">
@@ -3695,27 +3719,27 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>0x54a44d2ce4be4b546daee52057d4611c0f1d29571a9747f66b3462780e888ae0</t>
+          <t>0xc41db21ce0b5921299bba16424467dff9a9a6eb4d744a5aadf04422f8138f34f</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>0x4a09916b1325Eed50eE8973B13742a205B0B7c7E</t>
+          <t>0x68E1818FF20BBe84F9be9E0A4A395FB11079Bd35</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>17.0</t>
+          <t>22.0</t>
         </is>
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>1.2988</t>
+          <t>1.7712</t>
         </is>
       </c>
       <c r="F33" t="inlineStr"/>
@@ -3742,7 +3766,7 @@
       </c>
       <c r="L33" t="inlineStr">
         <is>
-          <t>0x588a71865f90131e16b5b72dfef6ddb7cec8deb7df1f8102477a62eaa807cc71</t>
+          <t>0x91a9ea8ebfd8b049218a8e072590d2f657e26fdb1f2a49b1016ae42171c68ef2</t>
         </is>
       </c>
       <c r="M33" t="inlineStr">
@@ -3772,7 +3796,7 @@
       </c>
       <c r="R33" t="inlineStr">
         <is>
-          <t>1784984402</t>
+          <t>1784984403</t>
         </is>
       </c>
       <c r="S33" t="inlineStr">
@@ -3782,7 +3806,7 @@
       </c>
       <c r="T33" t="inlineStr">
         <is>
-          <t>60.178243</t>
+          <t>29.185737</t>
         </is>
       </c>
       <c r="U33" t="inlineStr">
@@ -3795,27 +3819,27 @@
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>0xf9d293335e6b1b3fd21eba9ec71cbbd6cbce398d5d606b38175d3776a077cb91</t>
+          <t>0x97d57842a441d56ad4d0172a6e2460bdd3644bd55476d419863d144ec4fb3f02</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>0x4a09916b1325Eed50eE8973B13742a205B0B7c7E</t>
+          <t>0x68E1818FF20BBe84F9be9E0A4A395FB11079Bd35</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>41.0</t>
+          <t>3.0</t>
         </is>
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t>1.685</t>
+          <t>1.775</t>
         </is>
       </c>
       <c r="F34" t="inlineStr"/>
@@ -3842,7 +3866,7 @@
       </c>
       <c r="L34" t="inlineStr">
         <is>
-          <t>0xaf0827308b557ecc964e4c608c6b71f345660fa965da2a0e02882ee62ce45e49</t>
+          <t>0x2b00f05607bf61216841f59440e877cc0eeb424e834132492c721bd4faedc556</t>
         </is>
       </c>
       <c r="M34" t="inlineStr">
@@ -3872,7 +3896,7 @@
       </c>
       <c r="R34" t="inlineStr">
         <is>
-          <t>1784984401</t>
+          <t>1784984403</t>
         </is>
       </c>
       <c r="S34" t="inlineStr">
@@ -3882,7 +3906,7 @@
       </c>
       <c r="T34" t="inlineStr">
         <is>
-          <t>60.189781</t>
+          <t>4.444439</t>
         </is>
       </c>
       <c r="U34" t="inlineStr">
@@ -3895,12 +3919,12 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>0x80f610f55e907d511b2c5a8d77d03f9aca143e4e50b6d7fba92997ba46481bde</t>
+          <t>0x54a44d2ce4be4b546daee52057d4611c0f1d29571a9747f66b3462780e888ae0</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>0x47D0CE9b8d653c8884DB7E2a7F88d4849E0CD980</t>
+          <t>0x4a09916b1325Eed50eE8973B13742a205B0B7c7E</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
@@ -3910,12 +3934,12 @@
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>6.0</t>
+          <t>17.0</t>
         </is>
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>1.5537</t>
+          <t>1.2988</t>
         </is>
       </c>
       <c r="F35" t="inlineStr"/>
@@ -3942,7 +3966,7 @@
       </c>
       <c r="L35" t="inlineStr">
         <is>
-          <t>0x04fd78e33c10fb928e409323c26948f49fe4c81fcd47748d9153c9c611b38d0b</t>
+          <t>0x588a71865f90131e16b5b72dfef6ddb7cec8deb7df1f8102477a62eaa807cc71</t>
         </is>
       </c>
       <c r="M35" t="inlineStr">
@@ -3972,7 +3996,7 @@
       </c>
       <c r="R35" t="inlineStr">
         <is>
-          <t>1784983849</t>
+          <t>1784984402</t>
         </is>
       </c>
       <c r="S35" t="inlineStr">
@@ -3982,7 +4006,7 @@
       </c>
       <c r="T35" t="inlineStr">
         <is>
-          <t>11.988786</t>
+          <t>60.178243</t>
         </is>
       </c>
       <c r="U35" t="inlineStr">
@@ -3995,12 +4019,12 @@
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>0x6e3d6f822ebfe70f563004b4a5a4a6303f1d1cb9677e6e3a56324cda8cc92ba7</t>
+          <t>0xf9d293335e6b1b3fd21eba9ec71cbbd6cbce398d5d606b38175d3776a077cb91</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>0x68E1818FF20BBe84F9be9E0A4A395FB11079Bd35</t>
+          <t>0x4a09916b1325Eed50eE8973B13742a205B0B7c7E</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
@@ -4010,12 +4034,12 @@
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>25.0</t>
+          <t>41.0</t>
         </is>
       </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t>1.5513</t>
+          <t>1.685</t>
         </is>
       </c>
       <c r="F36" t="inlineStr"/>
@@ -4042,7 +4066,7 @@
       </c>
       <c r="L36" t="inlineStr">
         <is>
-          <t>0x04fd78e33c10fb928e409323c26948f49fe4c81fcd47748d9153c9c611b38d0b</t>
+          <t>0xaf0827308b557ecc964e4c608c6b71f345660fa965da2a0e02882ee62ce45e49</t>
         </is>
       </c>
       <c r="M36" t="inlineStr">
@@ -4072,7 +4096,7 @@
       </c>
       <c r="R36" t="inlineStr">
         <is>
-          <t>1784983797</t>
+          <t>1784984401</t>
         </is>
       </c>
       <c r="S36" t="inlineStr">
@@ -4082,7 +4106,7 @@
       </c>
       <c r="T36" t="inlineStr">
         <is>
-          <t>46.150404</t>
+          <t>60.189781</t>
         </is>
       </c>
       <c r="U36" t="inlineStr">
@@ -4095,27 +4119,27 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>0xc913b7104d801ceb0283dc9eefcce577969c93f7b16c1cc5515036561b5b8d8e</t>
+          <t>0x80f610f55e907d511b2c5a8d77d03f9aca143e4e50b6d7fba92997ba46481bde</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>0x68E1818FF20BBe84F9be9E0A4A395FB11079Bd35</t>
+          <t>0x47D0CE9b8d653c8884DB7E2a7F88d4849E0CD980</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>1</t>
         </is>
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>4.0</t>
+          <t>6.0</t>
         </is>
       </c>
       <c r="E37" t="inlineStr">
         <is>
-          <t>1.7712</t>
+          <t>1.5537</t>
         </is>
       </c>
       <c r="F37" t="inlineStr"/>
@@ -4142,7 +4166,7 @@
       </c>
       <c r="L37" t="inlineStr">
         <is>
-          <t>0x91a9ea8ebfd8b049218a8e072590d2f657e26fdb1f2a49b1016ae42171c68ef2</t>
+          <t>0x04fd78e33c10fb928e409323c26948f49fe4c81fcd47748d9153c9c611b38d0b</t>
         </is>
       </c>
       <c r="M37" t="inlineStr">
@@ -4172,7 +4196,7 @@
       </c>
       <c r="R37" t="inlineStr">
         <is>
-          <t>1784983703</t>
+          <t>1784983849</t>
         </is>
       </c>
       <c r="S37" t="inlineStr">
@@ -4182,7 +4206,7 @@
       </c>
       <c r="T37" t="inlineStr">
         <is>
-          <t>5.770489</t>
+          <t>11.988786</t>
         </is>
       </c>
       <c r="U37" t="inlineStr">
@@ -4195,7 +4219,7 @@
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>0x78c593e23cd10a2517f77039f922e2d360ba0b6d4c89dc91bac22f6854ce01ea</t>
+          <t>0x6e3d6f822ebfe70f563004b4a5a4a6303f1d1cb9677e6e3a56324cda8cc92ba7</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
@@ -4210,7 +4234,7 @@
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>2.0</t>
+          <t>25.0</t>
         </is>
       </c>
       <c r="E38" t="inlineStr">
@@ -4272,7 +4296,7 @@
       </c>
       <c r="R38" t="inlineStr">
         <is>
-          <t>1784983703</t>
+          <t>1784983797</t>
         </is>
       </c>
       <c r="S38" t="inlineStr">
@@ -4282,7 +4306,7 @@
       </c>
       <c r="T38" t="inlineStr">
         <is>
-          <t>4.389968</t>
+          <t>46.150404</t>
         </is>
       </c>
       <c r="U38" t="inlineStr">
@@ -4295,7 +4319,7 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>0x589562dc55239bfc299045a0e5bbfed420cc8f286ee7326d34ed350f83ecdd45</t>
+          <t>0xc913b7104d801ceb0283dc9eefcce577969c93f7b16c1cc5515036561b5b8d8e</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
@@ -4305,17 +4329,17 @@
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>12.0</t>
+          <t>4.0</t>
         </is>
       </c>
       <c r="E39" t="inlineStr">
         <is>
-          <t>1.5513</t>
+          <t>1.7712</t>
         </is>
       </c>
       <c r="F39" t="inlineStr"/>
@@ -4342,7 +4366,7 @@
       </c>
       <c r="L39" t="inlineStr">
         <is>
-          <t>0x04fd78e33c10fb928e409323c26948f49fe4c81fcd47748d9153c9c611b38d0b</t>
+          <t>0x91a9ea8ebfd8b049218a8e072590d2f657e26fdb1f2a49b1016ae42171c68ef2</t>
         </is>
       </c>
       <c r="M39" t="inlineStr">
@@ -4372,7 +4396,7 @@
       </c>
       <c r="R39" t="inlineStr">
         <is>
-          <t>1784983480</t>
+          <t>1784983703</t>
         </is>
       </c>
       <c r="S39" t="inlineStr">
@@ -4382,7 +4406,7 @@
       </c>
       <c r="T39" t="inlineStr">
         <is>
-          <t>22.284118</t>
+          <t>5.770489</t>
         </is>
       </c>
       <c r="U39" t="inlineStr">
@@ -4395,7 +4419,7 @@
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>0x629a7bab69ed2f6eae5804065863061a8e5f95bfbf35104c3a1d130585e021ca</t>
+          <t>0x78c593e23cd10a2517f77039f922e2d360ba0b6d4c89dc91bac22f6854ce01ea</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
@@ -4410,7 +4434,7 @@
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>1.0</t>
+          <t>2.0</t>
         </is>
       </c>
       <c r="E40" t="inlineStr">
@@ -4472,7 +4496,7 @@
       </c>
       <c r="R40" t="inlineStr">
         <is>
-          <t>1784983361</t>
+          <t>1784983703</t>
         </is>
       </c>
       <c r="S40" t="inlineStr">
@@ -4482,7 +4506,7 @@
       </c>
       <c r="T40" t="inlineStr">
         <is>
-          <t>2.228408</t>
+          <t>4.389968</t>
         </is>
       </c>
       <c r="U40" t="inlineStr">
@@ -4495,12 +4519,12 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>0x888b7311174b291a1eeccf40a054d1599070da16bd2f2f7adea95d18002cc686</t>
+          <t>0x589562dc55239bfc299045a0e5bbfed420cc8f286ee7326d34ed350f83ecdd45</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>0xB1854fc8aD8ce649EA80D007Fc67d318a239a5DA</t>
+          <t>0x68E1818FF20BBe84F9be9E0A4A395FB11079Bd35</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
@@ -4510,12 +4534,12 @@
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t>0.0</t>
+          <t>12.0</t>
         </is>
       </c>
       <c r="E41" t="inlineStr">
         <is>
-          <t>1.215</t>
+          <t>1.5513</t>
         </is>
       </c>
       <c r="F41" t="inlineStr"/>
@@ -4542,7 +4566,7 @@
       </c>
       <c r="L41" t="inlineStr">
         <is>
-          <t>0x91a9ea8ebfd8b049218a8e072590d2f657e26fdb1f2a49b1016ae42171c68ef2</t>
+          <t>0x04fd78e33c10fb928e409323c26948f49fe4c81fcd47748d9153c9c611b38d0b</t>
         </is>
       </c>
       <c r="M41" t="inlineStr">
@@ -4572,7 +4596,7 @@
       </c>
       <c r="R41" t="inlineStr">
         <is>
-          <t>1784981088</t>
+          <t>1784983480</t>
         </is>
       </c>
       <c r="S41" t="inlineStr">
@@ -4582,7 +4606,7 @@
       </c>
       <c r="T41" t="inlineStr">
         <is>
-          <t>1.443442</t>
+          <t>22.284118</t>
         </is>
       </c>
       <c r="U41" t="inlineStr">
@@ -4595,7 +4619,7 @@
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>0x5d44678e836886d72dc3bddfca4b44d2be2bfa7f56096dbedd259cac92e30df3</t>
+          <t>0x629a7bab69ed2f6eae5804065863061a8e5f95bfbf35104c3a1d130585e021ca</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
@@ -4605,17 +4629,17 @@
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>1</t>
         </is>
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t>16.0</t>
+          <t>1.0</t>
         </is>
       </c>
       <c r="E42" t="inlineStr">
         <is>
-          <t>1.7712</t>
+          <t>1.5513</t>
         </is>
       </c>
       <c r="F42" t="inlineStr"/>
@@ -4642,7 +4666,7 @@
       </c>
       <c r="L42" t="inlineStr">
         <is>
-          <t>0x91a9ea8ebfd8b049218a8e072590d2f657e26fdb1f2a49b1016ae42171c68ef2</t>
+          <t>0x04fd78e33c10fb928e409323c26948f49fe4c81fcd47748d9153c9c611b38d0b</t>
         </is>
       </c>
       <c r="M42" t="inlineStr">
@@ -4672,7 +4696,7 @@
       </c>
       <c r="R42" t="inlineStr">
         <is>
-          <t>1784981082</t>
+          <t>1784983361</t>
         </is>
       </c>
       <c r="S42" t="inlineStr">
@@ -4682,7 +4706,7 @@
       </c>
       <c r="T42" t="inlineStr">
         <is>
-          <t>21.377037</t>
+          <t>2.228408</t>
         </is>
       </c>
       <c r="U42" t="inlineStr">
@@ -4695,12 +4719,12 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>0x5a96bb0ca1d506186a0e2c1c2e13d657784bbb03ad3f75e66db86da80f485bae</t>
+          <t>0x888b7311174b291a1eeccf40a054d1599070da16bd2f2f7adea95d18002cc686</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>0x68E1818FF20BBe84F9be9E0A4A395FB11079Bd35</t>
+          <t>0xB1854fc8aD8ce649EA80D007Fc67d318a239a5DA</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
@@ -4710,12 +4734,12 @@
       </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t>19.0</t>
+          <t>0.0</t>
         </is>
       </c>
       <c r="E43" t="inlineStr">
         <is>
-          <t>1.5513</t>
+          <t>1.215</t>
         </is>
       </c>
       <c r="F43" t="inlineStr"/>
@@ -4742,7 +4766,7 @@
       </c>
       <c r="L43" t="inlineStr">
         <is>
-          <t>0x04fd78e33c10fb928e409323c26948f49fe4c81fcd47748d9153c9c611b38d0b</t>
+          <t>0x91a9ea8ebfd8b049218a8e072590d2f657e26fdb1f2a49b1016ae42171c68ef2</t>
         </is>
       </c>
       <c r="M43" t="inlineStr">
@@ -4772,7 +4796,7 @@
       </c>
       <c r="R43" t="inlineStr">
         <is>
-          <t>1784980847</t>
+          <t>1784981088</t>
         </is>
       </c>
       <c r="S43" t="inlineStr">
@@ -4782,7 +4806,7 @@
       </c>
       <c r="T43" t="inlineStr">
         <is>
-          <t>35.743728</t>
+          <t>1.443442</t>
         </is>
       </c>
       <c r="U43" t="inlineStr">
@@ -4795,27 +4819,27 @@
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>0xe6e61e0b4573e8e2199880691f7803f1943269d2b2b955ea7282a833c4dbc3c6</t>
+          <t>0x5d44678e836886d72dc3bddfca4b44d2be2bfa7f56096dbedd259cac92e30df3</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>0x47D0CE9b8d653c8884DB7E2a7F88d4849E0CD980</t>
+          <t>0x68E1818FF20BBe84F9be9E0A4A395FB11079Bd35</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
       <c r="D44" t="inlineStr">
         <is>
-          <t>22.0</t>
+          <t>16.0</t>
         </is>
       </c>
       <c r="E44" t="inlineStr">
         <is>
-          <t>1.555</t>
+          <t>1.7712</t>
         </is>
       </c>
       <c r="F44" t="inlineStr"/>
@@ -4842,7 +4866,7 @@
       </c>
       <c r="L44" t="inlineStr">
         <is>
-          <t>0x04fd78e33c10fb928e409323c26948f49fe4c81fcd47748d9153c9c611b38d0b</t>
+          <t>0x91a9ea8ebfd8b049218a8e072590d2f657e26fdb1f2a49b1016ae42171c68ef2</t>
         </is>
       </c>
       <c r="M44" t="inlineStr">
@@ -4872,7 +4896,7 @@
       </c>
       <c r="R44" t="inlineStr">
         <is>
-          <t>1784977858</t>
+          <t>1784981082</t>
         </is>
       </c>
       <c r="S44" t="inlineStr">
@@ -4882,7 +4906,7 @@
       </c>
       <c r="T44" t="inlineStr">
         <is>
-          <t>39.775279</t>
+          <t>21.377037</t>
         </is>
       </c>
       <c r="U44" t="inlineStr">
@@ -4895,12 +4919,12 @@
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>0x668fc309ba15ebe234fe9dd2d2bf696a9f4000c9ac85f8e7d55c998a052968dc</t>
+          <t>0x5a96bb0ca1d506186a0e2c1c2e13d657784bbb03ad3f75e66db86da80f485bae</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>0x47D0CE9b8d653c8884DB7E2a7F88d4849E0CD980</t>
+          <t>0x68E1818FF20BBe84F9be9E0A4A395FB11079Bd35</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
@@ -4910,12 +4934,12 @@
       </c>
       <c r="D45" t="inlineStr">
         <is>
-          <t>27.0</t>
+          <t>19.0</t>
         </is>
       </c>
       <c r="E45" t="inlineStr">
         <is>
-          <t>1.555</t>
+          <t>1.5513</t>
         </is>
       </c>
       <c r="F45" t="inlineStr"/>
@@ -4972,7 +4996,7 @@
       </c>
       <c r="R45" t="inlineStr">
         <is>
-          <t>1784977853</t>
+          <t>1784980847</t>
         </is>
       </c>
       <c r="S45" t="inlineStr">
@@ -4982,7 +5006,7 @@
       </c>
       <c r="T45" t="inlineStr">
         <is>
-          <t>49.797748</t>
+          <t>35.743728</t>
         </is>
       </c>
       <c r="U45" t="inlineStr">
@@ -4995,27 +5019,27 @@
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>0xabcdef492212262464335967adbaa23c5214ede2fab0ea2a12bce6e0027067aa</t>
+          <t>0xe6e61e0b4573e8e2199880691f7803f1943269d2b2b955ea7282a833c4dbc3c6</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>0xC88F614A48f8A705d7465b03aAF62ddaca0c3754</t>
+          <t>0x47D0CE9b8d653c8884DB7E2a7F88d4849E0CD980</t>
         </is>
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>1</t>
         </is>
       </c>
       <c r="D46" t="inlineStr">
         <is>
-          <t>20.0</t>
+          <t>22.0</t>
         </is>
       </c>
       <c r="E46" t="inlineStr">
         <is>
-          <t>1.435</t>
+          <t>1.555</t>
         </is>
       </c>
       <c r="F46" t="inlineStr"/>
@@ -5042,7 +5066,7 @@
       </c>
       <c r="L46" t="inlineStr">
         <is>
-          <t>0xef2cff3047642c7d3f79713526decc2ed1438c01d374590eb62929362f824801</t>
+          <t>0x04fd78e33c10fb928e409323c26948f49fe4c81fcd47748d9153c9c611b38d0b</t>
         </is>
       </c>
       <c r="M46" t="inlineStr">
@@ -5072,7 +5096,7 @@
       </c>
       <c r="R46" t="inlineStr">
         <is>
-          <t>1784968614</t>
+          <t>1784977858</t>
         </is>
       </c>
       <c r="S46" t="inlineStr">
@@ -5082,7 +5106,7 @@
       </c>
       <c r="T46" t="inlineStr">
         <is>
-          <t>47.149425</t>
+          <t>39.775279</t>
         </is>
       </c>
       <c r="U46" t="inlineStr">
@@ -5095,12 +5119,12 @@
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>0xf7e34584abe1fc7da16770ad9dc2fe59e91a45480c1ff509d55070c7d811c7e2</t>
+          <t>0x668fc309ba15ebe234fe9dd2d2bf696a9f4000c9ac85f8e7d55c998a052968dc</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>0x516bfc7CE57c0E1734388ECed5Bb9454aA6aeFae</t>
+          <t>0x47D0CE9b8d653c8884DB7E2a7F88d4849E0CD980</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
@@ -5110,12 +5134,12 @@
       </c>
       <c r="D47" t="inlineStr">
         <is>
-          <t>10.0</t>
+          <t>27.0</t>
         </is>
       </c>
       <c r="E47" t="inlineStr">
         <is>
-          <t>1.56</t>
+          <t>1.555</t>
         </is>
       </c>
       <c r="F47" t="inlineStr"/>
@@ -5142,7 +5166,7 @@
       </c>
       <c r="L47" t="inlineStr">
         <is>
-          <t>0xe1204c11efd43d8d3a0377591c468bba3ac169f58ab541c6d60665f2e0bbb051</t>
+          <t>0x04fd78e33c10fb928e409323c26948f49fe4c81fcd47748d9153c9c611b38d0b</t>
         </is>
       </c>
       <c r="M47" t="inlineStr">
@@ -5172,7 +5196,7 @@
       </c>
       <c r="R47" t="inlineStr">
         <is>
-          <t>1784907257</t>
+          <t>1784977853</t>
         </is>
       </c>
       <c r="S47" t="inlineStr">
@@ -5182,7 +5206,7 @@
       </c>
       <c r="T47" t="inlineStr">
         <is>
-          <t>17.857143</t>
+          <t>49.797748</t>
         </is>
       </c>
       <c r="U47" t="inlineStr">
@@ -5195,7 +5219,7 @@
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>0x030841d8eff7e23d98d8319e71f99f9eb17cb2a743343cfac134410b86f1178e</t>
+          <t>0xabcdef492212262464335967adbaa23c5214ede2fab0ea2a12bce6e0027067aa</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
@@ -5205,17 +5229,17 @@
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
       <c r="D48" t="inlineStr">
         <is>
-          <t>26.0</t>
+          <t>20.0</t>
         </is>
       </c>
       <c r="E48" t="inlineStr">
         <is>
-          <t>1.5737</t>
+          <t>1.435</t>
         </is>
       </c>
       <c r="F48" t="inlineStr"/>
@@ -5242,7 +5266,7 @@
       </c>
       <c r="L48" t="inlineStr">
         <is>
-          <t>0xe1204c11efd43d8d3a0377591c468bba3ac169f58ab541c6d60665f2e0bbb051</t>
+          <t>0xef2cff3047642c7d3f79713526decc2ed1438c01d374590eb62929362f824801</t>
         </is>
       </c>
       <c r="M48" t="inlineStr">
@@ -5272,7 +5296,7 @@
       </c>
       <c r="R48" t="inlineStr">
         <is>
-          <t>1784907053</t>
+          <t>1784968614</t>
         </is>
       </c>
       <c r="S48" t="inlineStr">
@@ -5282,7 +5306,7 @@
       </c>
       <c r="T48" t="inlineStr">
         <is>
-          <t>46.28739</t>
+          <t>47.149425</t>
         </is>
       </c>
       <c r="U48" t="inlineStr">
@@ -5295,12 +5319,12 @@
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>0xd486facb98ea7c7e7b67efb74b5231332788279dbd71dce40eea54aecf5d870e</t>
+          <t>0xf7e34584abe1fc7da16770ad9dc2fe59e91a45480c1ff509d55070c7d811c7e2</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>0xC88F614A48f8A705d7465b03aAF62ddaca0c3754</t>
+          <t>0x516bfc7CE57c0E1734388ECed5Bb9454aA6aeFae</t>
         </is>
       </c>
       <c r="C49" t="inlineStr">
@@ -5310,12 +5334,12 @@
       </c>
       <c r="D49" t="inlineStr">
         <is>
-          <t>14.0</t>
+          <t>10.0</t>
         </is>
       </c>
       <c r="E49" t="inlineStr">
         <is>
-          <t>1.315</t>
+          <t>1.56</t>
         </is>
       </c>
       <c r="F49" t="inlineStr"/>
@@ -5342,7 +5366,7 @@
       </c>
       <c r="L49" t="inlineStr">
         <is>
-          <t>0x588a71865f90131e16b5b72dfef6ddb7cec8deb7df1f8102477a62eaa807cc71</t>
+          <t>0xe1204c11efd43d8d3a0377591c468bba3ac169f58ab541c6d60665f2e0bbb051</t>
         </is>
       </c>
       <c r="M49" t="inlineStr">
@@ -5372,7 +5396,7 @@
       </c>
       <c r="R49" t="inlineStr">
         <is>
-          <t>1784907041</t>
+          <t>1784907257</t>
         </is>
       </c>
       <c r="S49" t="inlineStr">
@@ -5382,7 +5406,7 @@
       </c>
       <c r="T49" t="inlineStr">
         <is>
-          <t>47.587302</t>
+          <t>17.857143</t>
         </is>
       </c>
       <c r="U49" t="inlineStr">
@@ -5395,7 +5419,7 @@
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>0x8a9596cb004924470885fe466db8f8d059fcb9d1b24e71490dd35bfeba65a98d</t>
+          <t>0x030841d8eff7e23d98d8319e71f99f9eb17cb2a743343cfac134410b86f1178e</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
@@ -5410,12 +5434,12 @@
       </c>
       <c r="D50" t="inlineStr">
         <is>
-          <t>14.0</t>
+          <t>26.0</t>
         </is>
       </c>
       <c r="E50" t="inlineStr">
         <is>
-          <t>1.315</t>
+          <t>1.5737</t>
         </is>
       </c>
       <c r="F50" t="inlineStr"/>
@@ -5442,7 +5466,7 @@
       </c>
       <c r="L50" t="inlineStr">
         <is>
-          <t>0x06a233f1b733d63cee459a37ac1beffad92b8f9ec21c414e0c26e2876b05eebd</t>
+          <t>0xe1204c11efd43d8d3a0377591c468bba3ac169f58ab541c6d60665f2e0bbb051</t>
         </is>
       </c>
       <c r="M50" t="inlineStr">
@@ -5472,7 +5496,7 @@
       </c>
       <c r="R50" t="inlineStr">
         <is>
-          <t>1784907041</t>
+          <t>1784907053</t>
         </is>
       </c>
       <c r="S50" t="inlineStr">
@@ -5482,7 +5506,7 @@
       </c>
       <c r="T50" t="inlineStr">
         <is>
-          <t>47.555556</t>
+          <t>46.28739</t>
         </is>
       </c>
       <c r="U50" t="inlineStr">
@@ -5495,7 +5519,7 @@
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>0xdaf8fe8a287cecb340987a0eebd287e9d8e007af24d015fcadd720fceba485cd</t>
+          <t>0xd486facb98ea7c7e7b67efb74b5231332788279dbd71dce40eea54aecf5d870e</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
@@ -5510,12 +5534,12 @@
       </c>
       <c r="D51" t="inlineStr">
         <is>
-          <t>26.0</t>
+          <t>14.0</t>
         </is>
       </c>
       <c r="E51" t="inlineStr">
         <is>
-          <t>1.57</t>
+          <t>1.315</t>
         </is>
       </c>
       <c r="F51" t="inlineStr"/>
@@ -5542,7 +5566,7 @@
       </c>
       <c r="L51" t="inlineStr">
         <is>
-          <t>0xe1204c11efd43d8d3a0377591c468bba3ac169f58ab541c6d60665f2e0bbb051</t>
+          <t>0x588a71865f90131e16b5b72dfef6ddb7cec8deb7df1f8102477a62eaa807cc71</t>
         </is>
       </c>
       <c r="M51" t="inlineStr">
@@ -5572,7 +5596,7 @@
       </c>
       <c r="R51" t="inlineStr">
         <is>
-          <t>1784907040</t>
+          <t>1784907041</t>
         </is>
       </c>
       <c r="S51" t="inlineStr">
@@ -5582,7 +5606,7 @@
       </c>
       <c r="T51" t="inlineStr">
         <is>
-          <t>47.046509</t>
+          <t>47.587302</t>
         </is>
       </c>
       <c r="U51" t="inlineStr">
@@ -5595,7 +5619,7 @@
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>0x3f981c0415a637d3cb9137ae5b4b0b4b0c50f1a3af5d4e42f65e682f80daadba</t>
+          <t>0x8a9596cb004924470885fe466db8f8d059fcb9d1b24e71490dd35bfeba65a98d</t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
@@ -5610,12 +5634,12 @@
       </c>
       <c r="D52" t="inlineStr">
         <is>
-          <t>22.0</t>
+          <t>14.0</t>
         </is>
       </c>
       <c r="E52" t="inlineStr">
         <is>
-          <t>1.4625</t>
+          <t>1.315</t>
         </is>
       </c>
       <c r="F52" t="inlineStr"/>
@@ -5642,55 +5666,255 @@
       </c>
       <c r="L52" t="inlineStr">
         <is>
+          <t>0x06a233f1b733d63cee459a37ac1beffad92b8f9ec21c414e0c26e2876b05eebd</t>
+        </is>
+      </c>
+      <c r="M52" t="inlineStr">
+        <is>
+          <t>L19520873</t>
+        </is>
+      </c>
+      <c r="N52" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="O52" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="P52" t="inlineStr">
+        <is>
+          <t>SUCCESS</t>
+        </is>
+      </c>
+      <c r="Q52" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="R52" t="inlineStr">
+        <is>
+          <t>1784907041</t>
+        </is>
+      </c>
+      <c r="S52" t="inlineStr">
+        <is>
+          <t>1784988000</t>
+        </is>
+      </c>
+      <c r="T52" t="inlineStr">
+        <is>
+          <t>47.555556</t>
+        </is>
+      </c>
+      <c r="U52" t="inlineStr">
+        <is>
+          <t>SXR</t>
+        </is>
+      </c>
+      <c r="V52" t="inlineStr"/>
+    </row>
+    <row r="53">
+      <c r="A53" t="inlineStr">
+        <is>
+          <t>0xdaf8fe8a287cecb340987a0eebd287e9d8e007af24d015fcadd720fceba485cd</t>
+        </is>
+      </c>
+      <c r="B53" t="inlineStr">
+        <is>
+          <t>0xC88F614A48f8A705d7465b03aAF62ddaca0c3754</t>
+        </is>
+      </c>
+      <c r="C53" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="D53" t="inlineStr">
+        <is>
+          <t>26.0</t>
+        </is>
+      </c>
+      <c r="E53" t="inlineStr">
+        <is>
+          <t>1.57</t>
+        </is>
+      </c>
+      <c r="F53" t="inlineStr"/>
+      <c r="G53" t="inlineStr"/>
+      <c r="H53" t="inlineStr">
+        <is>
+          <t>Besta Deild Karla</t>
+        </is>
+      </c>
+      <c r="I53" t="inlineStr">
+        <is>
+          <t>IR Reykjavik vs Fylkir</t>
+        </is>
+      </c>
+      <c r="J53" t="inlineStr">
+        <is>
+          <t>IR Reykjavik</t>
+        </is>
+      </c>
+      <c r="K53" t="inlineStr">
+        <is>
+          <t>Fylkir</t>
+        </is>
+      </c>
+      <c r="L53" t="inlineStr">
+        <is>
+          <t>0xe1204c11efd43d8d3a0377591c468bba3ac169f58ab541c6d60665f2e0bbb051</t>
+        </is>
+      </c>
+      <c r="M53" t="inlineStr">
+        <is>
+          <t>L19520873</t>
+        </is>
+      </c>
+      <c r="N53" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="O53" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="P53" t="inlineStr">
+        <is>
+          <t>SUCCESS</t>
+        </is>
+      </c>
+      <c r="Q53" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="R53" t="inlineStr">
+        <is>
+          <t>1784907040</t>
+        </is>
+      </c>
+      <c r="S53" t="inlineStr">
+        <is>
+          <t>1784988000</t>
+        </is>
+      </c>
+      <c r="T53" t="inlineStr">
+        <is>
+          <t>47.046509</t>
+        </is>
+      </c>
+      <c r="U53" t="inlineStr">
+        <is>
+          <t>SXR</t>
+        </is>
+      </c>
+      <c r="V53" t="inlineStr"/>
+    </row>
+    <row r="54">
+      <c r="A54" t="inlineStr">
+        <is>
+          <t>0x3f981c0415a637d3cb9137ae5b4b0b4b0c50f1a3af5d4e42f65e682f80daadba</t>
+        </is>
+      </c>
+      <c r="B54" t="inlineStr">
+        <is>
+          <t>0xC88F614A48f8A705d7465b03aAF62ddaca0c3754</t>
+        </is>
+      </c>
+      <c r="C54" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="D54" t="inlineStr">
+        <is>
+          <t>22.0</t>
+        </is>
+      </c>
+      <c r="E54" t="inlineStr">
+        <is>
+          <t>1.4625</t>
+        </is>
+      </c>
+      <c r="F54" t="inlineStr"/>
+      <c r="G54" t="inlineStr"/>
+      <c r="H54" t="inlineStr">
+        <is>
+          <t>Besta Deild Karla</t>
+        </is>
+      </c>
+      <c r="I54" t="inlineStr">
+        <is>
+          <t>IR Reykjavik vs Fylkir</t>
+        </is>
+      </c>
+      <c r="J54" t="inlineStr">
+        <is>
+          <t>IR Reykjavik</t>
+        </is>
+      </c>
+      <c r="K54" t="inlineStr">
+        <is>
+          <t>Fylkir</t>
+        </is>
+      </c>
+      <c r="L54" t="inlineStr">
+        <is>
           <t>0xd5ae8f2322bcc6adaca1c1bb1baf6a74afa50cc30131840c87632f67865c23d0</t>
         </is>
       </c>
-      <c r="M52" t="inlineStr">
+      <c r="M54" t="inlineStr">
         <is>
           <t>L19520873</t>
         </is>
       </c>
-      <c r="N52" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="O52" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="P52" t="inlineStr">
+      <c r="N54" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="O54" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="P54" t="inlineStr">
         <is>
           <t>SUCCESS</t>
         </is>
       </c>
-      <c r="Q52" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="R52" t="inlineStr">
+      <c r="Q54" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="R54" t="inlineStr">
         <is>
           <t>1784907040</t>
         </is>
       </c>
-      <c r="S52" t="inlineStr">
+      <c r="S54" t="inlineStr">
         <is>
           <t>1784988000</t>
         </is>
       </c>
-      <c r="T52" t="inlineStr">
+      <c r="T54" t="inlineStr">
         <is>
           <t>47.589189</t>
         </is>
       </c>
-      <c r="U52" t="inlineStr">
+      <c r="U54" t="inlineStr">
         <is>
           <t>SXR</t>
         </is>
       </c>
-      <c r="V52" t="inlineStr"/>
+      <c r="V54" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>